<commit_message>
feat: add Standardized ASM tab with IS, BS, CF reformulation
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/ASM_Valuation_Model.xlsx
+++ b/output/ASM_Valuation_Model.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input AIXTRON" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input AMAT" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input LRCX" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Std ASM" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,10 +22,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00;(#,##0.00);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,16 +83,46 @@
     <font>
       <color rgb="000000FF"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
+    </font>
+    <font>
+      <color rgb="00008000"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B4C6E7"/>
+        <bgColor rgb="00B4C6E7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -99,11 +133,24 @@
     <border>
       <bottom style="medium"/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <bottom style="double"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -122,6 +169,26 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="13" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -25449,4 +25516,2353 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G99"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Standardized Financial Statements - ASM International NV</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>(EUR 000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="16" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C3" s="16" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D3" s="16" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E3" s="16" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F3" s="16" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G3" s="16" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Operating cash %</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G5" s="17" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Tax rate (effective)</t>
+        </is>
+      </c>
+      <c r="B6" s="18">
+        <f>IF(ISNUMBER('Input ASM'!B68),'Input ASM'!B68,0)</f>
+        <v/>
+      </c>
+      <c r="C6" s="18">
+        <f>IF(ISNUMBER('Input ASM'!C68),'Input ASM'!C68,0)</f>
+        <v/>
+      </c>
+      <c r="D6" s="18">
+        <f>IF(ISNUMBER('Input ASM'!D68),'Input ASM'!D68,0)</f>
+        <v/>
+      </c>
+      <c r="E6" s="18">
+        <f>IF(ISNUMBER('Input ASM'!E68),'Input ASM'!E68,0)</f>
+        <v/>
+      </c>
+      <c r="F6" s="18">
+        <f>IF(ISNUMBER('Input ASM'!F68),'Input ASM'!F68,0)</f>
+        <v/>
+      </c>
+      <c r="G6" s="18">
+        <f>IF(ISNUMBER('Input ASM'!G68),'Input ASM'!G68,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>INCOME STATEMENT</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="n"/>
+      <c r="C8" s="20" t="n"/>
+      <c r="D8" s="20" t="n"/>
+      <c r="E8" s="20" t="n"/>
+      <c r="F8" s="20" t="n"/>
+      <c r="G8" s="20" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B9" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B21),'Input ASM'!B21,0)</f>
+        <v/>
+      </c>
+      <c r="C9" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C21),'Input ASM'!C21,0)</f>
+        <v/>
+      </c>
+      <c r="D9" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D21),'Input ASM'!D21,0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E21),'Input ASM'!E21,0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F21),'Input ASM'!F21,0)</f>
+        <v/>
+      </c>
+      <c r="G9" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G21),'Input ASM'!G21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Cost of Sales</t>
+        </is>
+      </c>
+      <c r="B10" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B23),'Input ASM'!B23,0)</f>
+        <v/>
+      </c>
+      <c r="C10" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C23),'Input ASM'!C23,0)</f>
+        <v/>
+      </c>
+      <c r="D10" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D23),'Input ASM'!D23,0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E23),'Input ASM'!E23,0)</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F23),'Input ASM'!F23,0)</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G23),'Input ASM'!G23,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>Gross Profit</t>
+        </is>
+      </c>
+      <c r="B11" s="23">
+        <f>B9-B10</f>
+        <v/>
+      </c>
+      <c r="C11" s="23">
+        <f>C9-C10</f>
+        <v/>
+      </c>
+      <c r="D11" s="23">
+        <f>D9-D10</f>
+        <v/>
+      </c>
+      <c r="E11" s="23">
+        <f>E9-E10</f>
+        <v/>
+      </c>
+      <c r="F11" s="23">
+        <f>F9-F10</f>
+        <v/>
+      </c>
+      <c r="G11" s="23">
+        <f>G9-G10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SG&amp;A</t>
+        </is>
+      </c>
+      <c r="B12" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B26),'Input ASM'!B26,0)</f>
+        <v/>
+      </c>
+      <c r="C12" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C26),'Input ASM'!C26,0)</f>
+        <v/>
+      </c>
+      <c r="D12" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D26),'Input ASM'!D26,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E26),'Input ASM'!E26,0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F26),'Input ASM'!F26,0)</f>
+        <v/>
+      </c>
+      <c r="G12" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G26),'Input ASM'!G26,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  R&amp;D</t>
+        </is>
+      </c>
+      <c r="B13" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B27),'Input ASM'!B27,0)</f>
+        <v/>
+      </c>
+      <c r="C13" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C27),'Input ASM'!C27,0)</f>
+        <v/>
+      </c>
+      <c r="D13" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D27),'Input ASM'!D27,0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E27),'Input ASM'!E27,0)</f>
+        <v/>
+      </c>
+      <c r="F13" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F27),'Input ASM'!F27,0)</f>
+        <v/>
+      </c>
+      <c r="G13" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G27),'Input ASM'!G27,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Depreciation &amp; Amortization</t>
+        </is>
+      </c>
+      <c r="B14" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B113),'Input ASM'!B113,0)</f>
+        <v/>
+      </c>
+      <c r="C14" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C113),'Input ASM'!C113,0)</f>
+        <v/>
+      </c>
+      <c r="D14" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D113),'Input ASM'!D113,0)</f>
+        <v/>
+      </c>
+      <c r="E14" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E113),'Input ASM'!E113,0)</f>
+        <v/>
+      </c>
+      <c r="F14" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F113),'Input ASM'!F113,0)</f>
+        <v/>
+      </c>
+      <c r="G14" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G113),'Input ASM'!G113,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Other Operating Expense</t>
+        </is>
+      </c>
+      <c r="B15" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B29),'Input ASM'!B29,0)</f>
+        <v/>
+      </c>
+      <c r="C15" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C29),'Input ASM'!C29,0)</f>
+        <v/>
+      </c>
+      <c r="D15" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D29),'Input ASM'!D29,0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E29),'Input ASM'!E29,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F29),'Input ASM'!F29,0)</f>
+        <v/>
+      </c>
+      <c r="G15" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G29),'Input ASM'!G29,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>Total Operating Expense</t>
+        </is>
+      </c>
+      <c r="B16" s="25">
+        <f>B10+B12+B13+B14+B15</f>
+        <v/>
+      </c>
+      <c r="C16" s="25">
+        <f>C10+C12+C13+C14+C15</f>
+        <v/>
+      </c>
+      <c r="D16" s="25">
+        <f>D10+D12+D13+D14+D15</f>
+        <v/>
+      </c>
+      <c r="E16" s="25">
+        <f>E10+E12+E13+E14+E15</f>
+        <v/>
+      </c>
+      <c r="F16" s="25">
+        <f>F10+F12+F13+F14+F15</f>
+        <v/>
+      </c>
+      <c r="G16" s="25">
+        <f>G10+G12+G13+G14+G15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>Recurring Operating Profit</t>
+        </is>
+      </c>
+      <c r="B17" s="25">
+        <f>B9-B16</f>
+        <v/>
+      </c>
+      <c r="C17" s="25">
+        <f>C9-C16</f>
+        <v/>
+      </c>
+      <c r="D17" s="25">
+        <f>D9-D16</f>
+        <v/>
+      </c>
+      <c r="E17" s="25">
+        <f>E9-E16</f>
+        <v/>
+      </c>
+      <c r="F17" s="25">
+        <f>F9-F16</f>
+        <v/>
+      </c>
+      <c r="G17" s="25">
+        <f>G9-G16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>Non-recurring items:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Gain/Loss on Sale of Investments</t>
+        </is>
+      </c>
+      <c r="B20" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B39),'Input ASM'!B39,0)</f>
+        <v/>
+      </c>
+      <c r="C20" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C39),'Input ASM'!C39,0)</f>
+        <v/>
+      </c>
+      <c r="D20" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D39),'Input ASM'!D39,0)</f>
+        <v/>
+      </c>
+      <c r="E20" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E39),'Input ASM'!E39,0)</f>
+        <v/>
+      </c>
+      <c r="F20" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F39),'Input ASM'!F39,0)</f>
+        <v/>
+      </c>
+      <c r="G20" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G39),'Input ASM'!G39,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Gain/Loss on Sale of Assets</t>
+        </is>
+      </c>
+      <c r="B21" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B40),'Input ASM'!B40,0)</f>
+        <v/>
+      </c>
+      <c r="C21" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C40),'Input ASM'!C40,0)</f>
+        <v/>
+      </c>
+      <c r="D21" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D40),'Input ASM'!D40,0)</f>
+        <v/>
+      </c>
+      <c r="E21" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E40),'Input ASM'!E40,0)</f>
+        <v/>
+      </c>
+      <c r="F21" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F40),'Input ASM'!F40,0)</f>
+        <v/>
+      </c>
+      <c r="G21" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G40),'Input ASM'!G40,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Asset Writedown</t>
+        </is>
+      </c>
+      <c r="B22" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B41),'Input ASM'!B41,0)</f>
+        <v/>
+      </c>
+      <c r="C22" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C41),'Input ASM'!C41,0)</f>
+        <v/>
+      </c>
+      <c r="D22" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D41),'Input ASM'!D41,0)</f>
+        <v/>
+      </c>
+      <c r="E22" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E41),'Input ASM'!E41,0)</f>
+        <v/>
+      </c>
+      <c r="F22" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F41),'Input ASM'!F41,0)</f>
+        <v/>
+      </c>
+      <c r="G22" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G41),'Input ASM'!G41,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Other Unusual Items</t>
+        </is>
+      </c>
+      <c r="B23" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B42),'Input ASM'!B42,0)</f>
+        <v/>
+      </c>
+      <c r="C23" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C42),'Input ASM'!C42,0)</f>
+        <v/>
+      </c>
+      <c r="D23" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D42),'Input ASM'!D42,0)</f>
+        <v/>
+      </c>
+      <c r="E23" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E42),'Input ASM'!E42,0)</f>
+        <v/>
+      </c>
+      <c r="F23" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F42),'Input ASM'!F42,0)</f>
+        <v/>
+      </c>
+      <c r="G23" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G42),'Input ASM'!G42,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>Total Non-recurring</t>
+        </is>
+      </c>
+      <c r="B24" s="23">
+        <f>SUM(B20:B23)</f>
+        <v/>
+      </c>
+      <c r="C24" s="23">
+        <f>SUM(C20:C23)</f>
+        <v/>
+      </c>
+      <c r="D24" s="23">
+        <f>SUM(D20:D23)</f>
+        <v/>
+      </c>
+      <c r="E24" s="23">
+        <f>SUM(E20:E23)</f>
+        <v/>
+      </c>
+      <c r="F24" s="23">
+        <f>SUM(F20:F23)</f>
+        <v/>
+      </c>
+      <c r="G24" s="23">
+        <f>SUM(G20:G23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>EBIT</t>
+        </is>
+      </c>
+      <c r="B25" s="25">
+        <f>B17+B24</f>
+        <v/>
+      </c>
+      <c r="C25" s="25">
+        <f>C17+C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="25">
+        <f>D17+D24</f>
+        <v/>
+      </c>
+      <c r="E25" s="25">
+        <f>E17+E24</f>
+        <v/>
+      </c>
+      <c r="F25" s="25">
+        <f>F17+F24</f>
+        <v/>
+      </c>
+      <c r="G25" s="25">
+        <f>G17+G24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Investment Income (Equity Method)</t>
+        </is>
+      </c>
+      <c r="B27" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B36),'Input ASM'!B36,0)</f>
+        <v/>
+      </c>
+      <c r="C27" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C36),'Input ASM'!C36,0)</f>
+        <v/>
+      </c>
+      <c r="D27" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D36),'Input ASM'!D36,0)</f>
+        <v/>
+      </c>
+      <c r="E27" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E36),'Input ASM'!E36,0)</f>
+        <v/>
+      </c>
+      <c r="F27" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F36),'Input ASM'!F36,0)</f>
+        <v/>
+      </c>
+      <c r="G27" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G36),'Input ASM'!G36,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Interest Income</t>
+        </is>
+      </c>
+      <c r="B28" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B34),'Input ASM'!B34,0)</f>
+        <v/>
+      </c>
+      <c r="C28" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C34),'Input ASM'!C34,0)</f>
+        <v/>
+      </c>
+      <c r="D28" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D34),'Input ASM'!D34,0)</f>
+        <v/>
+      </c>
+      <c r="E28" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E34),'Input ASM'!E34,0)</f>
+        <v/>
+      </c>
+      <c r="F28" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F34),'Input ASM'!F34,0)</f>
+        <v/>
+      </c>
+      <c r="G28" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G34),'Input ASM'!G34,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Interest Expense</t>
+        </is>
+      </c>
+      <c r="B29" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B33),'Input ASM'!B33,0)</f>
+        <v/>
+      </c>
+      <c r="C29" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C33),'Input ASM'!C33,0)</f>
+        <v/>
+      </c>
+      <c r="D29" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D33),'Input ASM'!D33,0)</f>
+        <v/>
+      </c>
+      <c r="E29" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E33),'Input ASM'!E33,0)</f>
+        <v/>
+      </c>
+      <c r="F29" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F33),'Input ASM'!F33,0)</f>
+        <v/>
+      </c>
+      <c r="G29" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G33),'Input ASM'!G33,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FX Gains/(Losses)</t>
+        </is>
+      </c>
+      <c r="B30" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B37),'Input ASM'!B37,0)</f>
+        <v/>
+      </c>
+      <c r="C30" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C37),'Input ASM'!C37,0)</f>
+        <v/>
+      </c>
+      <c r="D30" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D37),'Input ASM'!D37,0)</f>
+        <v/>
+      </c>
+      <c r="E30" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E37),'Input ASM'!E37,0)</f>
+        <v/>
+      </c>
+      <c r="F30" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F37),'Input ASM'!F37,0)</f>
+        <v/>
+      </c>
+      <c r="G30" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G37),'Input ASM'!G37,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>Profit Before Tax</t>
+        </is>
+      </c>
+      <c r="B31" s="23">
+        <f>B25+B27+B28+B29+B30</f>
+        <v/>
+      </c>
+      <c r="C31" s="23">
+        <f>C25+C27+C28+C29+C30</f>
+        <v/>
+      </c>
+      <c r="D31" s="23">
+        <f>D25+D27+D28+D29+D30</f>
+        <v/>
+      </c>
+      <c r="E31" s="23">
+        <f>E25+E27+E28+E29+E30</f>
+        <v/>
+      </c>
+      <c r="F31" s="23">
+        <f>F25+F27+F28+F29+F30</f>
+        <v/>
+      </c>
+      <c r="G31" s="23">
+        <f>G25+G27+G28+G29+G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tax Expense</t>
+        </is>
+      </c>
+      <c r="B32" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B45),'Input ASM'!B45,0)</f>
+        <v/>
+      </c>
+      <c r="C32" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C45),'Input ASM'!C45,0)</f>
+        <v/>
+      </c>
+      <c r="D32" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D45),'Input ASM'!D45,0)</f>
+        <v/>
+      </c>
+      <c r="E32" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E45),'Input ASM'!E45,0)</f>
+        <v/>
+      </c>
+      <c r="F32" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F45),'Input ASM'!F45,0)</f>
+        <v/>
+      </c>
+      <c r="G32" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G45),'Input ASM'!G45,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="B33" s="27">
+        <f>B31-B32</f>
+        <v/>
+      </c>
+      <c r="C33" s="27">
+        <f>C31-C32</f>
+        <v/>
+      </c>
+      <c r="D33" s="27">
+        <f>D31-D32</f>
+        <v/>
+      </c>
+      <c r="E33" s="27">
+        <f>E31-E32</f>
+        <v/>
+      </c>
+      <c r="F33" s="27">
+        <f>F31-F32</f>
+        <v/>
+      </c>
+      <c r="G33" s="27">
+        <f>G31-G32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>Effective Tax Rate</t>
+        </is>
+      </c>
+      <c r="B35" s="28">
+        <f>IF(B31&lt;&gt;0,B32/B31,0)</f>
+        <v/>
+      </c>
+      <c r="C35" s="28">
+        <f>IF(C31&lt;&gt;0,C32/C31,0)</f>
+        <v/>
+      </c>
+      <c r="D35" s="28">
+        <f>IF(D31&lt;&gt;0,D32/D31,0)</f>
+        <v/>
+      </c>
+      <c r="E35" s="28">
+        <f>IF(E31&lt;&gt;0,E32/E31,0)</f>
+        <v/>
+      </c>
+      <c r="F35" s="28">
+        <f>IF(F31&lt;&gt;0,F32/F31,0)</f>
+        <v/>
+      </c>
+      <c r="G35" s="28">
+        <f>IF(G31&lt;&gt;0,G32/G31,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="22" t="inlineStr">
+        <is>
+          <t>NOPAT</t>
+        </is>
+      </c>
+      <c r="B36" s="23">
+        <f>B17*(1-B35)</f>
+        <v/>
+      </c>
+      <c r="C36" s="23">
+        <f>C17*(1-C35)</f>
+        <v/>
+      </c>
+      <c r="D36" s="23">
+        <f>D17*(1-D35)</f>
+        <v/>
+      </c>
+      <c r="E36" s="23">
+        <f>E17*(1-E35)</f>
+        <v/>
+      </c>
+      <c r="F36" s="23">
+        <f>F17*(1-F35)</f>
+        <v/>
+      </c>
+      <c r="G36" s="23">
+        <f>G17*(1-G35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Shares Outstanding (diluted)</t>
+        </is>
+      </c>
+      <c r="B38" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B57),'Input ASM'!B57,0)</f>
+        <v/>
+      </c>
+      <c r="C38" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C57),'Input ASM'!C57,0)</f>
+        <v/>
+      </c>
+      <c r="D38" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D57),'Input ASM'!D57,0)</f>
+        <v/>
+      </c>
+      <c r="E38" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E57),'Input ASM'!E57,0)</f>
+        <v/>
+      </c>
+      <c r="F38" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F57),'Input ASM'!F57,0)</f>
+        <v/>
+      </c>
+      <c r="G38" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G57),'Input ASM'!G57,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>EPS (diluted)</t>
+        </is>
+      </c>
+      <c r="B39" s="29">
+        <f>IF(B38&lt;&gt;0,B33/B38*1000,0)</f>
+        <v/>
+      </c>
+      <c r="C39" s="29">
+        <f>IF(C38&lt;&gt;0,C33/C38*1000,0)</f>
+        <v/>
+      </c>
+      <c r="D39" s="29">
+        <f>IF(D38&lt;&gt;0,D33/D38*1000,0)</f>
+        <v/>
+      </c>
+      <c r="E39" s="29">
+        <f>IF(E38&lt;&gt;0,E33/E38*1000,0)</f>
+        <v/>
+      </c>
+      <c r="F39" s="29">
+        <f>IF(F38&lt;&gt;0,F33/F38*1000,0)</f>
+        <v/>
+      </c>
+      <c r="G39" s="29">
+        <f>IF(G38&lt;&gt;0,G33/G38*1000,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>Dividends per Share</t>
+        </is>
+      </c>
+      <c r="B40" s="30">
+        <f>IF(ISNUMBER('Input ASM'!B60),'Input ASM'!B60,0)</f>
+        <v/>
+      </c>
+      <c r="C40" s="30">
+        <f>IF(ISNUMBER('Input ASM'!C60),'Input ASM'!C60,0)</f>
+        <v/>
+      </c>
+      <c r="D40" s="30">
+        <f>IF(ISNUMBER('Input ASM'!D60),'Input ASM'!D60,0)</f>
+        <v/>
+      </c>
+      <c r="E40" s="30">
+        <f>IF(ISNUMBER('Input ASM'!E60),'Input ASM'!E60,0)</f>
+        <v/>
+      </c>
+      <c r="F40" s="30">
+        <f>IF(ISNUMBER('Input ASM'!F60),'Input ASM'!F60,0)</f>
+        <v/>
+      </c>
+      <c r="G40" s="30">
+        <f>IF(ISNUMBER('Input ASM'!G60),'Input ASM'!G60,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>BALANCE SHEET (Reformulated)</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="n"/>
+      <c r="C43" s="20" t="n"/>
+      <c r="D43" s="20" t="n"/>
+      <c r="E43" s="20" t="n"/>
+      <c r="F43" s="20" t="n"/>
+      <c r="G43" s="20" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>Operating Working Capital:</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Trade Receivables</t>
+        </is>
+      </c>
+      <c r="B45" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B167),'Input ASM'!B167,0)</f>
+        <v/>
+      </c>
+      <c r="C45" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C167),'Input ASM'!C167,0)</f>
+        <v/>
+      </c>
+      <c r="D45" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D167),'Input ASM'!D167,0)</f>
+        <v/>
+      </c>
+      <c r="E45" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E167),'Input ASM'!E167,0)</f>
+        <v/>
+      </c>
+      <c r="F45" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F167),'Input ASM'!F167,0)</f>
+        <v/>
+      </c>
+      <c r="G45" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G167),'Input ASM'!G167,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + Other Receivables</t>
+        </is>
+      </c>
+      <c r="B46" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B168),'Input ASM'!B168,0)</f>
+        <v/>
+      </c>
+      <c r="C46" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C168),'Input ASM'!C168,0)</f>
+        <v/>
+      </c>
+      <c r="D46" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D168),'Input ASM'!D168,0)</f>
+        <v/>
+      </c>
+      <c r="E46" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E168),'Input ASM'!E168,0)</f>
+        <v/>
+      </c>
+      <c r="F46" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F168),'Input ASM'!F168,0)</f>
+        <v/>
+      </c>
+      <c r="G46" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G168),'Input ASM'!G168,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + Inventories</t>
+        </is>
+      </c>
+      <c r="B47" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B170),'Input ASM'!B170,0)</f>
+        <v/>
+      </c>
+      <c r="C47" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C170),'Input ASM'!C170,0)</f>
+        <v/>
+      </c>
+      <c r="D47" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D170),'Input ASM'!D170,0)</f>
+        <v/>
+      </c>
+      <c r="E47" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E170),'Input ASM'!E170,0)</f>
+        <v/>
+      </c>
+      <c r="F47" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F170),'Input ASM'!F170,0)</f>
+        <v/>
+      </c>
+      <c r="G47" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G170),'Input ASM'!G170,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + Prepaid &amp; Other CA</t>
+        </is>
+      </c>
+      <c r="B48" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B171),'Input ASM'!B171,0)+IF(ISNUMBER('Input ASM'!B172),'Input ASM'!B172,0)</f>
+        <v/>
+      </c>
+      <c r="C48" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C171),'Input ASM'!C171,0)+IF(ISNUMBER('Input ASM'!C172),'Input ASM'!C172,0)</f>
+        <v/>
+      </c>
+      <c r="D48" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D171),'Input ASM'!D171,0)+IF(ISNUMBER('Input ASM'!D172),'Input ASM'!D172,0)</f>
+        <v/>
+      </c>
+      <c r="E48" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E171),'Input ASM'!E171,0)+IF(ISNUMBER('Input ASM'!E172),'Input ASM'!E172,0)</f>
+        <v/>
+      </c>
+      <c r="F48" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F171),'Input ASM'!F171,0)+IF(ISNUMBER('Input ASM'!F172),'Input ASM'!F172,0)</f>
+        <v/>
+      </c>
+      <c r="G48" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G171),'Input ASM'!G171,0)+IF(ISNUMBER('Input ASM'!G172),'Input ASM'!G172,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Accounts Payable</t>
+        </is>
+      </c>
+      <c r="B49" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B185),'Input ASM'!B185,0)</f>
+        <v/>
+      </c>
+      <c r="C49" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C185),'Input ASM'!C185,0)</f>
+        <v/>
+      </c>
+      <c r="D49" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D185),'Input ASM'!D185,0)</f>
+        <v/>
+      </c>
+      <c r="E49" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E185),'Input ASM'!E185,0)</f>
+        <v/>
+      </c>
+      <c r="F49" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F185),'Input ASM'!F185,0)</f>
+        <v/>
+      </c>
+      <c r="G49" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G185),'Input ASM'!G185,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Accrued Expenses</t>
+        </is>
+      </c>
+      <c r="B50" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B186),'Input ASM'!B186,0)</f>
+        <v/>
+      </c>
+      <c r="C50" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C186),'Input ASM'!C186,0)</f>
+        <v/>
+      </c>
+      <c r="D50" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D186),'Input ASM'!D186,0)</f>
+        <v/>
+      </c>
+      <c r="E50" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E186),'Input ASM'!E186,0)</f>
+        <v/>
+      </c>
+      <c r="F50" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F186),'Input ASM'!F186,0)</f>
+        <v/>
+      </c>
+      <c r="G50" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G186),'Input ASM'!G186,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Unearned Revenue / Contract Liabilities</t>
+        </is>
+      </c>
+      <c r="B51" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B189),'Input ASM'!B189,0)</f>
+        <v/>
+      </c>
+      <c r="C51" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C189),'Input ASM'!C189,0)</f>
+        <v/>
+      </c>
+      <c r="D51" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D189),'Input ASM'!D189,0)</f>
+        <v/>
+      </c>
+      <c r="E51" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E189),'Input ASM'!E189,0)</f>
+        <v/>
+      </c>
+      <c r="F51" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F189),'Input ASM'!F189,0)</f>
+        <v/>
+      </c>
+      <c r="G51" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G189),'Input ASM'!G189,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Income Taxes Payable</t>
+        </is>
+      </c>
+      <c r="B52" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B188),'Input ASM'!B188,0)</f>
+        <v/>
+      </c>
+      <c r="C52" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C188),'Input ASM'!C188,0)</f>
+        <v/>
+      </c>
+      <c r="D52" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D188),'Input ASM'!D188,0)</f>
+        <v/>
+      </c>
+      <c r="E52" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E188),'Input ASM'!E188,0)</f>
+        <v/>
+      </c>
+      <c r="F52" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F188),'Input ASM'!F188,0)</f>
+        <v/>
+      </c>
+      <c r="G52" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G188),'Input ASM'!G188,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Other Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B53" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B190),'Input ASM'!B190,0)</f>
+        <v/>
+      </c>
+      <c r="C53" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C190),'Input ASM'!C190,0)</f>
+        <v/>
+      </c>
+      <c r="D53" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D190),'Input ASM'!D190,0)</f>
+        <v/>
+      </c>
+      <c r="E53" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E190),'Input ASM'!E190,0)</f>
+        <v/>
+      </c>
+      <c r="F53" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F190),'Input ASM'!F190,0)</f>
+        <v/>
+      </c>
+      <c r="G53" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G190),'Input ASM'!G190,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="24">
+        <f> Operating Working Capital</f>
+        <v/>
+      </c>
+      <c r="B54" s="25">
+        <f>B45+B46+B47+B48-B49-B50-B51-B52-B53</f>
+        <v/>
+      </c>
+      <c r="C54" s="25">
+        <f>C45+C46+C47+C48-C49-C50-C51-C52-C53</f>
+        <v/>
+      </c>
+      <c r="D54" s="25">
+        <f>D45+D46+D47+D48-D49-D50-D51-D52-D53</f>
+        <v/>
+      </c>
+      <c r="E54" s="25">
+        <f>E45+E46+E47+E48-E49-E50-E51-E52-E53</f>
+        <v/>
+      </c>
+      <c r="F54" s="25">
+        <f>F45+F46+F47+F48-F49-F50-F51-F52-F53</f>
+        <v/>
+      </c>
+      <c r="G54" s="25">
+        <f>G45+G46+G47+G48-G49-G50-G51-G52-G53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="22" t="inlineStr">
+        <is>
+          <t>Net Non-Current Operating Assets:</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PP&amp;E (net, incl. ROU)</t>
+        </is>
+      </c>
+      <c r="B57" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B176),'Input ASM'!B176,0)</f>
+        <v/>
+      </c>
+      <c r="C57" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C176),'Input ASM'!C176,0)</f>
+        <v/>
+      </c>
+      <c r="D57" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D176),'Input ASM'!D176,0)</f>
+        <v/>
+      </c>
+      <c r="E57" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E176),'Input ASM'!E176,0)</f>
+        <v/>
+      </c>
+      <c r="F57" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F176),'Input ASM'!F176,0)</f>
+        <v/>
+      </c>
+      <c r="G57" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G176),'Input ASM'!G176,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + Goodwill</t>
+        </is>
+      </c>
+      <c r="B58" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B178),'Input ASM'!B178,0)</f>
+        <v/>
+      </c>
+      <c r="C58" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C178),'Input ASM'!C178,0)</f>
+        <v/>
+      </c>
+      <c r="D58" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D178),'Input ASM'!D178,0)</f>
+        <v/>
+      </c>
+      <c r="E58" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E178),'Input ASM'!E178,0)</f>
+        <v/>
+      </c>
+      <c r="F58" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F178),'Input ASM'!F178,0)</f>
+        <v/>
+      </c>
+      <c r="G58" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G178),'Input ASM'!G178,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + Other Intangible Assets</t>
+        </is>
+      </c>
+      <c r="B59" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B179),'Input ASM'!B179,0)</f>
+        <v/>
+      </c>
+      <c r="C59" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C179),'Input ASM'!C179,0)</f>
+        <v/>
+      </c>
+      <c r="D59" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D179),'Input ASM'!D179,0)</f>
+        <v/>
+      </c>
+      <c r="E59" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E179),'Input ASM'!E179,0)</f>
+        <v/>
+      </c>
+      <c r="F59" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F179),'Input ASM'!F179,0)</f>
+        <v/>
+      </c>
+      <c r="G59" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G179),'Input ASM'!G179,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + Deferred Tax Assets</t>
+        </is>
+      </c>
+      <c r="B60" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B180),'Input ASM'!B180,0)</f>
+        <v/>
+      </c>
+      <c r="C60" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C180),'Input ASM'!C180,0)</f>
+        <v/>
+      </c>
+      <c r="D60" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D180),'Input ASM'!D180,0)</f>
+        <v/>
+      </c>
+      <c r="E60" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E180),'Input ASM'!E180,0)</f>
+        <v/>
+      </c>
+      <c r="F60" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F180),'Input ASM'!F180,0)</f>
+        <v/>
+      </c>
+      <c r="G60" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G180),'Input ASM'!G180,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + Deferred Charges &amp; LT Intangibles</t>
+        </is>
+      </c>
+      <c r="B61" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B181),'Input ASM'!B181,0)</f>
+        <v/>
+      </c>
+      <c r="C61" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C181),'Input ASM'!C181,0)</f>
+        <v/>
+      </c>
+      <c r="D61" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D181),'Input ASM'!D181,0)</f>
+        <v/>
+      </c>
+      <c r="E61" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E181),'Input ASM'!E181,0)</f>
+        <v/>
+      </c>
+      <c r="F61" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F181),'Input ASM'!F181,0)</f>
+        <v/>
+      </c>
+      <c r="G61" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G181),'Input ASM'!G181,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + Other Non-Current Assets</t>
+        </is>
+      </c>
+      <c r="B62" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B182),'Input ASM'!B182,0)</f>
+        <v/>
+      </c>
+      <c r="C62" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C182),'Input ASM'!C182,0)</f>
+        <v/>
+      </c>
+      <c r="D62" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D182),'Input ASM'!D182,0)</f>
+        <v/>
+      </c>
+      <c r="E62" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E182),'Input ASM'!E182,0)</f>
+        <v/>
+      </c>
+      <c r="F62" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F182),'Input ASM'!F182,0)</f>
+        <v/>
+      </c>
+      <c r="G62" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G182),'Input ASM'!G182,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Deferred Tax Liabilities</t>
+        </is>
+      </c>
+      <c r="B63" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B193),'Input ASM'!B193,0)</f>
+        <v/>
+      </c>
+      <c r="C63" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C193),'Input ASM'!C193,0)</f>
+        <v/>
+      </c>
+      <c r="D63" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D193),'Input ASM'!D193,0)</f>
+        <v/>
+      </c>
+      <c r="E63" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E193),'Input ASM'!E193,0)</f>
+        <v/>
+      </c>
+      <c r="F63" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F193),'Input ASM'!F193,0)</f>
+        <v/>
+      </c>
+      <c r="G63" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G193),'Input ASM'!G193,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Other Non-Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B64" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B194),'Input ASM'!B194,0)</f>
+        <v/>
+      </c>
+      <c r="C64" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C194),'Input ASM'!C194,0)</f>
+        <v/>
+      </c>
+      <c r="D64" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D194),'Input ASM'!D194,0)</f>
+        <v/>
+      </c>
+      <c r="E64" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E194),'Input ASM'!E194,0)</f>
+        <v/>
+      </c>
+      <c r="F64" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F194),'Input ASM'!F194,0)</f>
+        <v/>
+      </c>
+      <c r="G64" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G194),'Input ASM'!G194,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="24">
+        <f> Net Non-Current Operating Assets</f>
+        <v/>
+      </c>
+      <c r="B65" s="25">
+        <f>B57+B58+B59+B60+B61+B62-B63-B64</f>
+        <v/>
+      </c>
+      <c r="C65" s="25">
+        <f>C57+C58+C59+C60+C61+C62-C63-C64</f>
+        <v/>
+      </c>
+      <c r="D65" s="25">
+        <f>D57+D58+D59+D60+D61+D62-D63-D64</f>
+        <v/>
+      </c>
+      <c r="E65" s="25">
+        <f>E57+E58+E59+E60+E61+E62-E63-E64</f>
+        <v/>
+      </c>
+      <c r="F65" s="25">
+        <f>F57+F58+F59+F60+F61+F62-F63-F64</f>
+        <v/>
+      </c>
+      <c r="G65" s="25">
+        <f>G57+G58+G59+G60+G61+G62-G63-G64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="24">
+        <f> Net Operating Assets</f>
+        <v/>
+      </c>
+      <c r="B67" s="25">
+        <f>B54+B65</f>
+        <v/>
+      </c>
+      <c r="C67" s="25">
+        <f>C54+C65</f>
+        <v/>
+      </c>
+      <c r="D67" s="25">
+        <f>D54+D65</f>
+        <v/>
+      </c>
+      <c r="E67" s="25">
+        <f>E54+E65</f>
+        <v/>
+      </c>
+      <c r="F67" s="25">
+        <f>F54+F65</f>
+        <v/>
+      </c>
+      <c r="G67" s="25">
+        <f>G54+G65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="22" t="inlineStr">
+        <is>
+          <t>Investment Assets:</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Long-Term Investments</t>
+        </is>
+      </c>
+      <c r="B70" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B177),'Input ASM'!B177,0)</f>
+        <v/>
+      </c>
+      <c r="C70" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C177),'Input ASM'!C177,0)</f>
+        <v/>
+      </c>
+      <c r="D70" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D177),'Input ASM'!D177,0)</f>
+        <v/>
+      </c>
+      <c r="E70" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E177),'Input ASM'!E177,0)</f>
+        <v/>
+      </c>
+      <c r="F70" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F177),'Input ASM'!F177,0)</f>
+        <v/>
+      </c>
+      <c r="G70" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G177),'Input ASM'!G177,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="24">
+        <f> Total Investment Assets</f>
+        <v/>
+      </c>
+      <c r="B71" s="25">
+        <f>B70</f>
+        <v/>
+      </c>
+      <c r="C71" s="25">
+        <f>C70</f>
+        <v/>
+      </c>
+      <c r="D71" s="25">
+        <f>D70</f>
+        <v/>
+      </c>
+      <c r="E71" s="25">
+        <f>E70</f>
+        <v/>
+      </c>
+      <c r="F71" s="25">
+        <f>F70</f>
+        <v/>
+      </c>
+      <c r="G71" s="25">
+        <f>G70</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="26">
+        <f> Business Assets</f>
+        <v/>
+      </c>
+      <c r="B73" s="27">
+        <f>B67+B71</f>
+        <v/>
+      </c>
+      <c r="C73" s="27">
+        <f>C67+C71</f>
+        <v/>
+      </c>
+      <c r="D73" s="27">
+        <f>D67+D71</f>
+        <v/>
+      </c>
+      <c r="E73" s="27">
+        <f>E67+E71</f>
+        <v/>
+      </c>
+      <c r="F73" s="27">
+        <f>F67+F71</f>
+        <v/>
+      </c>
+      <c r="G73" s="27">
+        <f>G67+G71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="19" t="inlineStr">
+        <is>
+          <t>FINANCING</t>
+        </is>
+      </c>
+      <c r="B75" s="20" t="n"/>
+      <c r="C75" s="20" t="n"/>
+      <c r="D75" s="20" t="n"/>
+      <c r="E75" s="20" t="n"/>
+      <c r="F75" s="20" t="n"/>
+      <c r="G75" s="20" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lease Liabilities (current)</t>
+        </is>
+      </c>
+      <c r="B76" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B187),'Input ASM'!B187,0)</f>
+        <v/>
+      </c>
+      <c r="C76" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C187),'Input ASM'!C187,0)</f>
+        <v/>
+      </c>
+      <c r="D76" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D187),'Input ASM'!D187,0)</f>
+        <v/>
+      </c>
+      <c r="E76" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E187),'Input ASM'!E187,0)</f>
+        <v/>
+      </c>
+      <c r="F76" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F187),'Input ASM'!F187,0)</f>
+        <v/>
+      </c>
+      <c r="G76" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G187),'Input ASM'!G187,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + Lease Liabilities (non-current)</t>
+        </is>
+      </c>
+      <c r="B77" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B192),'Input ASM'!B192,0)</f>
+        <v/>
+      </c>
+      <c r="C77" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C192),'Input ASM'!C192,0)</f>
+        <v/>
+      </c>
+      <c r="D77" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D192),'Input ASM'!D192,0)</f>
+        <v/>
+      </c>
+      <c r="E77" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E192),'Input ASM'!E192,0)</f>
+        <v/>
+      </c>
+      <c r="F77" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F192),'Input ASM'!F192,0)</f>
+        <v/>
+      </c>
+      <c r="G77" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G192),'Input ASM'!G192,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="24">
+        <f> Total Debt</f>
+        <v/>
+      </c>
+      <c r="B78" s="25">
+        <f>B76+B77</f>
+        <v/>
+      </c>
+      <c r="C78" s="25">
+        <f>C76+C77</f>
+        <v/>
+      </c>
+      <c r="D78" s="25">
+        <f>D76+D77</f>
+        <v/>
+      </c>
+      <c r="E78" s="25">
+        <f>E76+E77</f>
+        <v/>
+      </c>
+      <c r="F78" s="25">
+        <f>F76+F77</f>
+        <v/>
+      </c>
+      <c r="G78" s="25">
+        <f>G76+G77</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Cash &amp; Equivalents</t>
+        </is>
+      </c>
+      <c r="B79" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B165),'Input ASM'!B165,0)</f>
+        <v/>
+      </c>
+      <c r="C79" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C165),'Input ASM'!C165,0)</f>
+        <v/>
+      </c>
+      <c r="D79" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D165),'Input ASM'!D165,0)</f>
+        <v/>
+      </c>
+      <c r="E79" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E165),'Input ASM'!E165,0)</f>
+        <v/>
+      </c>
+      <c r="F79" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F165),'Input ASM'!F165,0)</f>
+        <v/>
+      </c>
+      <c r="G79" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G165),'Input ASM'!G165,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="22">
+        <f> Net Debt</f>
+        <v/>
+      </c>
+      <c r="B80" s="23">
+        <f>B78-B79</f>
+        <v/>
+      </c>
+      <c r="C80" s="23">
+        <f>C78-C79</f>
+        <v/>
+      </c>
+      <c r="D80" s="23">
+        <f>D78-D79</f>
+        <v/>
+      </c>
+      <c r="E80" s="23">
+        <f>E78-E79</f>
+        <v/>
+      </c>
+      <c r="F80" s="23">
+        <f>F78-F79</f>
+        <v/>
+      </c>
+      <c r="G80" s="23">
+        <f>G78-G79</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="11" t="inlineStr">
+        <is>
+          <t>Group Equity</t>
+        </is>
+      </c>
+      <c r="B81" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B203),'Input ASM'!B203,0)</f>
+        <v/>
+      </c>
+      <c r="C81" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C203),'Input ASM'!C203,0)</f>
+        <v/>
+      </c>
+      <c r="D81" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D203),'Input ASM'!D203,0)</f>
+        <v/>
+      </c>
+      <c r="E81" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E203),'Input ASM'!E203,0)</f>
+        <v/>
+      </c>
+      <c r="F81" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F203),'Input ASM'!F203,0)</f>
+        <v/>
+      </c>
+      <c r="G81" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G203),'Input ASM'!G203,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="26">
+        <f> Invested Capital</f>
+        <v/>
+      </c>
+      <c r="B82" s="27">
+        <f>B80+B81</f>
+        <v/>
+      </c>
+      <c r="C82" s="27">
+        <f>C80+C81</f>
+        <v/>
+      </c>
+      <c r="D82" s="27">
+        <f>D80+D81</f>
+        <v/>
+      </c>
+      <c r="E82" s="27">
+        <f>E80+E81</f>
+        <v/>
+      </c>
+      <c r="F82" s="27">
+        <f>F80+F81</f>
+        <v/>
+      </c>
+      <c r="G82" s="27">
+        <f>G80+G81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="22" t="inlineStr">
+        <is>
+          <t>BS Check (should = 0)</t>
+        </is>
+      </c>
+      <c r="B83" s="23">
+        <f>B73-B82</f>
+        <v/>
+      </c>
+      <c r="C83" s="23">
+        <f>C73-C82</f>
+        <v/>
+      </c>
+      <c r="D83" s="23">
+        <f>D73-D82</f>
+        <v/>
+      </c>
+      <c r="E83" s="23">
+        <f>E73-E82</f>
+        <v/>
+      </c>
+      <c r="F83" s="23">
+        <f>F73-F82</f>
+        <v/>
+      </c>
+      <c r="G83" s="23">
+        <f>G73-G82</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="19" t="inlineStr">
+        <is>
+          <t>FREE CASH FLOW</t>
+        </is>
+      </c>
+      <c r="B86" s="20" t="n"/>
+      <c r="C86" s="20" t="n"/>
+      <c r="D86" s="20" t="n"/>
+      <c r="E86" s="20" t="n"/>
+      <c r="F86" s="20" t="n"/>
+      <c r="G86" s="20" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="11" t="inlineStr">
+        <is>
+          <t>NOPAT</t>
+        </is>
+      </c>
+      <c r="B87" s="31">
+        <f>B36</f>
+        <v/>
+      </c>
+      <c r="C87" s="31">
+        <f>C36</f>
+        <v/>
+      </c>
+      <c r="D87" s="31">
+        <f>D36</f>
+        <v/>
+      </c>
+      <c r="E87" s="31">
+        <f>E36</f>
+        <v/>
+      </c>
+      <c r="F87" s="31">
+        <f>F36</f>
+        <v/>
+      </c>
+      <c r="G87" s="31">
+        <f>G36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="11" t="inlineStr">
+        <is>
+          <t>+ D&amp;A</t>
+        </is>
+      </c>
+      <c r="B88" s="21">
+        <f>IF(ISNUMBER('Input ASM'!B113),'Input ASM'!B113,0)</f>
+        <v/>
+      </c>
+      <c r="C88" s="21">
+        <f>IF(ISNUMBER('Input ASM'!C113),'Input ASM'!C113,0)</f>
+        <v/>
+      </c>
+      <c r="D88" s="21">
+        <f>IF(ISNUMBER('Input ASM'!D113),'Input ASM'!D113,0)</f>
+        <v/>
+      </c>
+      <c r="E88" s="21">
+        <f>IF(ISNUMBER('Input ASM'!E113),'Input ASM'!E113,0)</f>
+        <v/>
+      </c>
+      <c r="F88" s="21">
+        <f>IF(ISNUMBER('Input ASM'!F113),'Input ASM'!F113,0)</f>
+        <v/>
+      </c>
+      <c r="G88" s="21">
+        <f>IF(ISNUMBER('Input ASM'!G113),'Input ASM'!G113,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="11" t="inlineStr">
+        <is>
+          <t>- Change in OWC</t>
+        </is>
+      </c>
+      <c r="B89" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="C89" s="31">
+        <f>C54-B54</f>
+        <v/>
+      </c>
+      <c r="D89" s="31">
+        <f>D54-C54</f>
+        <v/>
+      </c>
+      <c r="E89" s="31">
+        <f>E54-D54</f>
+        <v/>
+      </c>
+      <c r="F89" s="31">
+        <f>F54-E54</f>
+        <v/>
+      </c>
+      <c r="G89" s="31">
+        <f>G54-F54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="11" t="inlineStr">
+        <is>
+          <t>- CapEx</t>
+        </is>
+      </c>
+      <c r="B90" s="21">
+        <f>ABS(IF(ISNUMBER('Input ASM'!B127),'Input ASM'!B127,0))</f>
+        <v/>
+      </c>
+      <c r="C90" s="21">
+        <f>ABS(IF(ISNUMBER('Input ASM'!C127),'Input ASM'!C127,0))</f>
+        <v/>
+      </c>
+      <c r="D90" s="21">
+        <f>ABS(IF(ISNUMBER('Input ASM'!D127),'Input ASM'!D127,0))</f>
+        <v/>
+      </c>
+      <c r="E90" s="21">
+        <f>ABS(IF(ISNUMBER('Input ASM'!E127),'Input ASM'!E127,0))</f>
+        <v/>
+      </c>
+      <c r="F90" s="21">
+        <f>ABS(IF(ISNUMBER('Input ASM'!F127),'Input ASM'!F127,0))</f>
+        <v/>
+      </c>
+      <c r="G90" s="21">
+        <f>ABS(IF(ISNUMBER('Input ASM'!G127),'Input ASM'!G127,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="11" t="inlineStr">
+        <is>
+          <t>- Purchase of Intangibles</t>
+        </is>
+      </c>
+      <c r="B91" s="21">
+        <f>ABS(IF(ISNUMBER('Input ASM'!B130),'Input ASM'!B130,0))</f>
+        <v/>
+      </c>
+      <c r="C91" s="21">
+        <f>ABS(IF(ISNUMBER('Input ASM'!C130),'Input ASM'!C130,0))</f>
+        <v/>
+      </c>
+      <c r="D91" s="21">
+        <f>ABS(IF(ISNUMBER('Input ASM'!D130),'Input ASM'!D130,0))</f>
+        <v/>
+      </c>
+      <c r="E91" s="21">
+        <f>ABS(IF(ISNUMBER('Input ASM'!E130),'Input ASM'!E130,0))</f>
+        <v/>
+      </c>
+      <c r="F91" s="21">
+        <f>ABS(IF(ISNUMBER('Input ASM'!F130),'Input ASM'!F130,0))</f>
+        <v/>
+      </c>
+      <c r="G91" s="21">
+        <f>ABS(IF(ISNUMBER('Input ASM'!G130),'Input ASM'!G130,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="24">
+        <f> Operating CF after investment</f>
+        <v/>
+      </c>
+      <c r="B92" s="25">
+        <f>B87+B88-B89-B90-B91</f>
+        <v/>
+      </c>
+      <c r="C92" s="25">
+        <f>C87+C88-C89-C90-C91</f>
+        <v/>
+      </c>
+      <c r="D92" s="25">
+        <f>D87+D88-D89-D90-D91</f>
+        <v/>
+      </c>
+      <c r="E92" s="25">
+        <f>E87+E88-E89-E90-E91</f>
+        <v/>
+      </c>
+      <c r="F92" s="25">
+        <f>F87+F88-F89-F90-F91</f>
+        <v/>
+      </c>
+      <c r="G92" s="25">
+        <f>G87+G88-G89-G90-G91</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="11" t="inlineStr">
+        <is>
+          <t>+ Net Investment Profit after tax</t>
+        </is>
+      </c>
+      <c r="B94" s="31">
+        <f>B27*(1-B35)</f>
+        <v/>
+      </c>
+      <c r="C94" s="31">
+        <f>C27*(1-C35)</f>
+        <v/>
+      </c>
+      <c r="D94" s="31">
+        <f>D27*(1-D35)</f>
+        <v/>
+      </c>
+      <c r="E94" s="31">
+        <f>E27*(1-E35)</f>
+        <v/>
+      </c>
+      <c r="F94" s="31">
+        <f>F27*(1-F35)</f>
+        <v/>
+      </c>
+      <c r="G94" s="31">
+        <f>G27*(1-G35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="11" t="inlineStr">
+        <is>
+          <t>- Change in Investment Assets</t>
+        </is>
+      </c>
+      <c r="B95" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="C95" s="31">
+        <f>C71-B71</f>
+        <v/>
+      </c>
+      <c r="D95" s="31">
+        <f>D71-C71</f>
+        <v/>
+      </c>
+      <c r="E95" s="31">
+        <f>E71-D71</f>
+        <v/>
+      </c>
+      <c r="F95" s="31">
+        <f>F71-E71</f>
+        <v/>
+      </c>
+      <c r="G95" s="31">
+        <f>G71-F71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="24">
+        <f> FCF to Debt &amp; Equity</f>
+        <v/>
+      </c>
+      <c r="B96" s="25">
+        <f>B92+B94-B95</f>
+        <v/>
+      </c>
+      <c r="C96" s="25">
+        <f>C92+C94-C95</f>
+        <v/>
+      </c>
+      <c r="D96" s="25">
+        <f>D92+D94-D95</f>
+        <v/>
+      </c>
+      <c r="E96" s="25">
+        <f>E92+E94-E95</f>
+        <v/>
+      </c>
+      <c r="F96" s="25">
+        <f>F92+F94-F95</f>
+        <v/>
+      </c>
+      <c r="G96" s="25">
+        <f>G92+G94-G95</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="11" t="inlineStr">
+        <is>
+          <t>- Interest Expense after tax</t>
+        </is>
+      </c>
+      <c r="B97" s="31">
+        <f>B29*(1-B35)</f>
+        <v/>
+      </c>
+      <c r="C97" s="31">
+        <f>C29*(1-C35)</f>
+        <v/>
+      </c>
+      <c r="D97" s="31">
+        <f>D29*(1-D35)</f>
+        <v/>
+      </c>
+      <c r="E97" s="31">
+        <f>E29*(1-E35)</f>
+        <v/>
+      </c>
+      <c r="F97" s="31">
+        <f>F29*(1-F35)</f>
+        <v/>
+      </c>
+      <c r="G97" s="31">
+        <f>G29*(1-G35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="11" t="inlineStr">
+        <is>
+          <t>+ Change in Debt</t>
+        </is>
+      </c>
+      <c r="B98" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="C98" s="31">
+        <f>C78-B78</f>
+        <v/>
+      </c>
+      <c r="D98" s="31">
+        <f>D78-C78</f>
+        <v/>
+      </c>
+      <c r="E98" s="31">
+        <f>E78-D78</f>
+        <v/>
+      </c>
+      <c r="F98" s="31">
+        <f>F78-E78</f>
+        <v/>
+      </c>
+      <c r="G98" s="31">
+        <f>G78-F78</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="26">
+        <f> FCF to Equity</f>
+        <v/>
+      </c>
+      <c r="B99" s="27">
+        <f>B96-B97+B98</f>
+        <v/>
+      </c>
+      <c r="C99" s="27">
+        <f>C96-C97+C98</f>
+        <v/>
+      </c>
+      <c r="D99" s="27">
+        <f>D96-D97+D98</f>
+        <v/>
+      </c>
+      <c r="E99" s="27">
+        <f>E96-E97+E98</f>
+        <v/>
+      </c>
+      <c r="F99" s="27">
+        <f>F96-F97+F98</f>
+        <v/>
+      </c>
+      <c r="G99" s="27">
+        <f>G96-G97+G98</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add Forecast tab with assumptions, IS, BS, and FCF projections
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/ASM_Valuation_Model.xlsx
+++ b/output/ASM_Valuation_Model.xlsx
@@ -28,6 +28,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratios AMAT" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratios LRCX" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratio Comparison" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -178,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -228,6 +229,7 @@
     <xf numFmtId="168" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -24364,6 +24366,2220 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J68"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>ASM International NV - Financial Forecast</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>(EUR 000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="22" t="n"/>
+      <c r="B3" s="16" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C3" s="16" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D3" s="16" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>2025E</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>2028E</t>
+        </is>
+      </c>
+      <c r="I3" s="16" t="inlineStr">
+        <is>
+          <t>2029E</t>
+        </is>
+      </c>
+      <c r="J3" s="16" t="inlineStr">
+        <is>
+          <t>2030E</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>FORECAST ASSUMPTIONS</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="n"/>
+      <c r="C5" s="20" t="n"/>
+      <c r="D5" s="20" t="n"/>
+      <c r="E5" s="20" t="n"/>
+      <c r="F5" s="20" t="n"/>
+      <c r="G5" s="20" t="n"/>
+      <c r="H5" s="20" t="n"/>
+      <c r="I5" s="20" t="n"/>
+      <c r="J5" s="20" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Revenue Growth Rate</t>
+        </is>
+      </c>
+      <c r="B6" s="28">
+        <f>IF('Adj ASM'!D9&lt;&gt;0,'Adj ASM'!E9/'Adj ASM'!D9-1,0)</f>
+        <v/>
+      </c>
+      <c r="C6" s="28">
+        <f>IF('Adj ASM'!E9&lt;&gt;0,'Adj ASM'!F9/'Adj ASM'!E9-1,0)</f>
+        <v/>
+      </c>
+      <c r="D6" s="28">
+        <f>IF('Adj ASM'!F9&lt;&gt;0,'Adj ASM'!G9/'Adj ASM'!F9-1,0)</f>
+        <v/>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G6" s="17" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H6" s="17" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="I6" s="17" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J6" s="17" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Gross Profit Margin</t>
+        </is>
+      </c>
+      <c r="B7" s="28">
+        <f>IF('Adj ASM'!E9&lt;&gt;0,'Adj ASM'!E11/'Adj ASM'!E9,0)</f>
+        <v/>
+      </c>
+      <c r="C7" s="28">
+        <f>IF('Adj ASM'!F9&lt;&gt;0,'Adj ASM'!F11/'Adj ASM'!F9,0)</f>
+        <v/>
+      </c>
+      <c r="D7" s="28">
+        <f>IF('Adj ASM'!G9&lt;&gt;0,'Adj ASM'!G11/'Adj ASM'!G9,0)</f>
+        <v/>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>0.505</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <v>0.505</v>
+      </c>
+      <c r="G7" s="17" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="H7" s="17" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="I7" s="17" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J7" s="17" t="n">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>SG&amp;A / Revenue</t>
+        </is>
+      </c>
+      <c r="B8" s="28">
+        <f>IF('Adj ASM'!E9&lt;&gt;0,'Adj ASM'!E12/'Adj ASM'!E9,0)</f>
+        <v/>
+      </c>
+      <c r="C8" s="28">
+        <f>IF('Adj ASM'!F9&lt;&gt;0,'Adj ASM'!F12/'Adj ASM'!F9,0)</f>
+        <v/>
+      </c>
+      <c r="D8" s="28">
+        <f>IF('Adj ASM'!G9&lt;&gt;0,'Adj ASM'!G12/'Adj ASM'!G9,0)</f>
+        <v/>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>0.108</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="H8" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I8" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J8" s="17" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>R&amp;D / Revenue</t>
+        </is>
+      </c>
+      <c r="B9" s="28">
+        <f>IF('Adj ASM'!E9&lt;&gt;0,'Adj ASM'!E13/'Adj ASM'!E9,0)</f>
+        <v/>
+      </c>
+      <c r="C9" s="28">
+        <f>IF('Adj ASM'!F9&lt;&gt;0,'Adj ASM'!F13/'Adj ASM'!F9,0)</f>
+        <v/>
+      </c>
+      <c r="D9" s="28">
+        <f>IF('Adj ASM'!G9&lt;&gt;0,'Adj ASM'!G13/'Adj ASM'!G9,0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>0.126</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I9" s="17" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="J9" s="17" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>D&amp;A / Revenue</t>
+        </is>
+      </c>
+      <c r="B10" s="28">
+        <f>IF('Adj ASM'!E9&lt;&gt;0,'Adj ASM'!E14/'Adj ASM'!E9,0)</f>
+        <v/>
+      </c>
+      <c r="C10" s="28">
+        <f>IF('Adj ASM'!F9&lt;&gt;0,'Adj ASM'!F14/'Adj ASM'!F9,0)</f>
+        <v/>
+      </c>
+      <c r="D10" s="28">
+        <f>IF('Adj ASM'!G9&lt;&gt;0,'Adj ASM'!G14/'Adj ASM'!G9,0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="G10" s="17" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="H10" s="17" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="I10" s="17" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="J10" s="17" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Tax Rate</t>
+        </is>
+      </c>
+      <c r="B11" s="28">
+        <f>'Adj ASM'!E35</f>
+        <v/>
+      </c>
+      <c r="C11" s="28">
+        <f>'Adj ASM'!F35</f>
+        <v/>
+      </c>
+      <c r="D11" s="28">
+        <f>'Adj ASM'!G35</f>
+        <v/>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="G11" s="17" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="H11" s="17" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="I11" s="17" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="J11" s="17" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>OWC / Revenue</t>
+        </is>
+      </c>
+      <c r="B12" s="28">
+        <f>IF('Adj ASM'!E9&lt;&gt;0,'Adj ASM'!E54/'Adj ASM'!E9,0)</f>
+        <v/>
+      </c>
+      <c r="C12" s="28">
+        <f>IF('Adj ASM'!F9&lt;&gt;0,'Adj ASM'!F54/'Adj ASM'!F9,0)</f>
+        <v/>
+      </c>
+      <c r="D12" s="28">
+        <f>IF('Adj ASM'!G9&lt;&gt;0,'Adj ASM'!G54/'Adj ASM'!G9,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G12" s="17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H12" s="17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I12" s="17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J12" s="17" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Net NCA / Revenue</t>
+        </is>
+      </c>
+      <c r="B13" s="28">
+        <f>IF('Adj ASM'!E9&lt;&gt;0,'Adj ASM'!E65/'Adj ASM'!E9,0)</f>
+        <v/>
+      </c>
+      <c r="C13" s="28">
+        <f>IF('Adj ASM'!F9&lt;&gt;0,'Adj ASM'!F65/'Adj ASM'!F9,0)</f>
+        <v/>
+      </c>
+      <c r="D13" s="28">
+        <f>IF('Adj ASM'!G9&lt;&gt;0,'Adj ASM'!G65/'Adj ASM'!G9,0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="H13" s="17" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="I13" s="17" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="J13" s="17" t="n">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Investment Assets / Revenue</t>
+        </is>
+      </c>
+      <c r="B14" s="28">
+        <f>IF('Adj ASM'!E9&lt;&gt;0,'Adj ASM'!E71/'Adj ASM'!E9,0)</f>
+        <v/>
+      </c>
+      <c r="C14" s="28">
+        <f>IF('Adj ASM'!F9&lt;&gt;0,'Adj ASM'!F71/'Adj ASM'!F9,0)</f>
+        <v/>
+      </c>
+      <c r="D14" s="28">
+        <f>IF('Adj ASM'!G9&lt;&gt;0,'Adj ASM'!G71/'Adj ASM'!G9,0)</f>
+        <v/>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="G14" s="17" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="H14" s="17" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="I14" s="17" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="J14" s="17" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Debt / Capital</t>
+        </is>
+      </c>
+      <c r="B15" s="28">
+        <f>IF('Adj ASM'!E82&lt;&gt;0,'Adj ASM'!E78/'Adj ASM'!E82,0)</f>
+        <v/>
+      </c>
+      <c r="C15" s="28">
+        <f>IF('Adj ASM'!F82&lt;&gt;0,'Adj ASM'!F78/'Adj ASM'!F82,0)</f>
+        <v/>
+      </c>
+      <c r="D15" s="28">
+        <f>IF('Adj ASM'!G82&lt;&gt;0,'Adj ASM'!G78/'Adj ASM'!G82,0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G15" s="17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H15" s="17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I15" s="17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J15" s="17" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Terminal Growth Rate</t>
+        </is>
+      </c>
+      <c r="J16" s="17" t="n">
+        <v>0.025</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>CONDENSED INCOME STATEMENT</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="n"/>
+      <c r="C18" s="20" t="n"/>
+      <c r="D18" s="20" t="n"/>
+      <c r="E18" s="20" t="n"/>
+      <c r="F18" s="20" t="n"/>
+      <c r="G18" s="20" t="n"/>
+      <c r="H18" s="20" t="n"/>
+      <c r="I18" s="20" t="n"/>
+      <c r="J18" s="20" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B19" s="21">
+        <f>'Adj ASM'!E9</f>
+        <v/>
+      </c>
+      <c r="C19" s="21">
+        <f>'Adj ASM'!F9</f>
+        <v/>
+      </c>
+      <c r="D19" s="21">
+        <f>'Adj ASM'!G9</f>
+        <v/>
+      </c>
+      <c r="E19" s="23">
+        <f>D19*(1+E6)</f>
+        <v/>
+      </c>
+      <c r="F19" s="23">
+        <f>E19*(1+F6)</f>
+        <v/>
+      </c>
+      <c r="G19" s="23">
+        <f>F19*(1+G6)</f>
+        <v/>
+      </c>
+      <c r="H19" s="23">
+        <f>G19*(1+H6)</f>
+        <v/>
+      </c>
+      <c r="I19" s="23">
+        <f>H19*(1+I6)</f>
+        <v/>
+      </c>
+      <c r="J19" s="23">
+        <f>I19*(1+J6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Revenue Growth</t>
+        </is>
+      </c>
+      <c r="B20" s="28">
+        <f>B6</f>
+        <v/>
+      </c>
+      <c r="C20" s="28">
+        <f>C6</f>
+        <v/>
+      </c>
+      <c r="D20" s="28">
+        <f>D6</f>
+        <v/>
+      </c>
+      <c r="E20" s="28">
+        <f>E6</f>
+        <v/>
+      </c>
+      <c r="F20" s="28">
+        <f>F6</f>
+        <v/>
+      </c>
+      <c r="G20" s="28">
+        <f>G6</f>
+        <v/>
+      </c>
+      <c r="H20" s="28">
+        <f>H6</f>
+        <v/>
+      </c>
+      <c r="I20" s="28">
+        <f>I6</f>
+        <v/>
+      </c>
+      <c r="J20" s="28">
+        <f>J6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>Gross Profit</t>
+        </is>
+      </c>
+      <c r="B22" s="21">
+        <f>'Adj ASM'!E11</f>
+        <v/>
+      </c>
+      <c r="C22" s="21">
+        <f>'Adj ASM'!F11</f>
+        <v/>
+      </c>
+      <c r="D22" s="21">
+        <f>'Adj ASM'!G11</f>
+        <v/>
+      </c>
+      <c r="E22" s="23">
+        <f>E19*E7</f>
+        <v/>
+      </c>
+      <c r="F22" s="23">
+        <f>F19*F7</f>
+        <v/>
+      </c>
+      <c r="G22" s="23">
+        <f>G19*G7</f>
+        <v/>
+      </c>
+      <c r="H22" s="23">
+        <f>H19*H7</f>
+        <v/>
+      </c>
+      <c r="I22" s="23">
+        <f>I19*I7</f>
+        <v/>
+      </c>
+      <c r="J22" s="23">
+        <f>J19*J7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Gross Margin</t>
+        </is>
+      </c>
+      <c r="B23" s="28">
+        <f>IF(B19&lt;&gt;0,B22/B19,0)</f>
+        <v/>
+      </c>
+      <c r="C23" s="28">
+        <f>IF(C19&lt;&gt;0,C22/C19,0)</f>
+        <v/>
+      </c>
+      <c r="D23" s="28">
+        <f>IF(D19&lt;&gt;0,D22/D19,0)</f>
+        <v/>
+      </c>
+      <c r="E23" s="28">
+        <f>E7</f>
+        <v/>
+      </c>
+      <c r="F23" s="28">
+        <f>F7</f>
+        <v/>
+      </c>
+      <c r="G23" s="28">
+        <f>G7</f>
+        <v/>
+      </c>
+      <c r="H23" s="28">
+        <f>H7</f>
+        <v/>
+      </c>
+      <c r="I23" s="28">
+        <f>I7</f>
+        <v/>
+      </c>
+      <c r="J23" s="28">
+        <f>J7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SG&amp;A</t>
+        </is>
+      </c>
+      <c r="B24" s="21">
+        <f>'Adj ASM'!E12</f>
+        <v/>
+      </c>
+      <c r="C24" s="21">
+        <f>'Adj ASM'!F12</f>
+        <v/>
+      </c>
+      <c r="D24" s="21">
+        <f>'Adj ASM'!G12</f>
+        <v/>
+      </c>
+      <c r="E24" s="31">
+        <f>E19*E8</f>
+        <v/>
+      </c>
+      <c r="F24" s="31">
+        <f>F19*F8</f>
+        <v/>
+      </c>
+      <c r="G24" s="31">
+        <f>G19*G8</f>
+        <v/>
+      </c>
+      <c r="H24" s="31">
+        <f>H19*H8</f>
+        <v/>
+      </c>
+      <c r="I24" s="31">
+        <f>I19*I8</f>
+        <v/>
+      </c>
+      <c r="J24" s="31">
+        <f>J19*J8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  R&amp;D</t>
+        </is>
+      </c>
+      <c r="B25" s="21">
+        <f>'Adj ASM'!E13</f>
+        <v/>
+      </c>
+      <c r="C25" s="21">
+        <f>'Adj ASM'!F13</f>
+        <v/>
+      </c>
+      <c r="D25" s="21">
+        <f>'Adj ASM'!G13</f>
+        <v/>
+      </c>
+      <c r="E25" s="31">
+        <f>E19*E9</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>F19*F9</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>G19*G9</f>
+        <v/>
+      </c>
+      <c r="H25" s="31">
+        <f>H19*H9</f>
+        <v/>
+      </c>
+      <c r="I25" s="31">
+        <f>I19*I9</f>
+        <v/>
+      </c>
+      <c r="J25" s="31">
+        <f>J19*J9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D&amp;A</t>
+        </is>
+      </c>
+      <c r="B26" s="21">
+        <f>'Adj ASM'!E14</f>
+        <v/>
+      </c>
+      <c r="C26" s="21">
+        <f>'Adj ASM'!F14</f>
+        <v/>
+      </c>
+      <c r="D26" s="21">
+        <f>'Adj ASM'!G14</f>
+        <v/>
+      </c>
+      <c r="E26" s="31">
+        <f>E19*E10</f>
+        <v/>
+      </c>
+      <c r="F26" s="31">
+        <f>F19*F10</f>
+        <v/>
+      </c>
+      <c r="G26" s="31">
+        <f>G19*G10</f>
+        <v/>
+      </c>
+      <c r="H26" s="31">
+        <f>H19*H10</f>
+        <v/>
+      </c>
+      <c r="I26" s="31">
+        <f>I19*I10</f>
+        <v/>
+      </c>
+      <c r="J26" s="31">
+        <f>J19*J10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="24" t="inlineStr">
+        <is>
+          <t>EBIT</t>
+        </is>
+      </c>
+      <c r="B27" s="25">
+        <f>'Adj ASM'!E25</f>
+        <v/>
+      </c>
+      <c r="C27" s="25">
+        <f>'Adj ASM'!F25</f>
+        <v/>
+      </c>
+      <c r="D27" s="25">
+        <f>'Adj ASM'!G25</f>
+        <v/>
+      </c>
+      <c r="E27" s="25">
+        <f>E22-E24-E25-E26</f>
+        <v/>
+      </c>
+      <c r="F27" s="25">
+        <f>F22-F24-F25-F26</f>
+        <v/>
+      </c>
+      <c r="G27" s="25">
+        <f>G22-G24-G25-G26</f>
+        <v/>
+      </c>
+      <c r="H27" s="25">
+        <f>H22-H24-H25-H26</f>
+        <v/>
+      </c>
+      <c r="I27" s="25">
+        <f>I22-I24-I25-I26</f>
+        <v/>
+      </c>
+      <c r="J27" s="25">
+        <f>J22-J24-J25-J26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EBIT Margin</t>
+        </is>
+      </c>
+      <c r="B28" s="28">
+        <f>IF(B19&lt;&gt;0,B27/B19,0)</f>
+        <v/>
+      </c>
+      <c r="C28" s="28">
+        <f>IF(C19&lt;&gt;0,C27/C19,0)</f>
+        <v/>
+      </c>
+      <c r="D28" s="28">
+        <f>IF(D19&lt;&gt;0,D27/D19,0)</f>
+        <v/>
+      </c>
+      <c r="E28" s="28">
+        <f>IF(E19&lt;&gt;0,E27/E19,0)</f>
+        <v/>
+      </c>
+      <c r="F28" s="28">
+        <f>IF(F19&lt;&gt;0,F27/F19,0)</f>
+        <v/>
+      </c>
+      <c r="G28" s="28">
+        <f>IF(G19&lt;&gt;0,G27/G19,0)</f>
+        <v/>
+      </c>
+      <c r="H28" s="28">
+        <f>IF(H19&lt;&gt;0,H27/H19,0)</f>
+        <v/>
+      </c>
+      <c r="I28" s="28">
+        <f>IF(I19&lt;&gt;0,I27/I19,0)</f>
+        <v/>
+      </c>
+      <c r="J28" s="28">
+        <f>IF(J19&lt;&gt;0,J27/J19,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tax on EBIT</t>
+        </is>
+      </c>
+      <c r="B29" s="31">
+        <f>B27*B11</f>
+        <v/>
+      </c>
+      <c r="C29" s="31">
+        <f>C27*C11</f>
+        <v/>
+      </c>
+      <c r="D29" s="31">
+        <f>D27*D11</f>
+        <v/>
+      </c>
+      <c r="E29" s="31">
+        <f>E27*E11</f>
+        <v/>
+      </c>
+      <c r="F29" s="31">
+        <f>F27*F11</f>
+        <v/>
+      </c>
+      <c r="G29" s="31">
+        <f>G27*G11</f>
+        <v/>
+      </c>
+      <c r="H29" s="31">
+        <f>H27*H11</f>
+        <v/>
+      </c>
+      <c r="I29" s="31">
+        <f>I27*I11</f>
+        <v/>
+      </c>
+      <c r="J29" s="31">
+        <f>J27*J11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="24" t="inlineStr">
+        <is>
+          <t>NOPAT</t>
+        </is>
+      </c>
+      <c r="B30" s="25">
+        <f>'Adj ASM'!E36</f>
+        <v/>
+      </c>
+      <c r="C30" s="25">
+        <f>'Adj ASM'!F36</f>
+        <v/>
+      </c>
+      <c r="D30" s="25">
+        <f>'Adj ASM'!G36</f>
+        <v/>
+      </c>
+      <c r="E30" s="25">
+        <f>E27-E29</f>
+        <v/>
+      </c>
+      <c r="F30" s="25">
+        <f>F27-F29</f>
+        <v/>
+      </c>
+      <c r="G30" s="25">
+        <f>G27-G29</f>
+        <v/>
+      </c>
+      <c r="H30" s="25">
+        <f>H27-H29</f>
+        <v/>
+      </c>
+      <c r="I30" s="25">
+        <f>I27-I29</f>
+        <v/>
+      </c>
+      <c r="J30" s="25">
+        <f>J27-J29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NOPAT Margin</t>
+        </is>
+      </c>
+      <c r="B31" s="28">
+        <f>IF(B19&lt;&gt;0,B30/B19,0)</f>
+        <v/>
+      </c>
+      <c r="C31" s="28">
+        <f>IF(C19&lt;&gt;0,C30/C19,0)</f>
+        <v/>
+      </c>
+      <c r="D31" s="28">
+        <f>IF(D19&lt;&gt;0,D30/D19,0)</f>
+        <v/>
+      </c>
+      <c r="E31" s="28">
+        <f>IF(E19&lt;&gt;0,E30/E19,0)</f>
+        <v/>
+      </c>
+      <c r="F31" s="28">
+        <f>IF(F19&lt;&gt;0,F30/F19,0)</f>
+        <v/>
+      </c>
+      <c r="G31" s="28">
+        <f>IF(G19&lt;&gt;0,G30/G19,0)</f>
+        <v/>
+      </c>
+      <c r="H31" s="28">
+        <f>IF(H19&lt;&gt;0,H30/H19,0)</f>
+        <v/>
+      </c>
+      <c r="I31" s="28">
+        <f>IF(I19&lt;&gt;0,I30/I19,0)</f>
+        <v/>
+      </c>
+      <c r="J31" s="28">
+        <f>IF(J19&lt;&gt;0,J30/J19,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Investment Income</t>
+        </is>
+      </c>
+      <c r="B33" s="21">
+        <f>'Adj ASM'!E27</f>
+        <v/>
+      </c>
+      <c r="C33" s="21">
+        <f>'Adj ASM'!F27</f>
+        <v/>
+      </c>
+      <c r="D33" s="21">
+        <f>'Adj ASM'!G27</f>
+        <v/>
+      </c>
+      <c r="E33" s="31">
+        <f>D33</f>
+        <v/>
+      </c>
+      <c r="F33" s="31">
+        <f>D33</f>
+        <v/>
+      </c>
+      <c r="G33" s="31">
+        <f>D33</f>
+        <v/>
+      </c>
+      <c r="H33" s="31">
+        <f>D33</f>
+        <v/>
+      </c>
+      <c r="I33" s="31">
+        <f>D33</f>
+        <v/>
+      </c>
+      <c r="J33" s="31">
+        <f>D33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Interest Expense</t>
+        </is>
+      </c>
+      <c r="B34" s="21">
+        <f>'Adj ASM'!E29</f>
+        <v/>
+      </c>
+      <c r="C34" s="21">
+        <f>'Adj ASM'!F29</f>
+        <v/>
+      </c>
+      <c r="D34" s="21">
+        <f>'Adj ASM'!G29</f>
+        <v/>
+      </c>
+      <c r="E34" s="31">
+        <f>D34</f>
+        <v/>
+      </c>
+      <c r="F34" s="31">
+        <f>D34</f>
+        <v/>
+      </c>
+      <c r="G34" s="31">
+        <f>D34</f>
+        <v/>
+      </c>
+      <c r="H34" s="31">
+        <f>D34</f>
+        <v/>
+      </c>
+      <c r="I34" s="31">
+        <f>D34</f>
+        <v/>
+      </c>
+      <c r="J34" s="31">
+        <f>D34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="26" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="B35" s="43">
+        <f>'Adj ASM'!E33</f>
+        <v/>
+      </c>
+      <c r="C35" s="43">
+        <f>'Adj ASM'!F33</f>
+        <v/>
+      </c>
+      <c r="D35" s="43">
+        <f>'Adj ASM'!G33</f>
+        <v/>
+      </c>
+      <c r="E35" s="27">
+        <f>E30+E33+E34</f>
+        <v/>
+      </c>
+      <c r="F35" s="27">
+        <f>F30+F33+F34</f>
+        <v/>
+      </c>
+      <c r="G35" s="27">
+        <f>G30+G33+G34</f>
+        <v/>
+      </c>
+      <c r="H35" s="27">
+        <f>H30+H33+H34</f>
+        <v/>
+      </c>
+      <c r="I35" s="27">
+        <f>I30+I33+I34</f>
+        <v/>
+      </c>
+      <c r="J35" s="27">
+        <f>J30+J33+J34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>CONDENSED BALANCE SHEET</t>
+        </is>
+      </c>
+      <c r="B37" s="20" t="n"/>
+      <c r="C37" s="20" t="n"/>
+      <c r="D37" s="20" t="n"/>
+      <c r="E37" s="20" t="n"/>
+      <c r="F37" s="20" t="n"/>
+      <c r="G37" s="20" t="n"/>
+      <c r="H37" s="20" t="n"/>
+      <c r="I37" s="20" t="n"/>
+      <c r="J37" s="20" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Operating Working Capital</t>
+        </is>
+      </c>
+      <c r="B38" s="21">
+        <f>'Adj ASM'!E54</f>
+        <v/>
+      </c>
+      <c r="C38" s="21">
+        <f>'Adj ASM'!F54</f>
+        <v/>
+      </c>
+      <c r="D38" s="21">
+        <f>'Adj ASM'!G54</f>
+        <v/>
+      </c>
+      <c r="E38" s="31">
+        <f>E19*E12</f>
+        <v/>
+      </c>
+      <c r="F38" s="31">
+        <f>F19*F12</f>
+        <v/>
+      </c>
+      <c r="G38" s="31">
+        <f>G19*G12</f>
+        <v/>
+      </c>
+      <c r="H38" s="31">
+        <f>H19*H12</f>
+        <v/>
+      </c>
+      <c r="I38" s="31">
+        <f>I19*I12</f>
+        <v/>
+      </c>
+      <c r="J38" s="31">
+        <f>J19*J12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>+ Net Non-Current Operating Assets</t>
+        </is>
+      </c>
+      <c r="B39" s="21">
+        <f>'Adj ASM'!E65</f>
+        <v/>
+      </c>
+      <c r="C39" s="21">
+        <f>'Adj ASM'!F65</f>
+        <v/>
+      </c>
+      <c r="D39" s="21">
+        <f>'Adj ASM'!G65</f>
+        <v/>
+      </c>
+      <c r="E39" s="31">
+        <f>E19*E13</f>
+        <v/>
+      </c>
+      <c r="F39" s="31">
+        <f>F19*F13</f>
+        <v/>
+      </c>
+      <c r="G39" s="31">
+        <f>G19*G13</f>
+        <v/>
+      </c>
+      <c r="H39" s="31">
+        <f>H19*H13</f>
+        <v/>
+      </c>
+      <c r="I39" s="31">
+        <f>I19*I13</f>
+        <v/>
+      </c>
+      <c r="J39" s="31">
+        <f>J19*J13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="24">
+        <f> Net Operating Assets</f>
+        <v/>
+      </c>
+      <c r="B40" s="25">
+        <f>'Adj ASM'!E67</f>
+        <v/>
+      </c>
+      <c r="C40" s="25">
+        <f>'Adj ASM'!F67</f>
+        <v/>
+      </c>
+      <c r="D40" s="25">
+        <f>'Adj ASM'!G67</f>
+        <v/>
+      </c>
+      <c r="E40" s="25">
+        <f>E38+E39</f>
+        <v/>
+      </c>
+      <c r="F40" s="25">
+        <f>F38+F39</f>
+        <v/>
+      </c>
+      <c r="G40" s="25">
+        <f>G38+G39</f>
+        <v/>
+      </c>
+      <c r="H40" s="25">
+        <f>H38+H39</f>
+        <v/>
+      </c>
+      <c r="I40" s="25">
+        <f>I38+I39</f>
+        <v/>
+      </c>
+      <c r="J40" s="25">
+        <f>J38+J39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>+ Investment Assets</t>
+        </is>
+      </c>
+      <c r="B42" s="21">
+        <f>'Adj ASM'!E71</f>
+        <v/>
+      </c>
+      <c r="C42" s="21">
+        <f>'Adj ASM'!F71</f>
+        <v/>
+      </c>
+      <c r="D42" s="21">
+        <f>'Adj ASM'!G71</f>
+        <v/>
+      </c>
+      <c r="E42" s="31">
+        <f>E19*E14</f>
+        <v/>
+      </c>
+      <c r="F42" s="31">
+        <f>F19*F14</f>
+        <v/>
+      </c>
+      <c r="G42" s="31">
+        <f>G19*G14</f>
+        <v/>
+      </c>
+      <c r="H42" s="31">
+        <f>H19*H14</f>
+        <v/>
+      </c>
+      <c r="I42" s="31">
+        <f>I19*I14</f>
+        <v/>
+      </c>
+      <c r="J42" s="31">
+        <f>J19*J14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="26">
+        <f> Business Assets</f>
+        <v/>
+      </c>
+      <c r="B43" s="43">
+        <f>'Adj ASM'!E73</f>
+        <v/>
+      </c>
+      <c r="C43" s="43">
+        <f>'Adj ASM'!F73</f>
+        <v/>
+      </c>
+      <c r="D43" s="43">
+        <f>'Adj ASM'!G73</f>
+        <v/>
+      </c>
+      <c r="E43" s="27">
+        <f>E40+E42</f>
+        <v/>
+      </c>
+      <c r="F43" s="27">
+        <f>F40+F42</f>
+        <v/>
+      </c>
+      <c r="G43" s="27">
+        <f>G40+G42</f>
+        <v/>
+      </c>
+      <c r="H43" s="27">
+        <f>H40+H42</f>
+        <v/>
+      </c>
+      <c r="I43" s="27">
+        <f>I40+I42</f>
+        <v/>
+      </c>
+      <c r="J43" s="27">
+        <f>J40+J42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="22">
+        <f> Invested Capital</f>
+        <v/>
+      </c>
+      <c r="B45" s="21">
+        <f>'Adj ASM'!E82</f>
+        <v/>
+      </c>
+      <c r="C45" s="21">
+        <f>'Adj ASM'!F82</f>
+        <v/>
+      </c>
+      <c r="D45" s="21">
+        <f>'Adj ASM'!G82</f>
+        <v/>
+      </c>
+      <c r="E45" s="23">
+        <f>E43</f>
+        <v/>
+      </c>
+      <c r="F45" s="23">
+        <f>F43</f>
+        <v/>
+      </c>
+      <c r="G45" s="23">
+        <f>G43</f>
+        <v/>
+      </c>
+      <c r="H45" s="23">
+        <f>H43</f>
+        <v/>
+      </c>
+      <c r="I45" s="23">
+        <f>I43</f>
+        <v/>
+      </c>
+      <c r="J45" s="23">
+        <f>J43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Debt</t>
+        </is>
+      </c>
+      <c r="B46" s="21">
+        <f>'Adj ASM'!E78</f>
+        <v/>
+      </c>
+      <c r="C46" s="21">
+        <f>'Adj ASM'!F78</f>
+        <v/>
+      </c>
+      <c r="D46" s="21">
+        <f>'Adj ASM'!G78</f>
+        <v/>
+      </c>
+      <c r="E46" s="31">
+        <f>E45*E15</f>
+        <v/>
+      </c>
+      <c r="F46" s="31">
+        <f>F45*F15</f>
+        <v/>
+      </c>
+      <c r="G46" s="31">
+        <f>G45*G15</f>
+        <v/>
+      </c>
+      <c r="H46" s="31">
+        <f>H45*H15</f>
+        <v/>
+      </c>
+      <c r="I46" s="31">
+        <f>I45*I15</f>
+        <v/>
+      </c>
+      <c r="J46" s="31">
+        <f>J45*J15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Group Equity</t>
+        </is>
+      </c>
+      <c r="B47" s="21">
+        <f>'Adj ASM'!E81</f>
+        <v/>
+      </c>
+      <c r="C47" s="21">
+        <f>'Adj ASM'!F81</f>
+        <v/>
+      </c>
+      <c r="D47" s="21">
+        <f>'Adj ASM'!G81</f>
+        <v/>
+      </c>
+      <c r="E47" s="31">
+        <f>E45-E46</f>
+        <v/>
+      </c>
+      <c r="F47" s="31">
+        <f>F45-F46</f>
+        <v/>
+      </c>
+      <c r="G47" s="31">
+        <f>G45-G46</f>
+        <v/>
+      </c>
+      <c r="H47" s="31">
+        <f>H45-H46</f>
+        <v/>
+      </c>
+      <c r="I47" s="31">
+        <f>I45-I46</f>
+        <v/>
+      </c>
+      <c r="J47" s="31">
+        <f>J45-J46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="22" t="inlineStr">
+        <is>
+          <t>BS Check (should = 0)</t>
+        </is>
+      </c>
+      <c r="B48" s="23">
+        <f>B43-B45</f>
+        <v/>
+      </c>
+      <c r="C48" s="23">
+        <f>C43-C45</f>
+        <v/>
+      </c>
+      <c r="D48" s="23">
+        <f>D43-D45</f>
+        <v/>
+      </c>
+      <c r="E48" s="23">
+        <f>E43-E45</f>
+        <v/>
+      </c>
+      <c r="F48" s="23">
+        <f>F43-F45</f>
+        <v/>
+      </c>
+      <c r="G48" s="23">
+        <f>G43-G45</f>
+        <v/>
+      </c>
+      <c r="H48" s="23">
+        <f>H43-H45</f>
+        <v/>
+      </c>
+      <c r="I48" s="23">
+        <f>I43-I45</f>
+        <v/>
+      </c>
+      <c r="J48" s="23">
+        <f>J43-J45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="19" t="inlineStr">
+        <is>
+          <t>FREE CASH FLOW</t>
+        </is>
+      </c>
+      <c r="B50" s="20" t="n"/>
+      <c r="C50" s="20" t="n"/>
+      <c r="D50" s="20" t="n"/>
+      <c r="E50" s="20" t="n"/>
+      <c r="F50" s="20" t="n"/>
+      <c r="G50" s="20" t="n"/>
+      <c r="H50" s="20" t="n"/>
+      <c r="I50" s="20" t="n"/>
+      <c r="J50" s="20" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>NOPAT</t>
+        </is>
+      </c>
+      <c r="B51" s="31">
+        <f>B30</f>
+        <v/>
+      </c>
+      <c r="C51" s="31">
+        <f>C30</f>
+        <v/>
+      </c>
+      <c r="D51" s="31">
+        <f>D30</f>
+        <v/>
+      </c>
+      <c r="E51" s="31">
+        <f>E30</f>
+        <v/>
+      </c>
+      <c r="F51" s="31">
+        <f>F30</f>
+        <v/>
+      </c>
+      <c r="G51" s="31">
+        <f>G30</f>
+        <v/>
+      </c>
+      <c r="H51" s="31">
+        <f>H30</f>
+        <v/>
+      </c>
+      <c r="I51" s="31">
+        <f>I30</f>
+        <v/>
+      </c>
+      <c r="J51" s="31">
+        <f>J30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>+ D&amp;A</t>
+        </is>
+      </c>
+      <c r="B52" s="31">
+        <f>B26</f>
+        <v/>
+      </c>
+      <c r="C52" s="31">
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D52" s="31">
+        <f>D26</f>
+        <v/>
+      </c>
+      <c r="E52" s="31">
+        <f>E26</f>
+        <v/>
+      </c>
+      <c r="F52" s="31">
+        <f>F26</f>
+        <v/>
+      </c>
+      <c r="G52" s="31">
+        <f>G26</f>
+        <v/>
+      </c>
+      <c r="H52" s="31">
+        <f>H26</f>
+        <v/>
+      </c>
+      <c r="I52" s="31">
+        <f>I26</f>
+        <v/>
+      </c>
+      <c r="J52" s="31">
+        <f>J26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="11" t="inlineStr">
+        <is>
+          <t>- Change in OWC</t>
+        </is>
+      </c>
+      <c r="B53" s="31">
+        <f>B38-'Adj ASM'!D54</f>
+        <v/>
+      </c>
+      <c r="C53" s="31">
+        <f>C38-B38</f>
+        <v/>
+      </c>
+      <c r="D53" s="31">
+        <f>D38-C38</f>
+        <v/>
+      </c>
+      <c r="E53" s="31">
+        <f>E38-D38</f>
+        <v/>
+      </c>
+      <c r="F53" s="31">
+        <f>F38-E38</f>
+        <v/>
+      </c>
+      <c r="G53" s="31">
+        <f>G38-F38</f>
+        <v/>
+      </c>
+      <c r="H53" s="31">
+        <f>H38-G38</f>
+        <v/>
+      </c>
+      <c r="I53" s="31">
+        <f>I38-H38</f>
+        <v/>
+      </c>
+      <c r="J53" s="31">
+        <f>J38-I38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>- Change in Net NCA</t>
+        </is>
+      </c>
+      <c r="B54" s="31">
+        <f>B39-'Adj ASM'!D65</f>
+        <v/>
+      </c>
+      <c r="C54" s="31">
+        <f>C39-B39</f>
+        <v/>
+      </c>
+      <c r="D54" s="31">
+        <f>D39-C39</f>
+        <v/>
+      </c>
+      <c r="E54" s="31">
+        <f>E39-D39</f>
+        <v/>
+      </c>
+      <c r="F54" s="31">
+        <f>F39-E39</f>
+        <v/>
+      </c>
+      <c r="G54" s="31">
+        <f>G39-F39</f>
+        <v/>
+      </c>
+      <c r="H54" s="31">
+        <f>H39-G39</f>
+        <v/>
+      </c>
+      <c r="I54" s="31">
+        <f>I39-H39</f>
+        <v/>
+      </c>
+      <c r="J54" s="31">
+        <f>J39-I39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="24">
+        <f> Oper CF after investment</f>
+        <v/>
+      </c>
+      <c r="B55" s="25">
+        <f>B51+B52-B53-B54</f>
+        <v/>
+      </c>
+      <c r="C55" s="25">
+        <f>C51+C52-C53-C54</f>
+        <v/>
+      </c>
+      <c r="D55" s="25">
+        <f>D51+D52-D53-D54</f>
+        <v/>
+      </c>
+      <c r="E55" s="25">
+        <f>E51+E52-E53-E54</f>
+        <v/>
+      </c>
+      <c r="F55" s="25">
+        <f>F51+F52-F53-F54</f>
+        <v/>
+      </c>
+      <c r="G55" s="25">
+        <f>G51+G52-G53-G54</f>
+        <v/>
+      </c>
+      <c r="H55" s="25">
+        <f>H51+H52-H53-H54</f>
+        <v/>
+      </c>
+      <c r="I55" s="25">
+        <f>I51+I52-I53-I54</f>
+        <v/>
+      </c>
+      <c r="J55" s="25">
+        <f>J51+J52-J53-J54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>+ Net Inv Profit after tax</t>
+        </is>
+      </c>
+      <c r="B57" s="31">
+        <f>B33*(1-B11)</f>
+        <v/>
+      </c>
+      <c r="C57" s="31">
+        <f>C33*(1-C11)</f>
+        <v/>
+      </c>
+      <c r="D57" s="31">
+        <f>D33*(1-D11)</f>
+        <v/>
+      </c>
+      <c r="E57" s="31">
+        <f>E33*(1-E11)</f>
+        <v/>
+      </c>
+      <c r="F57" s="31">
+        <f>F33*(1-F11)</f>
+        <v/>
+      </c>
+      <c r="G57" s="31">
+        <f>G33*(1-G11)</f>
+        <v/>
+      </c>
+      <c r="H57" s="31">
+        <f>H33*(1-H11)</f>
+        <v/>
+      </c>
+      <c r="I57" s="31">
+        <f>I33*(1-I11)</f>
+        <v/>
+      </c>
+      <c r="J57" s="31">
+        <f>J33*(1-J11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>- Change in Inv Assets</t>
+        </is>
+      </c>
+      <c r="B58" s="31">
+        <f>B42-'Adj ASM'!D71</f>
+        <v/>
+      </c>
+      <c r="C58" s="31">
+        <f>C42-B42</f>
+        <v/>
+      </c>
+      <c r="D58" s="31">
+        <f>D42-C42</f>
+        <v/>
+      </c>
+      <c r="E58" s="31">
+        <f>E42-D42</f>
+        <v/>
+      </c>
+      <c r="F58" s="31">
+        <f>F42-E42</f>
+        <v/>
+      </c>
+      <c r="G58" s="31">
+        <f>G42-F42</f>
+        <v/>
+      </c>
+      <c r="H58" s="31">
+        <f>H42-G42</f>
+        <v/>
+      </c>
+      <c r="I58" s="31">
+        <f>I42-H42</f>
+        <v/>
+      </c>
+      <c r="J58" s="31">
+        <f>J42-I42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="24">
+        <f> FCF to Debt &amp; Equity</f>
+        <v/>
+      </c>
+      <c r="B59" s="25">
+        <f>B55+B57-B58</f>
+        <v/>
+      </c>
+      <c r="C59" s="25">
+        <f>C55+C57-C58</f>
+        <v/>
+      </c>
+      <c r="D59" s="25">
+        <f>D55+D57-D58</f>
+        <v/>
+      </c>
+      <c r="E59" s="25">
+        <f>E55+E57-E58</f>
+        <v/>
+      </c>
+      <c r="F59" s="25">
+        <f>F55+F57-F58</f>
+        <v/>
+      </c>
+      <c r="G59" s="25">
+        <f>G55+G57-G58</f>
+        <v/>
+      </c>
+      <c r="H59" s="25">
+        <f>H55+H57-H58</f>
+        <v/>
+      </c>
+      <c r="I59" s="25">
+        <f>I55+I57-I58</f>
+        <v/>
+      </c>
+      <c r="J59" s="25">
+        <f>J55+J57-J58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>- Interest after tax</t>
+        </is>
+      </c>
+      <c r="B60" s="31">
+        <f>B34*(1-B11)</f>
+        <v/>
+      </c>
+      <c r="C60" s="31">
+        <f>C34*(1-C11)</f>
+        <v/>
+      </c>
+      <c r="D60" s="31">
+        <f>D34*(1-D11)</f>
+        <v/>
+      </c>
+      <c r="E60" s="31">
+        <f>E34*(1-E11)</f>
+        <v/>
+      </c>
+      <c r="F60" s="31">
+        <f>F34*(1-F11)</f>
+        <v/>
+      </c>
+      <c r="G60" s="31">
+        <f>G34*(1-G11)</f>
+        <v/>
+      </c>
+      <c r="H60" s="31">
+        <f>H34*(1-H11)</f>
+        <v/>
+      </c>
+      <c r="I60" s="31">
+        <f>I34*(1-I11)</f>
+        <v/>
+      </c>
+      <c r="J60" s="31">
+        <f>J34*(1-J11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>+ Change in Debt</t>
+        </is>
+      </c>
+      <c r="B61" s="31">
+        <f>B46-'Adj ASM'!D78</f>
+        <v/>
+      </c>
+      <c r="C61" s="31">
+        <f>C46-B46</f>
+        <v/>
+      </c>
+      <c r="D61" s="31">
+        <f>D46-C46</f>
+        <v/>
+      </c>
+      <c r="E61" s="31">
+        <f>E46-D46</f>
+        <v/>
+      </c>
+      <c r="F61" s="31">
+        <f>F46-E46</f>
+        <v/>
+      </c>
+      <c r="G61" s="31">
+        <f>G46-F46</f>
+        <v/>
+      </c>
+      <c r="H61" s="31">
+        <f>H46-G46</f>
+        <v/>
+      </c>
+      <c r="I61" s="31">
+        <f>I46-H46</f>
+        <v/>
+      </c>
+      <c r="J61" s="31">
+        <f>J46-I46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="26">
+        <f> FCF to Equity</f>
+        <v/>
+      </c>
+      <c r="B62" s="27">
+        <f>B59-B60+B61</f>
+        <v/>
+      </c>
+      <c r="C62" s="27">
+        <f>C59-C60+C61</f>
+        <v/>
+      </c>
+      <c r="D62" s="27">
+        <f>D59-D60+D61</f>
+        <v/>
+      </c>
+      <c r="E62" s="27">
+        <f>E59-E60+E61</f>
+        <v/>
+      </c>
+      <c r="F62" s="27">
+        <f>F59-F60+F61</f>
+        <v/>
+      </c>
+      <c r="G62" s="27">
+        <f>G59-G60+G61</f>
+        <v/>
+      </c>
+      <c r="H62" s="27">
+        <f>H59-H60+H61</f>
+        <v/>
+      </c>
+      <c r="I62" s="27">
+        <f>I59-I60+I61</f>
+        <v/>
+      </c>
+      <c r="J62" s="27">
+        <f>J59-J60+J61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="19" t="inlineStr">
+        <is>
+          <t>KEY METRICS</t>
+        </is>
+      </c>
+      <c r="B64" s="20" t="n"/>
+      <c r="C64" s="20" t="n"/>
+      <c r="D64" s="20" t="n"/>
+      <c r="E64" s="20" t="n"/>
+      <c r="F64" s="20" t="n"/>
+      <c r="G64" s="20" t="n"/>
+      <c r="H64" s="20" t="n"/>
+      <c r="I64" s="20" t="n"/>
+      <c r="J64" s="20" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>NOPAT Margin</t>
+        </is>
+      </c>
+      <c r="B65" s="28">
+        <f>IF(B19&lt;&gt;0,B30/B19,0)</f>
+        <v/>
+      </c>
+      <c r="C65" s="28">
+        <f>IF(C19&lt;&gt;0,C30/C19,0)</f>
+        <v/>
+      </c>
+      <c r="D65" s="28">
+        <f>IF(D19&lt;&gt;0,D30/D19,0)</f>
+        <v/>
+      </c>
+      <c r="E65" s="28">
+        <f>IF(E19&lt;&gt;0,E30/E19,0)</f>
+        <v/>
+      </c>
+      <c r="F65" s="28">
+        <f>IF(F19&lt;&gt;0,F30/F19,0)</f>
+        <v/>
+      </c>
+      <c r="G65" s="28">
+        <f>IF(G19&lt;&gt;0,G30/G19,0)</f>
+        <v/>
+      </c>
+      <c r="H65" s="28">
+        <f>IF(H19&lt;&gt;0,H30/H19,0)</f>
+        <v/>
+      </c>
+      <c r="I65" s="28">
+        <f>IF(I19&lt;&gt;0,I30/I19,0)</f>
+        <v/>
+      </c>
+      <c r="J65" s="28">
+        <f>IF(J19&lt;&gt;0,J30/J19,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>ROE</t>
+        </is>
+      </c>
+      <c r="B66" s="28">
+        <f>IF((B47+'Adj ASM'!D81)/2&lt;&gt;0,B35/((B47+'Adj ASM'!D81)/2),0)</f>
+        <v/>
+      </c>
+      <c r="C66" s="28">
+        <f>IF((C47+B47)/2&lt;&gt;0,C35/((C47+B47)/2),0)</f>
+        <v/>
+      </c>
+      <c r="D66" s="28">
+        <f>IF((D47+C47)/2&lt;&gt;0,D35/((D47+C47)/2),0)</f>
+        <v/>
+      </c>
+      <c r="E66" s="28">
+        <f>IF((E47+D47)/2&lt;&gt;0,E35/((E47+D47)/2),0)</f>
+        <v/>
+      </c>
+      <c r="F66" s="28">
+        <f>IF((F47+E47)/2&lt;&gt;0,F35/((F47+E47)/2),0)</f>
+        <v/>
+      </c>
+      <c r="G66" s="28">
+        <f>IF((G47+F47)/2&lt;&gt;0,G35/((G47+F47)/2),0)</f>
+        <v/>
+      </c>
+      <c r="H66" s="28">
+        <f>IF((H47+G47)/2&lt;&gt;0,H35/((H47+G47)/2),0)</f>
+        <v/>
+      </c>
+      <c r="I66" s="28">
+        <f>IF((I47+H47)/2&lt;&gt;0,I35/((I47+H47)/2),0)</f>
+        <v/>
+      </c>
+      <c r="J66" s="28">
+        <f>IF((J47+I47)/2&lt;&gt;0,J35/((J47+I47)/2),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>RNOA</t>
+        </is>
+      </c>
+      <c r="B67" s="28">
+        <f>IF((B40+'Adj ASM'!D67)/2&lt;&gt;0,B30/((B40+'Adj ASM'!D67)/2),0)</f>
+        <v/>
+      </c>
+      <c r="C67" s="28">
+        <f>IF((C40+B40)/2&lt;&gt;0,C30/((C40+B40)/2),0)</f>
+        <v/>
+      </c>
+      <c r="D67" s="28">
+        <f>IF((D40+C40)/2&lt;&gt;0,D30/((D40+C40)/2),0)</f>
+        <v/>
+      </c>
+      <c r="E67" s="28">
+        <f>IF((E40+D40)/2&lt;&gt;0,E30/((E40+D40)/2),0)</f>
+        <v/>
+      </c>
+      <c r="F67" s="28">
+        <f>IF((F40+E40)/2&lt;&gt;0,F30/((F40+E40)/2),0)</f>
+        <v/>
+      </c>
+      <c r="G67" s="28">
+        <f>IF((G40+F40)/2&lt;&gt;0,G30/((G40+F40)/2),0)</f>
+        <v/>
+      </c>
+      <c r="H67" s="28">
+        <f>IF((H40+G40)/2&lt;&gt;0,H30/((H40+G40)/2),0)</f>
+        <v/>
+      </c>
+      <c r="I67" s="28">
+        <f>IF((I40+H40)/2&lt;&gt;0,I30/((I40+H40)/2),0)</f>
+        <v/>
+      </c>
+      <c r="J67" s="28">
+        <f>IF((J40+I40)/2&lt;&gt;0,J30/((J40+I40)/2),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>FCF to Equity</t>
+        </is>
+      </c>
+      <c r="B68" s="31">
+        <f>B62</f>
+        <v/>
+      </c>
+      <c r="C68" s="31">
+        <f>C62</f>
+        <v/>
+      </c>
+      <c r="D68" s="31">
+        <f>D62</f>
+        <v/>
+      </c>
+      <c r="E68" s="31">
+        <f>E62</f>
+        <v/>
+      </c>
+      <c r="F68" s="31">
+        <f>F62</f>
+        <v/>
+      </c>
+      <c r="G68" s="31">
+        <f>G62</f>
+        <v/>
+      </c>
+      <c r="H68" s="31">
+        <f>H62</f>
+        <v/>
+      </c>
+      <c r="I68" s="31">
+        <f>I62</f>
+        <v/>
+      </c>
+      <c r="J68" s="31">
+        <f>J62</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: add Valuation tab with WACC, DCF, PVAOI, comps, sensitivity, football field
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/ASM_Valuation_Model.xlsx
+++ b/output/ASM_Valuation_Model.xlsx
@@ -29,6 +29,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratios LRCX" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratio Comparison" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -37,12 +38,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0.00;(#,##0.00);&quot;-&quot;"/>
     <numFmt numFmtId="168" formatCode="0.00;(0.00);&quot;-&quot;"/>
+    <numFmt numFmtId="169" formatCode="0.0000"/>
+    <numFmt numFmtId="170" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -179,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -230,6 +233,28 @@
     <xf numFmtId="168" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="14" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="11" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="11" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="11" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="13" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -26580,6 +26605,2558 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J164"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>ASM International NV - Valuation Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>(EUR 000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>COST OF CAPITAL</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="n"/>
+      <c r="C3" s="20" t="n"/>
+      <c r="D3" s="20" t="n"/>
+      <c r="E3" s="20" t="n"/>
+      <c r="F3" s="20" t="n"/>
+      <c r="G3" s="20" t="n"/>
+      <c r="H3" s="20" t="n"/>
+      <c r="I3" s="20" t="n"/>
+      <c r="J3" s="20" t="n"/>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Risk-free Rate</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>0.025</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Equity Beta</t>
+        </is>
+      </c>
+      <c r="B6" s="44" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Equity Risk Premium</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>Cost of Equity (Re)</t>
+        </is>
+      </c>
+      <c r="B8" s="28">
+        <f>B5+B6*B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Cost of Debt (pre-tax)</t>
+        </is>
+      </c>
+      <c r="B10" s="28">
+        <f>IF('Adj ASM'!G78&lt;&gt;0,ABS('Adj ASM'!G29)/'Adj ASM'!G78,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Tax Rate</t>
+        </is>
+      </c>
+      <c r="B11" s="18">
+        <f>'Forecast'!G11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Cost of Debt (after-tax)</t>
+        </is>
+      </c>
+      <c r="B12" s="28">
+        <f>B10*(1-B11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Market Cap (EUR 000)</t>
+        </is>
+      </c>
+      <c r="B14" s="45" t="n">
+        <v>25000000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Net Debt</t>
+        </is>
+      </c>
+      <c r="B15" s="21">
+        <f>'Adj ASM'!G80</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>E/V</t>
+        </is>
+      </c>
+      <c r="B16" s="28">
+        <f>IF((B14+B15)&lt;&gt;0,B14/(B14+B15),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>D/V</t>
+        </is>
+      </c>
+      <c r="B17" s="28">
+        <f>1-B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>WACC</t>
+        </is>
+      </c>
+      <c r="B18" s="46">
+        <f>B16*B8+B17*B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Shares Outstanding (diluted)</t>
+        </is>
+      </c>
+      <c r="B20" s="21">
+        <f>'Adj ASM'!G38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Current Share Price (EUR)</t>
+        </is>
+      </c>
+      <c r="B21" s="47" t="n">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Terminal Growth Rate</t>
+        </is>
+      </c>
+      <c r="B22" s="18">
+        <f>'Forecast'!J16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>DCF - FREE CASH FLOW TO DEBT &amp; EQUITY</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n"/>
+      <c r="C25" s="20" t="n"/>
+      <c r="D25" s="20" t="n"/>
+      <c r="E25" s="20" t="n"/>
+      <c r="F25" s="20" t="n"/>
+      <c r="G25" s="20" t="n"/>
+      <c r="H25" s="20" t="n"/>
+      <c r="I25" s="20" t="n"/>
+      <c r="J25" s="20" t="n"/>
+    </row>
+    <row r="27">
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>2025E</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="G27" s="16" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>2028E</t>
+        </is>
+      </c>
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <t>2029E</t>
+        </is>
+      </c>
+      <c r="J27" s="16" t="inlineStr">
+        <is>
+          <t>2030E</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>FCF to Debt &amp; Equity</t>
+        </is>
+      </c>
+      <c r="E28" s="21">
+        <f>'Forecast'!E59</f>
+        <v/>
+      </c>
+      <c r="F28" s="21">
+        <f>'Forecast'!F59</f>
+        <v/>
+      </c>
+      <c r="G28" s="21">
+        <f>'Forecast'!G59</f>
+        <v/>
+      </c>
+      <c r="H28" s="21">
+        <f>'Forecast'!H59</f>
+        <v/>
+      </c>
+      <c r="I28" s="21">
+        <f>'Forecast'!I59</f>
+        <v/>
+      </c>
+      <c r="J28" s="21">
+        <f>'Forecast'!J59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Terminal Value</t>
+        </is>
+      </c>
+      <c r="J29" s="31">
+        <f>J28*(1+$B$22)/($B$18-$B$22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Total Cash Flow</t>
+        </is>
+      </c>
+      <c r="E30" s="31">
+        <f>E28</f>
+        <v/>
+      </c>
+      <c r="F30" s="31">
+        <f>F28</f>
+        <v/>
+      </c>
+      <c r="G30" s="31">
+        <f>G28</f>
+        <v/>
+      </c>
+      <c r="H30" s="31">
+        <f>H28</f>
+        <v/>
+      </c>
+      <c r="I30" s="31">
+        <f>I28</f>
+        <v/>
+      </c>
+      <c r="J30" s="31">
+        <f>J28+J29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Discount Factor</t>
+        </is>
+      </c>
+      <c r="E31" s="48">
+        <f>1/(1+$B$18)^1</f>
+        <v/>
+      </c>
+      <c r="F31" s="48">
+        <f>1/(1+$B$18)^2</f>
+        <v/>
+      </c>
+      <c r="G31" s="48">
+        <f>1/(1+$B$18)^3</f>
+        <v/>
+      </c>
+      <c r="H31" s="48">
+        <f>1/(1+$B$18)^4</f>
+        <v/>
+      </c>
+      <c r="I31" s="48">
+        <f>1/(1+$B$18)^5</f>
+        <v/>
+      </c>
+      <c r="J31" s="48">
+        <f>1/(1+$B$18)^6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>PV of Cash Flow</t>
+        </is>
+      </c>
+      <c r="E32" s="31">
+        <f>E30*E31</f>
+        <v/>
+      </c>
+      <c r="F32" s="31">
+        <f>F30*F31</f>
+        <v/>
+      </c>
+      <c r="G32" s="31">
+        <f>G30*G31</f>
+        <v/>
+      </c>
+      <c r="H32" s="31">
+        <f>H30*H31</f>
+        <v/>
+      </c>
+      <c r="I32" s="31">
+        <f>I30*I31</f>
+        <v/>
+      </c>
+      <c r="J32" s="31">
+        <f>J30*J31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="22" t="inlineStr">
+        <is>
+          <t>Sum of PV of Cash Flows</t>
+        </is>
+      </c>
+      <c r="B34" s="23">
+        <f>SUM(E32:J32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>Enterprise Value</t>
+        </is>
+      </c>
+      <c r="B35" s="31">
+        <f>B34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>- Net Debt</t>
+        </is>
+      </c>
+      <c r="B36" s="31">
+        <f>B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="22">
+        <f> Equity Value</f>
+        <v/>
+      </c>
+      <c r="B37" s="23">
+        <f>B35-B36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>/ Shares Outstanding</t>
+        </is>
+      </c>
+      <c r="B38" s="31">
+        <f>B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="26" t="inlineStr">
+        <is>
+          <t>Implied Price (DCF FCFF)</t>
+        </is>
+      </c>
+      <c r="B39" s="49">
+        <f>IF(B38&lt;&gt;0,B37/B38*1000,0)</f>
+        <v/>
+      </c>
+      <c r="C39" s="50" t="n"/>
+      <c r="D39" s="50" t="n"/>
+      <c r="E39" s="50" t="n"/>
+      <c r="F39" s="50" t="n"/>
+      <c r="G39" s="50" t="n"/>
+      <c r="H39" s="50" t="n"/>
+      <c r="I39" s="50" t="n"/>
+      <c r="J39" s="50" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>DCF - FREE CASH FLOW TO EQUITY</t>
+        </is>
+      </c>
+      <c r="B42" s="20" t="n"/>
+      <c r="C42" s="20" t="n"/>
+      <c r="D42" s="20" t="n"/>
+      <c r="E42" s="20" t="n"/>
+      <c r="F42" s="20" t="n"/>
+      <c r="G42" s="20" t="n"/>
+      <c r="H42" s="20" t="n"/>
+      <c r="I42" s="20" t="n"/>
+      <c r="J42" s="20" t="n"/>
+    </row>
+    <row r="44">
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t>2025E</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="G44" s="16" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+      <c r="H44" s="16" t="inlineStr">
+        <is>
+          <t>2028E</t>
+        </is>
+      </c>
+      <c r="I44" s="16" t="inlineStr">
+        <is>
+          <t>2029E</t>
+        </is>
+      </c>
+      <c r="J44" s="16" t="inlineStr">
+        <is>
+          <t>2030E</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>FCF to Equity</t>
+        </is>
+      </c>
+      <c r="E45" s="21">
+        <f>'Forecast'!E62</f>
+        <v/>
+      </c>
+      <c r="F45" s="21">
+        <f>'Forecast'!F62</f>
+        <v/>
+      </c>
+      <c r="G45" s="21">
+        <f>'Forecast'!G62</f>
+        <v/>
+      </c>
+      <c r="H45" s="21">
+        <f>'Forecast'!H62</f>
+        <v/>
+      </c>
+      <c r="I45" s="21">
+        <f>'Forecast'!I62</f>
+        <v/>
+      </c>
+      <c r="J45" s="21">
+        <f>'Forecast'!J62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>Terminal Value</t>
+        </is>
+      </c>
+      <c r="J46" s="31">
+        <f>J45*(1+$B$22)/($B$8-$B$22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>Total Cash Flow</t>
+        </is>
+      </c>
+      <c r="E47" s="31">
+        <f>E45</f>
+        <v/>
+      </c>
+      <c r="F47" s="31">
+        <f>F45</f>
+        <v/>
+      </c>
+      <c r="G47" s="31">
+        <f>G45</f>
+        <v/>
+      </c>
+      <c r="H47" s="31">
+        <f>H45</f>
+        <v/>
+      </c>
+      <c r="I47" s="31">
+        <f>I45</f>
+        <v/>
+      </c>
+      <c r="J47" s="31">
+        <f>J45+J46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>Discount Factor</t>
+        </is>
+      </c>
+      <c r="E48" s="48">
+        <f>1/(1+$B$8)^1</f>
+        <v/>
+      </c>
+      <c r="F48" s="48">
+        <f>1/(1+$B$8)^2</f>
+        <v/>
+      </c>
+      <c r="G48" s="48">
+        <f>1/(1+$B$8)^3</f>
+        <v/>
+      </c>
+      <c r="H48" s="48">
+        <f>1/(1+$B$8)^4</f>
+        <v/>
+      </c>
+      <c r="I48" s="48">
+        <f>1/(1+$B$8)^5</f>
+        <v/>
+      </c>
+      <c r="J48" s="48">
+        <f>1/(1+$B$8)^6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>PV of Cash Flow</t>
+        </is>
+      </c>
+      <c r="E49" s="31">
+        <f>E47*E48</f>
+        <v/>
+      </c>
+      <c r="F49" s="31">
+        <f>F47*F48</f>
+        <v/>
+      </c>
+      <c r="G49" s="31">
+        <f>G47*G48</f>
+        <v/>
+      </c>
+      <c r="H49" s="31">
+        <f>H47*H48</f>
+        <v/>
+      </c>
+      <c r="I49" s="31">
+        <f>I47*I48</f>
+        <v/>
+      </c>
+      <c r="J49" s="31">
+        <f>J47*J48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="22" t="inlineStr">
+        <is>
+          <t>Equity Value (Sum of PV)</t>
+        </is>
+      </c>
+      <c r="B51" s="23">
+        <f>SUM(E49:J49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>/ Shares Outstanding</t>
+        </is>
+      </c>
+      <c r="B52" s="31">
+        <f>B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="26" t="inlineStr">
+        <is>
+          <t>Implied Price (DCF FCFE)</t>
+        </is>
+      </c>
+      <c r="B53" s="49">
+        <f>IF(B52&lt;&gt;0,B51/B52*1000,0)</f>
+        <v/>
+      </c>
+      <c r="C53" s="50" t="n"/>
+      <c r="D53" s="50" t="n"/>
+      <c r="E53" s="50" t="n"/>
+      <c r="F53" s="50" t="n"/>
+      <c r="G53" s="50" t="n"/>
+      <c r="H53" s="50" t="n"/>
+      <c r="I53" s="50" t="n"/>
+      <c r="J53" s="50" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="19" t="inlineStr">
+        <is>
+          <t>PV OF ABNORMAL OPERATING INCOME (PVAOI)</t>
+        </is>
+      </c>
+      <c r="B56" s="20" t="n"/>
+      <c r="C56" s="20" t="n"/>
+      <c r="D56" s="20" t="n"/>
+      <c r="E56" s="20" t="n"/>
+      <c r="F56" s="20" t="n"/>
+      <c r="G56" s="20" t="n"/>
+      <c r="H56" s="20" t="n"/>
+      <c r="I56" s="20" t="n"/>
+      <c r="J56" s="20" t="n"/>
+    </row>
+    <row r="58">
+      <c r="E58" s="16" t="inlineStr">
+        <is>
+          <t>2025E</t>
+        </is>
+      </c>
+      <c r="F58" s="16" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="G58" s="16" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+      <c r="H58" s="16" t="inlineStr">
+        <is>
+          <t>2028E</t>
+        </is>
+      </c>
+      <c r="I58" s="16" t="inlineStr">
+        <is>
+          <t>2029E</t>
+        </is>
+      </c>
+      <c r="J58" s="16" t="inlineStr">
+        <is>
+          <t>2030E</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>NOPAT</t>
+        </is>
+      </c>
+      <c r="E59" s="21">
+        <f>'Forecast'!E30</f>
+        <v/>
+      </c>
+      <c r="F59" s="21">
+        <f>'Forecast'!F30</f>
+        <v/>
+      </c>
+      <c r="G59" s="21">
+        <f>'Forecast'!G30</f>
+        <v/>
+      </c>
+      <c r="H59" s="21">
+        <f>'Forecast'!H30</f>
+        <v/>
+      </c>
+      <c r="I59" s="21">
+        <f>'Forecast'!I30</f>
+        <v/>
+      </c>
+      <c r="J59" s="21">
+        <f>'Forecast'!J30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>Beg BV of NOA</t>
+        </is>
+      </c>
+      <c r="E60" s="21">
+        <f>'Forecast'!D40</f>
+        <v/>
+      </c>
+      <c r="F60" s="21">
+        <f>'Forecast'!E40</f>
+        <v/>
+      </c>
+      <c r="G60" s="21">
+        <f>'Forecast'!F40</f>
+        <v/>
+      </c>
+      <c r="H60" s="21">
+        <f>'Forecast'!G40</f>
+        <v/>
+      </c>
+      <c r="I60" s="21">
+        <f>'Forecast'!H40</f>
+        <v/>
+      </c>
+      <c r="J60" s="21">
+        <f>'Forecast'!I40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>Normal Earnings (WACC x Beg NOA)</t>
+        </is>
+      </c>
+      <c r="E61" s="31">
+        <f>$B$18*E60</f>
+        <v/>
+      </c>
+      <c r="F61" s="31">
+        <f>$B$18*F60</f>
+        <v/>
+      </c>
+      <c r="G61" s="31">
+        <f>$B$18*G60</f>
+        <v/>
+      </c>
+      <c r="H61" s="31">
+        <f>$B$18*H60</f>
+        <v/>
+      </c>
+      <c r="I61" s="31">
+        <f>$B$18*I60</f>
+        <v/>
+      </c>
+      <c r="J61" s="31">
+        <f>$B$18*J60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>Abnormal NOPAT</t>
+        </is>
+      </c>
+      <c r="E62" s="31">
+        <f>E59-E61</f>
+        <v/>
+      </c>
+      <c r="F62" s="31">
+        <f>F59-F61</f>
+        <v/>
+      </c>
+      <c r="G62" s="31">
+        <f>G59-G61</f>
+        <v/>
+      </c>
+      <c r="H62" s="31">
+        <f>H59-H61</f>
+        <v/>
+      </c>
+      <c r="I62" s="31">
+        <f>I59-I61</f>
+        <v/>
+      </c>
+      <c r="J62" s="31">
+        <f>J59-J61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>Terminal Value</t>
+        </is>
+      </c>
+      <c r="J63" s="31">
+        <f>J62*(1+$B$22)/($B$18-$B$22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>Discount Factor</t>
+        </is>
+      </c>
+      <c r="E64" s="48">
+        <f>1/(1+$B$18)^1</f>
+        <v/>
+      </c>
+      <c r="F64" s="48">
+        <f>1/(1+$B$18)^2</f>
+        <v/>
+      </c>
+      <c r="G64" s="48">
+        <f>1/(1+$B$18)^3</f>
+        <v/>
+      </c>
+      <c r="H64" s="48">
+        <f>1/(1+$B$18)^4</f>
+        <v/>
+      </c>
+      <c r="I64" s="48">
+        <f>1/(1+$B$18)^5</f>
+        <v/>
+      </c>
+      <c r="J64" s="48">
+        <f>1/(1+$B$18)^6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>PV of Abnormal NOPAT</t>
+        </is>
+      </c>
+      <c r="E65" s="31">
+        <f>E62*E64</f>
+        <v/>
+      </c>
+      <c r="F65" s="31">
+        <f>F62*F64</f>
+        <v/>
+      </c>
+      <c r="G65" s="31">
+        <f>G62*G64</f>
+        <v/>
+      </c>
+      <c r="H65" s="31">
+        <f>H62*H64</f>
+        <v/>
+      </c>
+      <c r="I65" s="31">
+        <f>I62*I64</f>
+        <v/>
+      </c>
+      <c r="J65" s="31">
+        <f>(J62+J63)*J64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="22" t="inlineStr">
+        <is>
+          <t>Sum PV of Abnormal NOPAT</t>
+        </is>
+      </c>
+      <c r="B67" s="23">
+        <f>SUM(E65:J65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>+ Beg BV of NOA (2024)</t>
+        </is>
+      </c>
+      <c r="B68" s="21">
+        <f>'Forecast'!D40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="22">
+        <f> Enterprise Value</f>
+        <v/>
+      </c>
+      <c r="B69" s="23">
+        <f>B67+B68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>- Net Debt</t>
+        </is>
+      </c>
+      <c r="B70" s="31">
+        <f>B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="22">
+        <f> Equity Value</f>
+        <v/>
+      </c>
+      <c r="B71" s="23">
+        <f>B69-B70</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>/ Shares Outstanding</t>
+        </is>
+      </c>
+      <c r="B72" s="31">
+        <f>B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="26" t="inlineStr">
+        <is>
+          <t>Implied Price (PVAOI)</t>
+        </is>
+      </c>
+      <c r="B73" s="49">
+        <f>IF(B72&lt;&gt;0,B71/B72*1000,0)</f>
+        <v/>
+      </c>
+      <c r="C73" s="50" t="n"/>
+      <c r="D73" s="50" t="n"/>
+      <c r="E73" s="50" t="n"/>
+      <c r="F73" s="50" t="n"/>
+      <c r="G73" s="50" t="n"/>
+      <c r="H73" s="50" t="n"/>
+      <c r="I73" s="50" t="n"/>
+      <c r="J73" s="50" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="19" t="inlineStr">
+        <is>
+          <t>PV OF ABNORMAL EARNINGS (PVAE)</t>
+        </is>
+      </c>
+      <c r="B76" s="20" t="n"/>
+      <c r="C76" s="20" t="n"/>
+      <c r="D76" s="20" t="n"/>
+      <c r="E76" s="20" t="n"/>
+      <c r="F76" s="20" t="n"/>
+      <c r="G76" s="20" t="n"/>
+      <c r="H76" s="20" t="n"/>
+      <c r="I76" s="20" t="n"/>
+      <c r="J76" s="20" t="n"/>
+    </row>
+    <row r="78">
+      <c r="E78" s="16" t="inlineStr">
+        <is>
+          <t>2025E</t>
+        </is>
+      </c>
+      <c r="F78" s="16" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="G78" s="16" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+      <c r="H78" s="16" t="inlineStr">
+        <is>
+          <t>2028E</t>
+        </is>
+      </c>
+      <c r="I78" s="16" t="inlineStr">
+        <is>
+          <t>2029E</t>
+        </is>
+      </c>
+      <c r="J78" s="16" t="inlineStr">
+        <is>
+          <t>2030E</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="E79" s="21">
+        <f>'Forecast'!E35</f>
+        <v/>
+      </c>
+      <c r="F79" s="21">
+        <f>'Forecast'!F35</f>
+        <v/>
+      </c>
+      <c r="G79" s="21">
+        <f>'Forecast'!G35</f>
+        <v/>
+      </c>
+      <c r="H79" s="21">
+        <f>'Forecast'!H35</f>
+        <v/>
+      </c>
+      <c r="I79" s="21">
+        <f>'Forecast'!I35</f>
+        <v/>
+      </c>
+      <c r="J79" s="21">
+        <f>'Forecast'!J35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>Beg BV of Equity</t>
+        </is>
+      </c>
+      <c r="E80" s="21">
+        <f>'Forecast'!D47</f>
+        <v/>
+      </c>
+      <c r="F80" s="21">
+        <f>'Forecast'!E47</f>
+        <v/>
+      </c>
+      <c r="G80" s="21">
+        <f>'Forecast'!F47</f>
+        <v/>
+      </c>
+      <c r="H80" s="21">
+        <f>'Forecast'!G47</f>
+        <v/>
+      </c>
+      <c r="I80" s="21">
+        <f>'Forecast'!H47</f>
+        <v/>
+      </c>
+      <c r="J80" s="21">
+        <f>'Forecast'!I47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="11" t="inlineStr">
+        <is>
+          <t>Normal Earnings (Re x Beg Equity)</t>
+        </is>
+      </c>
+      <c r="E81" s="31">
+        <f>$B$8*E80</f>
+        <v/>
+      </c>
+      <c r="F81" s="31">
+        <f>$B$8*F80</f>
+        <v/>
+      </c>
+      <c r="G81" s="31">
+        <f>$B$8*G80</f>
+        <v/>
+      </c>
+      <c r="H81" s="31">
+        <f>$B$8*H80</f>
+        <v/>
+      </c>
+      <c r="I81" s="31">
+        <f>$B$8*I80</f>
+        <v/>
+      </c>
+      <c r="J81" s="31">
+        <f>$B$8*J80</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="inlineStr">
+        <is>
+          <t>Abnormal Earnings</t>
+        </is>
+      </c>
+      <c r="E82" s="31">
+        <f>E79-E81</f>
+        <v/>
+      </c>
+      <c r="F82" s="31">
+        <f>F79-F81</f>
+        <v/>
+      </c>
+      <c r="G82" s="31">
+        <f>G79-G81</f>
+        <v/>
+      </c>
+      <c r="H82" s="31">
+        <f>H79-H81</f>
+        <v/>
+      </c>
+      <c r="I82" s="31">
+        <f>I79-I81</f>
+        <v/>
+      </c>
+      <c r="J82" s="31">
+        <f>J79-J81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="11" t="inlineStr">
+        <is>
+          <t>Terminal Value</t>
+        </is>
+      </c>
+      <c r="J83" s="31">
+        <f>J82*(1+$B$22)/($B$8-$B$22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="inlineStr">
+        <is>
+          <t>Discount Factor</t>
+        </is>
+      </c>
+      <c r="E84" s="48">
+        <f>1/(1+$B$8)^1</f>
+        <v/>
+      </c>
+      <c r="F84" s="48">
+        <f>1/(1+$B$8)^2</f>
+        <v/>
+      </c>
+      <c r="G84" s="48">
+        <f>1/(1+$B$8)^3</f>
+        <v/>
+      </c>
+      <c r="H84" s="48">
+        <f>1/(1+$B$8)^4</f>
+        <v/>
+      </c>
+      <c r="I84" s="48">
+        <f>1/(1+$B$8)^5</f>
+        <v/>
+      </c>
+      <c r="J84" s="48">
+        <f>1/(1+$B$8)^6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="11" t="inlineStr">
+        <is>
+          <t>PV of Abnormal Earnings</t>
+        </is>
+      </c>
+      <c r="E85" s="31">
+        <f>E82*E84</f>
+        <v/>
+      </c>
+      <c r="F85" s="31">
+        <f>F82*F84</f>
+        <v/>
+      </c>
+      <c r="G85" s="31">
+        <f>G82*G84</f>
+        <v/>
+      </c>
+      <c r="H85" s="31">
+        <f>H82*H84</f>
+        <v/>
+      </c>
+      <c r="I85" s="31">
+        <f>I82*I84</f>
+        <v/>
+      </c>
+      <c r="J85" s="31">
+        <f>(J82+J83)*J84</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="22" t="inlineStr">
+        <is>
+          <t>Sum PV of Abnormal Earnings</t>
+        </is>
+      </c>
+      <c r="B87" s="23">
+        <f>SUM(E85:J85)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="11" t="inlineStr">
+        <is>
+          <t>+ Current BV Equity (2024)</t>
+        </is>
+      </c>
+      <c r="B88" s="21">
+        <f>'Adj ASM'!G81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="22">
+        <f> Equity Value</f>
+        <v/>
+      </c>
+      <c r="B89" s="23">
+        <f>B87+B88</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="11" t="inlineStr">
+        <is>
+          <t>/ Shares Outstanding</t>
+        </is>
+      </c>
+      <c r="B90" s="31">
+        <f>B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="26" t="inlineStr">
+        <is>
+          <t>Implied Price (PVAE)</t>
+        </is>
+      </c>
+      <c r="B91" s="49">
+        <f>IF(B90&lt;&gt;0,B89/B90*1000,0)</f>
+        <v/>
+      </c>
+      <c r="C91" s="50" t="n"/>
+      <c r="D91" s="50" t="n"/>
+      <c r="E91" s="50" t="n"/>
+      <c r="F91" s="50" t="n"/>
+      <c r="G91" s="50" t="n"/>
+      <c r="H91" s="50" t="n"/>
+      <c r="I91" s="50" t="n"/>
+      <c r="J91" s="50" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="19" t="inlineStr">
+        <is>
+          <t>SENSITIVITY ANALYSIS</t>
+        </is>
+      </c>
+      <c r="B94" s="20" t="n"/>
+      <c r="C94" s="20" t="n"/>
+      <c r="D94" s="20" t="n"/>
+      <c r="E94" s="20" t="n"/>
+      <c r="F94" s="20" t="n"/>
+      <c r="G94" s="20" t="n"/>
+      <c r="H94" s="20" t="n"/>
+      <c r="I94" s="20" t="n"/>
+      <c r="J94" s="20" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="22" t="inlineStr">
+        <is>
+          <t>DCF (FCFF) - Implied Share Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="51" t="inlineStr">
+        <is>
+          <t>WACC \ Terminal Growth</t>
+        </is>
+      </c>
+      <c r="B97" s="52" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C97" s="52" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D97" s="52" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E97" s="52" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F97" s="52" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G97" s="52" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="H97" s="52" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="53" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="B98" s="54">
+        <f>('Forecast'!E59/(1+$A$98)^1+'Forecast'!F59/(1+$A$98)^2+'Forecast'!G59/(1+$A$98)^3+'Forecast'!H59/(1+$A$98)^4+'Forecast'!I59/(1+$A$98)^5+'Forecast'!J59/(1+$A$98)^6+'Forecast'!J59*(1+B97)/($A$98-B97)/(1+$A$98)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C98" s="54">
+        <f>('Forecast'!E59/(1+$A$98)^1+'Forecast'!F59/(1+$A$98)^2+'Forecast'!G59/(1+$A$98)^3+'Forecast'!H59/(1+$A$98)^4+'Forecast'!I59/(1+$A$98)^5+'Forecast'!J59/(1+$A$98)^6+'Forecast'!J59*(1+C97)/($A$98-C97)/(1+$A$98)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D98" s="54">
+        <f>('Forecast'!E59/(1+$A$98)^1+'Forecast'!F59/(1+$A$98)^2+'Forecast'!G59/(1+$A$98)^3+'Forecast'!H59/(1+$A$98)^4+'Forecast'!I59/(1+$A$98)^5+'Forecast'!J59/(1+$A$98)^6+'Forecast'!J59*(1+D97)/($A$98-D97)/(1+$A$98)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E98" s="54">
+        <f>('Forecast'!E59/(1+$A$98)^1+'Forecast'!F59/(1+$A$98)^2+'Forecast'!G59/(1+$A$98)^3+'Forecast'!H59/(1+$A$98)^4+'Forecast'!I59/(1+$A$98)^5+'Forecast'!J59/(1+$A$98)^6+'Forecast'!J59*(1+E97)/($A$98-E97)/(1+$A$98)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F98" s="54">
+        <f>('Forecast'!E59/(1+$A$98)^1+'Forecast'!F59/(1+$A$98)^2+'Forecast'!G59/(1+$A$98)^3+'Forecast'!H59/(1+$A$98)^4+'Forecast'!I59/(1+$A$98)^5+'Forecast'!J59/(1+$A$98)^6+'Forecast'!J59*(1+F97)/($A$98-F97)/(1+$A$98)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G98" s="54">
+        <f>('Forecast'!E59/(1+$A$98)^1+'Forecast'!F59/(1+$A$98)^2+'Forecast'!G59/(1+$A$98)^3+'Forecast'!H59/(1+$A$98)^4+'Forecast'!I59/(1+$A$98)^5+'Forecast'!J59/(1+$A$98)^6+'Forecast'!J59*(1+G97)/($A$98-G97)/(1+$A$98)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H98" s="54">
+        <f>('Forecast'!E59/(1+$A$98)^1+'Forecast'!F59/(1+$A$98)^2+'Forecast'!G59/(1+$A$98)^3+'Forecast'!H59/(1+$A$98)^4+'Forecast'!I59/(1+$A$98)^5+'Forecast'!J59/(1+$A$98)^6+'Forecast'!J59*(1+H97)/($A$98-H97)/(1+$A$98)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="53" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="B99" s="54">
+        <f>('Forecast'!E59/(1+$A$99)^1+'Forecast'!F59/(1+$A$99)^2+'Forecast'!G59/(1+$A$99)^3+'Forecast'!H59/(1+$A$99)^4+'Forecast'!I59/(1+$A$99)^5+'Forecast'!J59/(1+$A$99)^6+'Forecast'!J59*(1+B97)/($A$99-B97)/(1+$A$99)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C99" s="54">
+        <f>('Forecast'!E59/(1+$A$99)^1+'Forecast'!F59/(1+$A$99)^2+'Forecast'!G59/(1+$A$99)^3+'Forecast'!H59/(1+$A$99)^4+'Forecast'!I59/(1+$A$99)^5+'Forecast'!J59/(1+$A$99)^6+'Forecast'!J59*(1+C97)/($A$99-C97)/(1+$A$99)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D99" s="54">
+        <f>('Forecast'!E59/(1+$A$99)^1+'Forecast'!F59/(1+$A$99)^2+'Forecast'!G59/(1+$A$99)^3+'Forecast'!H59/(1+$A$99)^4+'Forecast'!I59/(1+$A$99)^5+'Forecast'!J59/(1+$A$99)^6+'Forecast'!J59*(1+D97)/($A$99-D97)/(1+$A$99)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E99" s="54">
+        <f>('Forecast'!E59/(1+$A$99)^1+'Forecast'!F59/(1+$A$99)^2+'Forecast'!G59/(1+$A$99)^3+'Forecast'!H59/(1+$A$99)^4+'Forecast'!I59/(1+$A$99)^5+'Forecast'!J59/(1+$A$99)^6+'Forecast'!J59*(1+E97)/($A$99-E97)/(1+$A$99)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F99" s="54">
+        <f>('Forecast'!E59/(1+$A$99)^1+'Forecast'!F59/(1+$A$99)^2+'Forecast'!G59/(1+$A$99)^3+'Forecast'!H59/(1+$A$99)^4+'Forecast'!I59/(1+$A$99)^5+'Forecast'!J59/(1+$A$99)^6+'Forecast'!J59*(1+F97)/($A$99-F97)/(1+$A$99)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G99" s="54">
+        <f>('Forecast'!E59/(1+$A$99)^1+'Forecast'!F59/(1+$A$99)^2+'Forecast'!G59/(1+$A$99)^3+'Forecast'!H59/(1+$A$99)^4+'Forecast'!I59/(1+$A$99)^5+'Forecast'!J59/(1+$A$99)^6+'Forecast'!J59*(1+G97)/($A$99-G97)/(1+$A$99)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H99" s="54">
+        <f>('Forecast'!E59/(1+$A$99)^1+'Forecast'!F59/(1+$A$99)^2+'Forecast'!G59/(1+$A$99)^3+'Forecast'!H59/(1+$A$99)^4+'Forecast'!I59/(1+$A$99)^5+'Forecast'!J59/(1+$A$99)^6+'Forecast'!J59*(1+H97)/($A$99-H97)/(1+$A$99)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="53" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="B100" s="54">
+        <f>('Forecast'!E59/(1+$A$100)^1+'Forecast'!F59/(1+$A$100)^2+'Forecast'!G59/(1+$A$100)^3+'Forecast'!H59/(1+$A$100)^4+'Forecast'!I59/(1+$A$100)^5+'Forecast'!J59/(1+$A$100)^6+'Forecast'!J59*(1+B97)/($A$100-B97)/(1+$A$100)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C100" s="54">
+        <f>('Forecast'!E59/(1+$A$100)^1+'Forecast'!F59/(1+$A$100)^2+'Forecast'!G59/(1+$A$100)^3+'Forecast'!H59/(1+$A$100)^4+'Forecast'!I59/(1+$A$100)^5+'Forecast'!J59/(1+$A$100)^6+'Forecast'!J59*(1+C97)/($A$100-C97)/(1+$A$100)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D100" s="54">
+        <f>('Forecast'!E59/(1+$A$100)^1+'Forecast'!F59/(1+$A$100)^2+'Forecast'!G59/(1+$A$100)^3+'Forecast'!H59/(1+$A$100)^4+'Forecast'!I59/(1+$A$100)^5+'Forecast'!J59/(1+$A$100)^6+'Forecast'!J59*(1+D97)/($A$100-D97)/(1+$A$100)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E100" s="54">
+        <f>('Forecast'!E59/(1+$A$100)^1+'Forecast'!F59/(1+$A$100)^2+'Forecast'!G59/(1+$A$100)^3+'Forecast'!H59/(1+$A$100)^4+'Forecast'!I59/(1+$A$100)^5+'Forecast'!J59/(1+$A$100)^6+'Forecast'!J59*(1+E97)/($A$100-E97)/(1+$A$100)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F100" s="54">
+        <f>('Forecast'!E59/(1+$A$100)^1+'Forecast'!F59/(1+$A$100)^2+'Forecast'!G59/(1+$A$100)^3+'Forecast'!H59/(1+$A$100)^4+'Forecast'!I59/(1+$A$100)^5+'Forecast'!J59/(1+$A$100)^6+'Forecast'!J59*(1+F97)/($A$100-F97)/(1+$A$100)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G100" s="54">
+        <f>('Forecast'!E59/(1+$A$100)^1+'Forecast'!F59/(1+$A$100)^2+'Forecast'!G59/(1+$A$100)^3+'Forecast'!H59/(1+$A$100)^4+'Forecast'!I59/(1+$A$100)^5+'Forecast'!J59/(1+$A$100)^6+'Forecast'!J59*(1+G97)/($A$100-G97)/(1+$A$100)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H100" s="54">
+        <f>('Forecast'!E59/(1+$A$100)^1+'Forecast'!F59/(1+$A$100)^2+'Forecast'!G59/(1+$A$100)^3+'Forecast'!H59/(1+$A$100)^4+'Forecast'!I59/(1+$A$100)^5+'Forecast'!J59/(1+$A$100)^6+'Forecast'!J59*(1+H97)/($A$100-H97)/(1+$A$100)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="53" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="B101" s="54">
+        <f>('Forecast'!E59/(1+$A$101)^1+'Forecast'!F59/(1+$A$101)^2+'Forecast'!G59/(1+$A$101)^3+'Forecast'!H59/(1+$A$101)^4+'Forecast'!I59/(1+$A$101)^5+'Forecast'!J59/(1+$A$101)^6+'Forecast'!J59*(1+B97)/($A$101-B97)/(1+$A$101)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C101" s="54">
+        <f>('Forecast'!E59/(1+$A$101)^1+'Forecast'!F59/(1+$A$101)^2+'Forecast'!G59/(1+$A$101)^3+'Forecast'!H59/(1+$A$101)^4+'Forecast'!I59/(1+$A$101)^5+'Forecast'!J59/(1+$A$101)^6+'Forecast'!J59*(1+C97)/($A$101-C97)/(1+$A$101)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D101" s="54">
+        <f>('Forecast'!E59/(1+$A$101)^1+'Forecast'!F59/(1+$A$101)^2+'Forecast'!G59/(1+$A$101)^3+'Forecast'!H59/(1+$A$101)^4+'Forecast'!I59/(1+$A$101)^5+'Forecast'!J59/(1+$A$101)^6+'Forecast'!J59*(1+D97)/($A$101-D97)/(1+$A$101)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E101" s="54">
+        <f>('Forecast'!E59/(1+$A$101)^1+'Forecast'!F59/(1+$A$101)^2+'Forecast'!G59/(1+$A$101)^3+'Forecast'!H59/(1+$A$101)^4+'Forecast'!I59/(1+$A$101)^5+'Forecast'!J59/(1+$A$101)^6+'Forecast'!J59*(1+E97)/($A$101-E97)/(1+$A$101)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F101" s="54">
+        <f>('Forecast'!E59/(1+$A$101)^1+'Forecast'!F59/(1+$A$101)^2+'Forecast'!G59/(1+$A$101)^3+'Forecast'!H59/(1+$A$101)^4+'Forecast'!I59/(1+$A$101)^5+'Forecast'!J59/(1+$A$101)^6+'Forecast'!J59*(1+F97)/($A$101-F97)/(1+$A$101)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G101" s="54">
+        <f>('Forecast'!E59/(1+$A$101)^1+'Forecast'!F59/(1+$A$101)^2+'Forecast'!G59/(1+$A$101)^3+'Forecast'!H59/(1+$A$101)^4+'Forecast'!I59/(1+$A$101)^5+'Forecast'!J59/(1+$A$101)^6+'Forecast'!J59*(1+G97)/($A$101-G97)/(1+$A$101)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H101" s="54">
+        <f>('Forecast'!E59/(1+$A$101)^1+'Forecast'!F59/(1+$A$101)^2+'Forecast'!G59/(1+$A$101)^3+'Forecast'!H59/(1+$A$101)^4+'Forecast'!I59/(1+$A$101)^5+'Forecast'!J59/(1+$A$101)^6+'Forecast'!J59*(1+H97)/($A$101-H97)/(1+$A$101)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="53" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="B102" s="54">
+        <f>('Forecast'!E59/(1+$A$102)^1+'Forecast'!F59/(1+$A$102)^2+'Forecast'!G59/(1+$A$102)^3+'Forecast'!H59/(1+$A$102)^4+'Forecast'!I59/(1+$A$102)^5+'Forecast'!J59/(1+$A$102)^6+'Forecast'!J59*(1+B97)/($A$102-B97)/(1+$A$102)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C102" s="54">
+        <f>('Forecast'!E59/(1+$A$102)^1+'Forecast'!F59/(1+$A$102)^2+'Forecast'!G59/(1+$A$102)^3+'Forecast'!H59/(1+$A$102)^4+'Forecast'!I59/(1+$A$102)^5+'Forecast'!J59/(1+$A$102)^6+'Forecast'!J59*(1+C97)/($A$102-C97)/(1+$A$102)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D102" s="54">
+        <f>('Forecast'!E59/(1+$A$102)^1+'Forecast'!F59/(1+$A$102)^2+'Forecast'!G59/(1+$A$102)^3+'Forecast'!H59/(1+$A$102)^4+'Forecast'!I59/(1+$A$102)^5+'Forecast'!J59/(1+$A$102)^6+'Forecast'!J59*(1+D97)/($A$102-D97)/(1+$A$102)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E102" s="54">
+        <f>('Forecast'!E59/(1+$A$102)^1+'Forecast'!F59/(1+$A$102)^2+'Forecast'!G59/(1+$A$102)^3+'Forecast'!H59/(1+$A$102)^4+'Forecast'!I59/(1+$A$102)^5+'Forecast'!J59/(1+$A$102)^6+'Forecast'!J59*(1+E97)/($A$102-E97)/(1+$A$102)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F102" s="54">
+        <f>('Forecast'!E59/(1+$A$102)^1+'Forecast'!F59/(1+$A$102)^2+'Forecast'!G59/(1+$A$102)^3+'Forecast'!H59/(1+$A$102)^4+'Forecast'!I59/(1+$A$102)^5+'Forecast'!J59/(1+$A$102)^6+'Forecast'!J59*(1+F97)/($A$102-F97)/(1+$A$102)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G102" s="54">
+        <f>('Forecast'!E59/(1+$A$102)^1+'Forecast'!F59/(1+$A$102)^2+'Forecast'!G59/(1+$A$102)^3+'Forecast'!H59/(1+$A$102)^4+'Forecast'!I59/(1+$A$102)^5+'Forecast'!J59/(1+$A$102)^6+'Forecast'!J59*(1+G97)/($A$102-G97)/(1+$A$102)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H102" s="54">
+        <f>('Forecast'!E59/(1+$A$102)^1+'Forecast'!F59/(1+$A$102)^2+'Forecast'!G59/(1+$A$102)^3+'Forecast'!H59/(1+$A$102)^4+'Forecast'!I59/(1+$A$102)^5+'Forecast'!J59/(1+$A$102)^6+'Forecast'!J59*(1+H97)/($A$102-H97)/(1+$A$102)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="53" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="B103" s="54">
+        <f>('Forecast'!E59/(1+$A$103)^1+'Forecast'!F59/(1+$A$103)^2+'Forecast'!G59/(1+$A$103)^3+'Forecast'!H59/(1+$A$103)^4+'Forecast'!I59/(1+$A$103)^5+'Forecast'!J59/(1+$A$103)^6+'Forecast'!J59*(1+B97)/($A$103-B97)/(1+$A$103)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C103" s="54">
+        <f>('Forecast'!E59/(1+$A$103)^1+'Forecast'!F59/(1+$A$103)^2+'Forecast'!G59/(1+$A$103)^3+'Forecast'!H59/(1+$A$103)^4+'Forecast'!I59/(1+$A$103)^5+'Forecast'!J59/(1+$A$103)^6+'Forecast'!J59*(1+C97)/($A$103-C97)/(1+$A$103)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D103" s="54">
+        <f>('Forecast'!E59/(1+$A$103)^1+'Forecast'!F59/(1+$A$103)^2+'Forecast'!G59/(1+$A$103)^3+'Forecast'!H59/(1+$A$103)^4+'Forecast'!I59/(1+$A$103)^5+'Forecast'!J59/(1+$A$103)^6+'Forecast'!J59*(1+D97)/($A$103-D97)/(1+$A$103)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E103" s="54">
+        <f>('Forecast'!E59/(1+$A$103)^1+'Forecast'!F59/(1+$A$103)^2+'Forecast'!G59/(1+$A$103)^3+'Forecast'!H59/(1+$A$103)^4+'Forecast'!I59/(1+$A$103)^5+'Forecast'!J59/(1+$A$103)^6+'Forecast'!J59*(1+E97)/($A$103-E97)/(1+$A$103)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F103" s="54">
+        <f>('Forecast'!E59/(1+$A$103)^1+'Forecast'!F59/(1+$A$103)^2+'Forecast'!G59/(1+$A$103)^3+'Forecast'!H59/(1+$A$103)^4+'Forecast'!I59/(1+$A$103)^5+'Forecast'!J59/(1+$A$103)^6+'Forecast'!J59*(1+F97)/($A$103-F97)/(1+$A$103)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G103" s="54">
+        <f>('Forecast'!E59/(1+$A$103)^1+'Forecast'!F59/(1+$A$103)^2+'Forecast'!G59/(1+$A$103)^3+'Forecast'!H59/(1+$A$103)^4+'Forecast'!I59/(1+$A$103)^5+'Forecast'!J59/(1+$A$103)^6+'Forecast'!J59*(1+G97)/($A$103-G97)/(1+$A$103)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H103" s="54">
+        <f>('Forecast'!E59/(1+$A$103)^1+'Forecast'!F59/(1+$A$103)^2+'Forecast'!G59/(1+$A$103)^3+'Forecast'!H59/(1+$A$103)^4+'Forecast'!I59/(1+$A$103)^5+'Forecast'!J59/(1+$A$103)^6+'Forecast'!J59*(1+H97)/($A$103-H97)/(1+$A$103)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="53" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B104" s="54">
+        <f>('Forecast'!E59/(1+$A$104)^1+'Forecast'!F59/(1+$A$104)^2+'Forecast'!G59/(1+$A$104)^3+'Forecast'!H59/(1+$A$104)^4+'Forecast'!I59/(1+$A$104)^5+'Forecast'!J59/(1+$A$104)^6+'Forecast'!J59*(1+B97)/($A$104-B97)/(1+$A$104)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C104" s="54">
+        <f>('Forecast'!E59/(1+$A$104)^1+'Forecast'!F59/(1+$A$104)^2+'Forecast'!G59/(1+$A$104)^3+'Forecast'!H59/(1+$A$104)^4+'Forecast'!I59/(1+$A$104)^5+'Forecast'!J59/(1+$A$104)^6+'Forecast'!J59*(1+C97)/($A$104-C97)/(1+$A$104)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D104" s="54">
+        <f>('Forecast'!E59/(1+$A$104)^1+'Forecast'!F59/(1+$A$104)^2+'Forecast'!G59/(1+$A$104)^3+'Forecast'!H59/(1+$A$104)^4+'Forecast'!I59/(1+$A$104)^5+'Forecast'!J59/(1+$A$104)^6+'Forecast'!J59*(1+D97)/($A$104-D97)/(1+$A$104)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E104" s="54">
+        <f>('Forecast'!E59/(1+$A$104)^1+'Forecast'!F59/(1+$A$104)^2+'Forecast'!G59/(1+$A$104)^3+'Forecast'!H59/(1+$A$104)^4+'Forecast'!I59/(1+$A$104)^5+'Forecast'!J59/(1+$A$104)^6+'Forecast'!J59*(1+E97)/($A$104-E97)/(1+$A$104)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F104" s="54">
+        <f>('Forecast'!E59/(1+$A$104)^1+'Forecast'!F59/(1+$A$104)^2+'Forecast'!G59/(1+$A$104)^3+'Forecast'!H59/(1+$A$104)^4+'Forecast'!I59/(1+$A$104)^5+'Forecast'!J59/(1+$A$104)^6+'Forecast'!J59*(1+F97)/($A$104-F97)/(1+$A$104)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G104" s="54">
+        <f>('Forecast'!E59/(1+$A$104)^1+'Forecast'!F59/(1+$A$104)^2+'Forecast'!G59/(1+$A$104)^3+'Forecast'!H59/(1+$A$104)^4+'Forecast'!I59/(1+$A$104)^5+'Forecast'!J59/(1+$A$104)^6+'Forecast'!J59*(1+G97)/($A$104-G97)/(1+$A$104)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H104" s="54">
+        <f>('Forecast'!E59/(1+$A$104)^1+'Forecast'!F59/(1+$A$104)^2+'Forecast'!G59/(1+$A$104)^3+'Forecast'!H59/(1+$A$104)^4+'Forecast'!I59/(1+$A$104)^5+'Forecast'!J59/(1+$A$104)^6+'Forecast'!J59*(1+H97)/($A$104-H97)/(1+$A$104)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="53" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="B105" s="54">
+        <f>('Forecast'!E59/(1+$A$105)^1+'Forecast'!F59/(1+$A$105)^2+'Forecast'!G59/(1+$A$105)^3+'Forecast'!H59/(1+$A$105)^4+'Forecast'!I59/(1+$A$105)^5+'Forecast'!J59/(1+$A$105)^6+'Forecast'!J59*(1+B97)/($A$105-B97)/(1+$A$105)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C105" s="54">
+        <f>('Forecast'!E59/(1+$A$105)^1+'Forecast'!F59/(1+$A$105)^2+'Forecast'!G59/(1+$A$105)^3+'Forecast'!H59/(1+$A$105)^4+'Forecast'!I59/(1+$A$105)^5+'Forecast'!J59/(1+$A$105)^6+'Forecast'!J59*(1+C97)/($A$105-C97)/(1+$A$105)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D105" s="54">
+        <f>('Forecast'!E59/(1+$A$105)^1+'Forecast'!F59/(1+$A$105)^2+'Forecast'!G59/(1+$A$105)^3+'Forecast'!H59/(1+$A$105)^4+'Forecast'!I59/(1+$A$105)^5+'Forecast'!J59/(1+$A$105)^6+'Forecast'!J59*(1+D97)/($A$105-D97)/(1+$A$105)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E105" s="54">
+        <f>('Forecast'!E59/(1+$A$105)^1+'Forecast'!F59/(1+$A$105)^2+'Forecast'!G59/(1+$A$105)^3+'Forecast'!H59/(1+$A$105)^4+'Forecast'!I59/(1+$A$105)^5+'Forecast'!J59/(1+$A$105)^6+'Forecast'!J59*(1+E97)/($A$105-E97)/(1+$A$105)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F105" s="54">
+        <f>('Forecast'!E59/(1+$A$105)^1+'Forecast'!F59/(1+$A$105)^2+'Forecast'!G59/(1+$A$105)^3+'Forecast'!H59/(1+$A$105)^4+'Forecast'!I59/(1+$A$105)^5+'Forecast'!J59/(1+$A$105)^6+'Forecast'!J59*(1+F97)/($A$105-F97)/(1+$A$105)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G105" s="54">
+        <f>('Forecast'!E59/(1+$A$105)^1+'Forecast'!F59/(1+$A$105)^2+'Forecast'!G59/(1+$A$105)^3+'Forecast'!H59/(1+$A$105)^4+'Forecast'!I59/(1+$A$105)^5+'Forecast'!J59/(1+$A$105)^6+'Forecast'!J59*(1+G97)/($A$105-G97)/(1+$A$105)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H105" s="54">
+        <f>('Forecast'!E59/(1+$A$105)^1+'Forecast'!F59/(1+$A$105)^2+'Forecast'!G59/(1+$A$105)^3+'Forecast'!H59/(1+$A$105)^4+'Forecast'!I59/(1+$A$105)^5+'Forecast'!J59/(1+$A$105)^6+'Forecast'!J59*(1+H97)/($A$105-H97)/(1+$A$105)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="53" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="B106" s="54">
+        <f>('Forecast'!E59/(1+$A$106)^1+'Forecast'!F59/(1+$A$106)^2+'Forecast'!G59/(1+$A$106)^3+'Forecast'!H59/(1+$A$106)^4+'Forecast'!I59/(1+$A$106)^5+'Forecast'!J59/(1+$A$106)^6+'Forecast'!J59*(1+B97)/($A$106-B97)/(1+$A$106)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C106" s="54">
+        <f>('Forecast'!E59/(1+$A$106)^1+'Forecast'!F59/(1+$A$106)^2+'Forecast'!G59/(1+$A$106)^3+'Forecast'!H59/(1+$A$106)^4+'Forecast'!I59/(1+$A$106)^5+'Forecast'!J59/(1+$A$106)^6+'Forecast'!J59*(1+C97)/($A$106-C97)/(1+$A$106)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D106" s="54">
+        <f>('Forecast'!E59/(1+$A$106)^1+'Forecast'!F59/(1+$A$106)^2+'Forecast'!G59/(1+$A$106)^3+'Forecast'!H59/(1+$A$106)^4+'Forecast'!I59/(1+$A$106)^5+'Forecast'!J59/(1+$A$106)^6+'Forecast'!J59*(1+D97)/($A$106-D97)/(1+$A$106)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E106" s="54">
+        <f>('Forecast'!E59/(1+$A$106)^1+'Forecast'!F59/(1+$A$106)^2+'Forecast'!G59/(1+$A$106)^3+'Forecast'!H59/(1+$A$106)^4+'Forecast'!I59/(1+$A$106)^5+'Forecast'!J59/(1+$A$106)^6+'Forecast'!J59*(1+E97)/($A$106-E97)/(1+$A$106)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F106" s="54">
+        <f>('Forecast'!E59/(1+$A$106)^1+'Forecast'!F59/(1+$A$106)^2+'Forecast'!G59/(1+$A$106)^3+'Forecast'!H59/(1+$A$106)^4+'Forecast'!I59/(1+$A$106)^5+'Forecast'!J59/(1+$A$106)^6+'Forecast'!J59*(1+F97)/($A$106-F97)/(1+$A$106)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G106" s="54">
+        <f>('Forecast'!E59/(1+$A$106)^1+'Forecast'!F59/(1+$A$106)^2+'Forecast'!G59/(1+$A$106)^3+'Forecast'!H59/(1+$A$106)^4+'Forecast'!I59/(1+$A$106)^5+'Forecast'!J59/(1+$A$106)^6+'Forecast'!J59*(1+G97)/($A$106-G97)/(1+$A$106)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H106" s="54">
+        <f>('Forecast'!E59/(1+$A$106)^1+'Forecast'!F59/(1+$A$106)^2+'Forecast'!G59/(1+$A$106)^3+'Forecast'!H59/(1+$A$106)^4+'Forecast'!I59/(1+$A$106)^5+'Forecast'!J59/(1+$A$106)^6+'Forecast'!J59*(1+H97)/($A$106-H97)/(1+$A$106)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="53" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="B107" s="54">
+        <f>('Forecast'!E59/(1+$A$107)^1+'Forecast'!F59/(1+$A$107)^2+'Forecast'!G59/(1+$A$107)^3+'Forecast'!H59/(1+$A$107)^4+'Forecast'!I59/(1+$A$107)^5+'Forecast'!J59/(1+$A$107)^6+'Forecast'!J59*(1+B97)/($A$107-B97)/(1+$A$107)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C107" s="54">
+        <f>('Forecast'!E59/(1+$A$107)^1+'Forecast'!F59/(1+$A$107)^2+'Forecast'!G59/(1+$A$107)^3+'Forecast'!H59/(1+$A$107)^4+'Forecast'!I59/(1+$A$107)^5+'Forecast'!J59/(1+$A$107)^6+'Forecast'!J59*(1+C97)/($A$107-C97)/(1+$A$107)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D107" s="54">
+        <f>('Forecast'!E59/(1+$A$107)^1+'Forecast'!F59/(1+$A$107)^2+'Forecast'!G59/(1+$A$107)^3+'Forecast'!H59/(1+$A$107)^4+'Forecast'!I59/(1+$A$107)^5+'Forecast'!J59/(1+$A$107)^6+'Forecast'!J59*(1+D97)/($A$107-D97)/(1+$A$107)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E107" s="54">
+        <f>('Forecast'!E59/(1+$A$107)^1+'Forecast'!F59/(1+$A$107)^2+'Forecast'!G59/(1+$A$107)^3+'Forecast'!H59/(1+$A$107)^4+'Forecast'!I59/(1+$A$107)^5+'Forecast'!J59/(1+$A$107)^6+'Forecast'!J59*(1+E97)/($A$107-E97)/(1+$A$107)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F107" s="54">
+        <f>('Forecast'!E59/(1+$A$107)^1+'Forecast'!F59/(1+$A$107)^2+'Forecast'!G59/(1+$A$107)^3+'Forecast'!H59/(1+$A$107)^4+'Forecast'!I59/(1+$A$107)^5+'Forecast'!J59/(1+$A$107)^6+'Forecast'!J59*(1+F97)/($A$107-F97)/(1+$A$107)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G107" s="54">
+        <f>('Forecast'!E59/(1+$A$107)^1+'Forecast'!F59/(1+$A$107)^2+'Forecast'!G59/(1+$A$107)^3+'Forecast'!H59/(1+$A$107)^4+'Forecast'!I59/(1+$A$107)^5+'Forecast'!J59/(1+$A$107)^6+'Forecast'!J59*(1+G97)/($A$107-G97)/(1+$A$107)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H107" s="54">
+        <f>('Forecast'!E59/(1+$A$107)^1+'Forecast'!F59/(1+$A$107)^2+'Forecast'!G59/(1+$A$107)^3+'Forecast'!H59/(1+$A$107)^4+'Forecast'!I59/(1+$A$107)^5+'Forecast'!J59/(1+$A$107)^6+'Forecast'!J59*(1+H97)/($A$107-H97)/(1+$A$107)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="53" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="B108" s="54">
+        <f>('Forecast'!E59/(1+$A$108)^1+'Forecast'!F59/(1+$A$108)^2+'Forecast'!G59/(1+$A$108)^3+'Forecast'!H59/(1+$A$108)^4+'Forecast'!I59/(1+$A$108)^5+'Forecast'!J59/(1+$A$108)^6+'Forecast'!J59*(1+B97)/($A$108-B97)/(1+$A$108)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C108" s="54">
+        <f>('Forecast'!E59/(1+$A$108)^1+'Forecast'!F59/(1+$A$108)^2+'Forecast'!G59/(1+$A$108)^3+'Forecast'!H59/(1+$A$108)^4+'Forecast'!I59/(1+$A$108)^5+'Forecast'!J59/(1+$A$108)^6+'Forecast'!J59*(1+C97)/($A$108-C97)/(1+$A$108)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D108" s="54">
+        <f>('Forecast'!E59/(1+$A$108)^1+'Forecast'!F59/(1+$A$108)^2+'Forecast'!G59/(1+$A$108)^3+'Forecast'!H59/(1+$A$108)^4+'Forecast'!I59/(1+$A$108)^5+'Forecast'!J59/(1+$A$108)^6+'Forecast'!J59*(1+D97)/($A$108-D97)/(1+$A$108)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E108" s="54">
+        <f>('Forecast'!E59/(1+$A$108)^1+'Forecast'!F59/(1+$A$108)^2+'Forecast'!G59/(1+$A$108)^3+'Forecast'!H59/(1+$A$108)^4+'Forecast'!I59/(1+$A$108)^5+'Forecast'!J59/(1+$A$108)^6+'Forecast'!J59*(1+E97)/($A$108-E97)/(1+$A$108)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F108" s="54">
+        <f>('Forecast'!E59/(1+$A$108)^1+'Forecast'!F59/(1+$A$108)^2+'Forecast'!G59/(1+$A$108)^3+'Forecast'!H59/(1+$A$108)^4+'Forecast'!I59/(1+$A$108)^5+'Forecast'!J59/(1+$A$108)^6+'Forecast'!J59*(1+F97)/($A$108-F97)/(1+$A$108)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G108" s="54">
+        <f>('Forecast'!E59/(1+$A$108)^1+'Forecast'!F59/(1+$A$108)^2+'Forecast'!G59/(1+$A$108)^3+'Forecast'!H59/(1+$A$108)^4+'Forecast'!I59/(1+$A$108)^5+'Forecast'!J59/(1+$A$108)^6+'Forecast'!J59*(1+G97)/($A$108-G97)/(1+$A$108)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H108" s="54">
+        <f>('Forecast'!E59/(1+$A$108)^1+'Forecast'!F59/(1+$A$108)^2+'Forecast'!G59/(1+$A$108)^3+'Forecast'!H59/(1+$A$108)^4+'Forecast'!I59/(1+$A$108)^5+'Forecast'!J59/(1+$A$108)^6+'Forecast'!J59*(1+H97)/($A$108-H97)/(1+$A$108)^6-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="22" t="inlineStr">
+        <is>
+          <t>PVAOI - Implied Share Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="51" t="inlineStr">
+        <is>
+          <t>WACC \ Terminal Growth</t>
+        </is>
+      </c>
+      <c r="B112" s="52" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C112" s="52" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D112" s="52" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E112" s="52" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F112" s="52" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G112" s="52" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="H112" s="52" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="53" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="B113" s="54">
+        <f>(('Forecast'!E30-$A$113*'Forecast'!D40)/(1+$A$113)^1+('Forecast'!F30-$A$113*'Forecast'!E40)/(1+$A$113)^2+('Forecast'!G30-$A$113*'Forecast'!F40)/(1+$A$113)^3+('Forecast'!H30-$A$113*'Forecast'!G40)/(1+$A$113)^4+('Forecast'!I30-$A$113*'Forecast'!H40)/(1+$A$113)^5+('Forecast'!J30-$A$113*'Forecast'!I40)/(1+$A$113)^6+('Forecast'!J30-$A$113*'Forecast'!I40)*(1+B112)/($A$113-B112)/(1+$A$113)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C113" s="54">
+        <f>(('Forecast'!E30-$A$113*'Forecast'!D40)/(1+$A$113)^1+('Forecast'!F30-$A$113*'Forecast'!E40)/(1+$A$113)^2+('Forecast'!G30-$A$113*'Forecast'!F40)/(1+$A$113)^3+('Forecast'!H30-$A$113*'Forecast'!G40)/(1+$A$113)^4+('Forecast'!I30-$A$113*'Forecast'!H40)/(1+$A$113)^5+('Forecast'!J30-$A$113*'Forecast'!I40)/(1+$A$113)^6+('Forecast'!J30-$A$113*'Forecast'!I40)*(1+C112)/($A$113-C112)/(1+$A$113)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D113" s="54">
+        <f>(('Forecast'!E30-$A$113*'Forecast'!D40)/(1+$A$113)^1+('Forecast'!F30-$A$113*'Forecast'!E40)/(1+$A$113)^2+('Forecast'!G30-$A$113*'Forecast'!F40)/(1+$A$113)^3+('Forecast'!H30-$A$113*'Forecast'!G40)/(1+$A$113)^4+('Forecast'!I30-$A$113*'Forecast'!H40)/(1+$A$113)^5+('Forecast'!J30-$A$113*'Forecast'!I40)/(1+$A$113)^6+('Forecast'!J30-$A$113*'Forecast'!I40)*(1+D112)/($A$113-D112)/(1+$A$113)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E113" s="54">
+        <f>(('Forecast'!E30-$A$113*'Forecast'!D40)/(1+$A$113)^1+('Forecast'!F30-$A$113*'Forecast'!E40)/(1+$A$113)^2+('Forecast'!G30-$A$113*'Forecast'!F40)/(1+$A$113)^3+('Forecast'!H30-$A$113*'Forecast'!G40)/(1+$A$113)^4+('Forecast'!I30-$A$113*'Forecast'!H40)/(1+$A$113)^5+('Forecast'!J30-$A$113*'Forecast'!I40)/(1+$A$113)^6+('Forecast'!J30-$A$113*'Forecast'!I40)*(1+E112)/($A$113-E112)/(1+$A$113)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F113" s="54">
+        <f>(('Forecast'!E30-$A$113*'Forecast'!D40)/(1+$A$113)^1+('Forecast'!F30-$A$113*'Forecast'!E40)/(1+$A$113)^2+('Forecast'!G30-$A$113*'Forecast'!F40)/(1+$A$113)^3+('Forecast'!H30-$A$113*'Forecast'!G40)/(1+$A$113)^4+('Forecast'!I30-$A$113*'Forecast'!H40)/(1+$A$113)^5+('Forecast'!J30-$A$113*'Forecast'!I40)/(1+$A$113)^6+('Forecast'!J30-$A$113*'Forecast'!I40)*(1+F112)/($A$113-F112)/(1+$A$113)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G113" s="54">
+        <f>(('Forecast'!E30-$A$113*'Forecast'!D40)/(1+$A$113)^1+('Forecast'!F30-$A$113*'Forecast'!E40)/(1+$A$113)^2+('Forecast'!G30-$A$113*'Forecast'!F40)/(1+$A$113)^3+('Forecast'!H30-$A$113*'Forecast'!G40)/(1+$A$113)^4+('Forecast'!I30-$A$113*'Forecast'!H40)/(1+$A$113)^5+('Forecast'!J30-$A$113*'Forecast'!I40)/(1+$A$113)^6+('Forecast'!J30-$A$113*'Forecast'!I40)*(1+G112)/($A$113-G112)/(1+$A$113)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H113" s="54">
+        <f>(('Forecast'!E30-$A$113*'Forecast'!D40)/(1+$A$113)^1+('Forecast'!F30-$A$113*'Forecast'!E40)/(1+$A$113)^2+('Forecast'!G30-$A$113*'Forecast'!F40)/(1+$A$113)^3+('Forecast'!H30-$A$113*'Forecast'!G40)/(1+$A$113)^4+('Forecast'!I30-$A$113*'Forecast'!H40)/(1+$A$113)^5+('Forecast'!J30-$A$113*'Forecast'!I40)/(1+$A$113)^6+('Forecast'!J30-$A$113*'Forecast'!I40)*(1+H112)/($A$113-H112)/(1+$A$113)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="53" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="B114" s="54">
+        <f>(('Forecast'!E30-$A$114*'Forecast'!D40)/(1+$A$114)^1+('Forecast'!F30-$A$114*'Forecast'!E40)/(1+$A$114)^2+('Forecast'!G30-$A$114*'Forecast'!F40)/(1+$A$114)^3+('Forecast'!H30-$A$114*'Forecast'!G40)/(1+$A$114)^4+('Forecast'!I30-$A$114*'Forecast'!H40)/(1+$A$114)^5+('Forecast'!J30-$A$114*'Forecast'!I40)/(1+$A$114)^6+('Forecast'!J30-$A$114*'Forecast'!I40)*(1+B112)/($A$114-B112)/(1+$A$114)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C114" s="54">
+        <f>(('Forecast'!E30-$A$114*'Forecast'!D40)/(1+$A$114)^1+('Forecast'!F30-$A$114*'Forecast'!E40)/(1+$A$114)^2+('Forecast'!G30-$A$114*'Forecast'!F40)/(1+$A$114)^3+('Forecast'!H30-$A$114*'Forecast'!G40)/(1+$A$114)^4+('Forecast'!I30-$A$114*'Forecast'!H40)/(1+$A$114)^5+('Forecast'!J30-$A$114*'Forecast'!I40)/(1+$A$114)^6+('Forecast'!J30-$A$114*'Forecast'!I40)*(1+C112)/($A$114-C112)/(1+$A$114)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D114" s="54">
+        <f>(('Forecast'!E30-$A$114*'Forecast'!D40)/(1+$A$114)^1+('Forecast'!F30-$A$114*'Forecast'!E40)/(1+$A$114)^2+('Forecast'!G30-$A$114*'Forecast'!F40)/(1+$A$114)^3+('Forecast'!H30-$A$114*'Forecast'!G40)/(1+$A$114)^4+('Forecast'!I30-$A$114*'Forecast'!H40)/(1+$A$114)^5+('Forecast'!J30-$A$114*'Forecast'!I40)/(1+$A$114)^6+('Forecast'!J30-$A$114*'Forecast'!I40)*(1+D112)/($A$114-D112)/(1+$A$114)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E114" s="54">
+        <f>(('Forecast'!E30-$A$114*'Forecast'!D40)/(1+$A$114)^1+('Forecast'!F30-$A$114*'Forecast'!E40)/(1+$A$114)^2+('Forecast'!G30-$A$114*'Forecast'!F40)/(1+$A$114)^3+('Forecast'!H30-$A$114*'Forecast'!G40)/(1+$A$114)^4+('Forecast'!I30-$A$114*'Forecast'!H40)/(1+$A$114)^5+('Forecast'!J30-$A$114*'Forecast'!I40)/(1+$A$114)^6+('Forecast'!J30-$A$114*'Forecast'!I40)*(1+E112)/($A$114-E112)/(1+$A$114)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F114" s="54">
+        <f>(('Forecast'!E30-$A$114*'Forecast'!D40)/(1+$A$114)^1+('Forecast'!F30-$A$114*'Forecast'!E40)/(1+$A$114)^2+('Forecast'!G30-$A$114*'Forecast'!F40)/(1+$A$114)^3+('Forecast'!H30-$A$114*'Forecast'!G40)/(1+$A$114)^4+('Forecast'!I30-$A$114*'Forecast'!H40)/(1+$A$114)^5+('Forecast'!J30-$A$114*'Forecast'!I40)/(1+$A$114)^6+('Forecast'!J30-$A$114*'Forecast'!I40)*(1+F112)/($A$114-F112)/(1+$A$114)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G114" s="54">
+        <f>(('Forecast'!E30-$A$114*'Forecast'!D40)/(1+$A$114)^1+('Forecast'!F30-$A$114*'Forecast'!E40)/(1+$A$114)^2+('Forecast'!G30-$A$114*'Forecast'!F40)/(1+$A$114)^3+('Forecast'!H30-$A$114*'Forecast'!G40)/(1+$A$114)^4+('Forecast'!I30-$A$114*'Forecast'!H40)/(1+$A$114)^5+('Forecast'!J30-$A$114*'Forecast'!I40)/(1+$A$114)^6+('Forecast'!J30-$A$114*'Forecast'!I40)*(1+G112)/($A$114-G112)/(1+$A$114)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H114" s="54">
+        <f>(('Forecast'!E30-$A$114*'Forecast'!D40)/(1+$A$114)^1+('Forecast'!F30-$A$114*'Forecast'!E40)/(1+$A$114)^2+('Forecast'!G30-$A$114*'Forecast'!F40)/(1+$A$114)^3+('Forecast'!H30-$A$114*'Forecast'!G40)/(1+$A$114)^4+('Forecast'!I30-$A$114*'Forecast'!H40)/(1+$A$114)^5+('Forecast'!J30-$A$114*'Forecast'!I40)/(1+$A$114)^6+('Forecast'!J30-$A$114*'Forecast'!I40)*(1+H112)/($A$114-H112)/(1+$A$114)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="53" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="B115" s="54">
+        <f>(('Forecast'!E30-$A$115*'Forecast'!D40)/(1+$A$115)^1+('Forecast'!F30-$A$115*'Forecast'!E40)/(1+$A$115)^2+('Forecast'!G30-$A$115*'Forecast'!F40)/(1+$A$115)^3+('Forecast'!H30-$A$115*'Forecast'!G40)/(1+$A$115)^4+('Forecast'!I30-$A$115*'Forecast'!H40)/(1+$A$115)^5+('Forecast'!J30-$A$115*'Forecast'!I40)/(1+$A$115)^6+('Forecast'!J30-$A$115*'Forecast'!I40)*(1+B112)/($A$115-B112)/(1+$A$115)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C115" s="54">
+        <f>(('Forecast'!E30-$A$115*'Forecast'!D40)/(1+$A$115)^1+('Forecast'!F30-$A$115*'Forecast'!E40)/(1+$A$115)^2+('Forecast'!G30-$A$115*'Forecast'!F40)/(1+$A$115)^3+('Forecast'!H30-$A$115*'Forecast'!G40)/(1+$A$115)^4+('Forecast'!I30-$A$115*'Forecast'!H40)/(1+$A$115)^5+('Forecast'!J30-$A$115*'Forecast'!I40)/(1+$A$115)^6+('Forecast'!J30-$A$115*'Forecast'!I40)*(1+C112)/($A$115-C112)/(1+$A$115)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D115" s="54">
+        <f>(('Forecast'!E30-$A$115*'Forecast'!D40)/(1+$A$115)^1+('Forecast'!F30-$A$115*'Forecast'!E40)/(1+$A$115)^2+('Forecast'!G30-$A$115*'Forecast'!F40)/(1+$A$115)^3+('Forecast'!H30-$A$115*'Forecast'!G40)/(1+$A$115)^4+('Forecast'!I30-$A$115*'Forecast'!H40)/(1+$A$115)^5+('Forecast'!J30-$A$115*'Forecast'!I40)/(1+$A$115)^6+('Forecast'!J30-$A$115*'Forecast'!I40)*(1+D112)/($A$115-D112)/(1+$A$115)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E115" s="54">
+        <f>(('Forecast'!E30-$A$115*'Forecast'!D40)/(1+$A$115)^1+('Forecast'!F30-$A$115*'Forecast'!E40)/(1+$A$115)^2+('Forecast'!G30-$A$115*'Forecast'!F40)/(1+$A$115)^3+('Forecast'!H30-$A$115*'Forecast'!G40)/(1+$A$115)^4+('Forecast'!I30-$A$115*'Forecast'!H40)/(1+$A$115)^5+('Forecast'!J30-$A$115*'Forecast'!I40)/(1+$A$115)^6+('Forecast'!J30-$A$115*'Forecast'!I40)*(1+E112)/($A$115-E112)/(1+$A$115)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F115" s="54">
+        <f>(('Forecast'!E30-$A$115*'Forecast'!D40)/(1+$A$115)^1+('Forecast'!F30-$A$115*'Forecast'!E40)/(1+$A$115)^2+('Forecast'!G30-$A$115*'Forecast'!F40)/(1+$A$115)^3+('Forecast'!H30-$A$115*'Forecast'!G40)/(1+$A$115)^4+('Forecast'!I30-$A$115*'Forecast'!H40)/(1+$A$115)^5+('Forecast'!J30-$A$115*'Forecast'!I40)/(1+$A$115)^6+('Forecast'!J30-$A$115*'Forecast'!I40)*(1+F112)/($A$115-F112)/(1+$A$115)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G115" s="54">
+        <f>(('Forecast'!E30-$A$115*'Forecast'!D40)/(1+$A$115)^1+('Forecast'!F30-$A$115*'Forecast'!E40)/(1+$A$115)^2+('Forecast'!G30-$A$115*'Forecast'!F40)/(1+$A$115)^3+('Forecast'!H30-$A$115*'Forecast'!G40)/(1+$A$115)^4+('Forecast'!I30-$A$115*'Forecast'!H40)/(1+$A$115)^5+('Forecast'!J30-$A$115*'Forecast'!I40)/(1+$A$115)^6+('Forecast'!J30-$A$115*'Forecast'!I40)*(1+G112)/($A$115-G112)/(1+$A$115)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H115" s="54">
+        <f>(('Forecast'!E30-$A$115*'Forecast'!D40)/(1+$A$115)^1+('Forecast'!F30-$A$115*'Forecast'!E40)/(1+$A$115)^2+('Forecast'!G30-$A$115*'Forecast'!F40)/(1+$A$115)^3+('Forecast'!H30-$A$115*'Forecast'!G40)/(1+$A$115)^4+('Forecast'!I30-$A$115*'Forecast'!H40)/(1+$A$115)^5+('Forecast'!J30-$A$115*'Forecast'!I40)/(1+$A$115)^6+('Forecast'!J30-$A$115*'Forecast'!I40)*(1+H112)/($A$115-H112)/(1+$A$115)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="53" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="B116" s="54">
+        <f>(('Forecast'!E30-$A$116*'Forecast'!D40)/(1+$A$116)^1+('Forecast'!F30-$A$116*'Forecast'!E40)/(1+$A$116)^2+('Forecast'!G30-$A$116*'Forecast'!F40)/(1+$A$116)^3+('Forecast'!H30-$A$116*'Forecast'!G40)/(1+$A$116)^4+('Forecast'!I30-$A$116*'Forecast'!H40)/(1+$A$116)^5+('Forecast'!J30-$A$116*'Forecast'!I40)/(1+$A$116)^6+('Forecast'!J30-$A$116*'Forecast'!I40)*(1+B112)/($A$116-B112)/(1+$A$116)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C116" s="54">
+        <f>(('Forecast'!E30-$A$116*'Forecast'!D40)/(1+$A$116)^1+('Forecast'!F30-$A$116*'Forecast'!E40)/(1+$A$116)^2+('Forecast'!G30-$A$116*'Forecast'!F40)/(1+$A$116)^3+('Forecast'!H30-$A$116*'Forecast'!G40)/(1+$A$116)^4+('Forecast'!I30-$A$116*'Forecast'!H40)/(1+$A$116)^5+('Forecast'!J30-$A$116*'Forecast'!I40)/(1+$A$116)^6+('Forecast'!J30-$A$116*'Forecast'!I40)*(1+C112)/($A$116-C112)/(1+$A$116)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D116" s="54">
+        <f>(('Forecast'!E30-$A$116*'Forecast'!D40)/(1+$A$116)^1+('Forecast'!F30-$A$116*'Forecast'!E40)/(1+$A$116)^2+('Forecast'!G30-$A$116*'Forecast'!F40)/(1+$A$116)^3+('Forecast'!H30-$A$116*'Forecast'!G40)/(1+$A$116)^4+('Forecast'!I30-$A$116*'Forecast'!H40)/(1+$A$116)^5+('Forecast'!J30-$A$116*'Forecast'!I40)/(1+$A$116)^6+('Forecast'!J30-$A$116*'Forecast'!I40)*(1+D112)/($A$116-D112)/(1+$A$116)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E116" s="54">
+        <f>(('Forecast'!E30-$A$116*'Forecast'!D40)/(1+$A$116)^1+('Forecast'!F30-$A$116*'Forecast'!E40)/(1+$A$116)^2+('Forecast'!G30-$A$116*'Forecast'!F40)/(1+$A$116)^3+('Forecast'!H30-$A$116*'Forecast'!G40)/(1+$A$116)^4+('Forecast'!I30-$A$116*'Forecast'!H40)/(1+$A$116)^5+('Forecast'!J30-$A$116*'Forecast'!I40)/(1+$A$116)^6+('Forecast'!J30-$A$116*'Forecast'!I40)*(1+E112)/($A$116-E112)/(1+$A$116)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F116" s="54">
+        <f>(('Forecast'!E30-$A$116*'Forecast'!D40)/(1+$A$116)^1+('Forecast'!F30-$A$116*'Forecast'!E40)/(1+$A$116)^2+('Forecast'!G30-$A$116*'Forecast'!F40)/(1+$A$116)^3+('Forecast'!H30-$A$116*'Forecast'!G40)/(1+$A$116)^4+('Forecast'!I30-$A$116*'Forecast'!H40)/(1+$A$116)^5+('Forecast'!J30-$A$116*'Forecast'!I40)/(1+$A$116)^6+('Forecast'!J30-$A$116*'Forecast'!I40)*(1+F112)/($A$116-F112)/(1+$A$116)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G116" s="54">
+        <f>(('Forecast'!E30-$A$116*'Forecast'!D40)/(1+$A$116)^1+('Forecast'!F30-$A$116*'Forecast'!E40)/(1+$A$116)^2+('Forecast'!G30-$A$116*'Forecast'!F40)/(1+$A$116)^3+('Forecast'!H30-$A$116*'Forecast'!G40)/(1+$A$116)^4+('Forecast'!I30-$A$116*'Forecast'!H40)/(1+$A$116)^5+('Forecast'!J30-$A$116*'Forecast'!I40)/(1+$A$116)^6+('Forecast'!J30-$A$116*'Forecast'!I40)*(1+G112)/($A$116-G112)/(1+$A$116)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H116" s="54">
+        <f>(('Forecast'!E30-$A$116*'Forecast'!D40)/(1+$A$116)^1+('Forecast'!F30-$A$116*'Forecast'!E40)/(1+$A$116)^2+('Forecast'!G30-$A$116*'Forecast'!F40)/(1+$A$116)^3+('Forecast'!H30-$A$116*'Forecast'!G40)/(1+$A$116)^4+('Forecast'!I30-$A$116*'Forecast'!H40)/(1+$A$116)^5+('Forecast'!J30-$A$116*'Forecast'!I40)/(1+$A$116)^6+('Forecast'!J30-$A$116*'Forecast'!I40)*(1+H112)/($A$116-H112)/(1+$A$116)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="53" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="B117" s="54">
+        <f>(('Forecast'!E30-$A$117*'Forecast'!D40)/(1+$A$117)^1+('Forecast'!F30-$A$117*'Forecast'!E40)/(1+$A$117)^2+('Forecast'!G30-$A$117*'Forecast'!F40)/(1+$A$117)^3+('Forecast'!H30-$A$117*'Forecast'!G40)/(1+$A$117)^4+('Forecast'!I30-$A$117*'Forecast'!H40)/(1+$A$117)^5+('Forecast'!J30-$A$117*'Forecast'!I40)/(1+$A$117)^6+('Forecast'!J30-$A$117*'Forecast'!I40)*(1+B112)/($A$117-B112)/(1+$A$117)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C117" s="54">
+        <f>(('Forecast'!E30-$A$117*'Forecast'!D40)/(1+$A$117)^1+('Forecast'!F30-$A$117*'Forecast'!E40)/(1+$A$117)^2+('Forecast'!G30-$A$117*'Forecast'!F40)/(1+$A$117)^3+('Forecast'!H30-$A$117*'Forecast'!G40)/(1+$A$117)^4+('Forecast'!I30-$A$117*'Forecast'!H40)/(1+$A$117)^5+('Forecast'!J30-$A$117*'Forecast'!I40)/(1+$A$117)^6+('Forecast'!J30-$A$117*'Forecast'!I40)*(1+C112)/($A$117-C112)/(1+$A$117)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D117" s="54">
+        <f>(('Forecast'!E30-$A$117*'Forecast'!D40)/(1+$A$117)^1+('Forecast'!F30-$A$117*'Forecast'!E40)/(1+$A$117)^2+('Forecast'!G30-$A$117*'Forecast'!F40)/(1+$A$117)^3+('Forecast'!H30-$A$117*'Forecast'!G40)/(1+$A$117)^4+('Forecast'!I30-$A$117*'Forecast'!H40)/(1+$A$117)^5+('Forecast'!J30-$A$117*'Forecast'!I40)/(1+$A$117)^6+('Forecast'!J30-$A$117*'Forecast'!I40)*(1+D112)/($A$117-D112)/(1+$A$117)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E117" s="54">
+        <f>(('Forecast'!E30-$A$117*'Forecast'!D40)/(1+$A$117)^1+('Forecast'!F30-$A$117*'Forecast'!E40)/(1+$A$117)^2+('Forecast'!G30-$A$117*'Forecast'!F40)/(1+$A$117)^3+('Forecast'!H30-$A$117*'Forecast'!G40)/(1+$A$117)^4+('Forecast'!I30-$A$117*'Forecast'!H40)/(1+$A$117)^5+('Forecast'!J30-$A$117*'Forecast'!I40)/(1+$A$117)^6+('Forecast'!J30-$A$117*'Forecast'!I40)*(1+E112)/($A$117-E112)/(1+$A$117)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F117" s="54">
+        <f>(('Forecast'!E30-$A$117*'Forecast'!D40)/(1+$A$117)^1+('Forecast'!F30-$A$117*'Forecast'!E40)/(1+$A$117)^2+('Forecast'!G30-$A$117*'Forecast'!F40)/(1+$A$117)^3+('Forecast'!H30-$A$117*'Forecast'!G40)/(1+$A$117)^4+('Forecast'!I30-$A$117*'Forecast'!H40)/(1+$A$117)^5+('Forecast'!J30-$A$117*'Forecast'!I40)/(1+$A$117)^6+('Forecast'!J30-$A$117*'Forecast'!I40)*(1+F112)/($A$117-F112)/(1+$A$117)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G117" s="54">
+        <f>(('Forecast'!E30-$A$117*'Forecast'!D40)/(1+$A$117)^1+('Forecast'!F30-$A$117*'Forecast'!E40)/(1+$A$117)^2+('Forecast'!G30-$A$117*'Forecast'!F40)/(1+$A$117)^3+('Forecast'!H30-$A$117*'Forecast'!G40)/(1+$A$117)^4+('Forecast'!I30-$A$117*'Forecast'!H40)/(1+$A$117)^5+('Forecast'!J30-$A$117*'Forecast'!I40)/(1+$A$117)^6+('Forecast'!J30-$A$117*'Forecast'!I40)*(1+G112)/($A$117-G112)/(1+$A$117)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H117" s="54">
+        <f>(('Forecast'!E30-$A$117*'Forecast'!D40)/(1+$A$117)^1+('Forecast'!F30-$A$117*'Forecast'!E40)/(1+$A$117)^2+('Forecast'!G30-$A$117*'Forecast'!F40)/(1+$A$117)^3+('Forecast'!H30-$A$117*'Forecast'!G40)/(1+$A$117)^4+('Forecast'!I30-$A$117*'Forecast'!H40)/(1+$A$117)^5+('Forecast'!J30-$A$117*'Forecast'!I40)/(1+$A$117)^6+('Forecast'!J30-$A$117*'Forecast'!I40)*(1+H112)/($A$117-H112)/(1+$A$117)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="53" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="B118" s="54">
+        <f>(('Forecast'!E30-$A$118*'Forecast'!D40)/(1+$A$118)^1+('Forecast'!F30-$A$118*'Forecast'!E40)/(1+$A$118)^2+('Forecast'!G30-$A$118*'Forecast'!F40)/(1+$A$118)^3+('Forecast'!H30-$A$118*'Forecast'!G40)/(1+$A$118)^4+('Forecast'!I30-$A$118*'Forecast'!H40)/(1+$A$118)^5+('Forecast'!J30-$A$118*'Forecast'!I40)/(1+$A$118)^6+('Forecast'!J30-$A$118*'Forecast'!I40)*(1+B112)/($A$118-B112)/(1+$A$118)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C118" s="54">
+        <f>(('Forecast'!E30-$A$118*'Forecast'!D40)/(1+$A$118)^1+('Forecast'!F30-$A$118*'Forecast'!E40)/(1+$A$118)^2+('Forecast'!G30-$A$118*'Forecast'!F40)/(1+$A$118)^3+('Forecast'!H30-$A$118*'Forecast'!G40)/(1+$A$118)^4+('Forecast'!I30-$A$118*'Forecast'!H40)/(1+$A$118)^5+('Forecast'!J30-$A$118*'Forecast'!I40)/(1+$A$118)^6+('Forecast'!J30-$A$118*'Forecast'!I40)*(1+C112)/($A$118-C112)/(1+$A$118)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D118" s="54">
+        <f>(('Forecast'!E30-$A$118*'Forecast'!D40)/(1+$A$118)^1+('Forecast'!F30-$A$118*'Forecast'!E40)/(1+$A$118)^2+('Forecast'!G30-$A$118*'Forecast'!F40)/(1+$A$118)^3+('Forecast'!H30-$A$118*'Forecast'!G40)/(1+$A$118)^4+('Forecast'!I30-$A$118*'Forecast'!H40)/(1+$A$118)^5+('Forecast'!J30-$A$118*'Forecast'!I40)/(1+$A$118)^6+('Forecast'!J30-$A$118*'Forecast'!I40)*(1+D112)/($A$118-D112)/(1+$A$118)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E118" s="54">
+        <f>(('Forecast'!E30-$A$118*'Forecast'!D40)/(1+$A$118)^1+('Forecast'!F30-$A$118*'Forecast'!E40)/(1+$A$118)^2+('Forecast'!G30-$A$118*'Forecast'!F40)/(1+$A$118)^3+('Forecast'!H30-$A$118*'Forecast'!G40)/(1+$A$118)^4+('Forecast'!I30-$A$118*'Forecast'!H40)/(1+$A$118)^5+('Forecast'!J30-$A$118*'Forecast'!I40)/(1+$A$118)^6+('Forecast'!J30-$A$118*'Forecast'!I40)*(1+E112)/($A$118-E112)/(1+$A$118)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F118" s="54">
+        <f>(('Forecast'!E30-$A$118*'Forecast'!D40)/(1+$A$118)^1+('Forecast'!F30-$A$118*'Forecast'!E40)/(1+$A$118)^2+('Forecast'!G30-$A$118*'Forecast'!F40)/(1+$A$118)^3+('Forecast'!H30-$A$118*'Forecast'!G40)/(1+$A$118)^4+('Forecast'!I30-$A$118*'Forecast'!H40)/(1+$A$118)^5+('Forecast'!J30-$A$118*'Forecast'!I40)/(1+$A$118)^6+('Forecast'!J30-$A$118*'Forecast'!I40)*(1+F112)/($A$118-F112)/(1+$A$118)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G118" s="54">
+        <f>(('Forecast'!E30-$A$118*'Forecast'!D40)/(1+$A$118)^1+('Forecast'!F30-$A$118*'Forecast'!E40)/(1+$A$118)^2+('Forecast'!G30-$A$118*'Forecast'!F40)/(1+$A$118)^3+('Forecast'!H30-$A$118*'Forecast'!G40)/(1+$A$118)^4+('Forecast'!I30-$A$118*'Forecast'!H40)/(1+$A$118)^5+('Forecast'!J30-$A$118*'Forecast'!I40)/(1+$A$118)^6+('Forecast'!J30-$A$118*'Forecast'!I40)*(1+G112)/($A$118-G112)/(1+$A$118)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H118" s="54">
+        <f>(('Forecast'!E30-$A$118*'Forecast'!D40)/(1+$A$118)^1+('Forecast'!F30-$A$118*'Forecast'!E40)/(1+$A$118)^2+('Forecast'!G30-$A$118*'Forecast'!F40)/(1+$A$118)^3+('Forecast'!H30-$A$118*'Forecast'!G40)/(1+$A$118)^4+('Forecast'!I30-$A$118*'Forecast'!H40)/(1+$A$118)^5+('Forecast'!J30-$A$118*'Forecast'!I40)/(1+$A$118)^6+('Forecast'!J30-$A$118*'Forecast'!I40)*(1+H112)/($A$118-H112)/(1+$A$118)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="53" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B119" s="54">
+        <f>(('Forecast'!E30-$A$119*'Forecast'!D40)/(1+$A$119)^1+('Forecast'!F30-$A$119*'Forecast'!E40)/(1+$A$119)^2+('Forecast'!G30-$A$119*'Forecast'!F40)/(1+$A$119)^3+('Forecast'!H30-$A$119*'Forecast'!G40)/(1+$A$119)^4+('Forecast'!I30-$A$119*'Forecast'!H40)/(1+$A$119)^5+('Forecast'!J30-$A$119*'Forecast'!I40)/(1+$A$119)^6+('Forecast'!J30-$A$119*'Forecast'!I40)*(1+B112)/($A$119-B112)/(1+$A$119)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C119" s="54">
+        <f>(('Forecast'!E30-$A$119*'Forecast'!D40)/(1+$A$119)^1+('Forecast'!F30-$A$119*'Forecast'!E40)/(1+$A$119)^2+('Forecast'!G30-$A$119*'Forecast'!F40)/(1+$A$119)^3+('Forecast'!H30-$A$119*'Forecast'!G40)/(1+$A$119)^4+('Forecast'!I30-$A$119*'Forecast'!H40)/(1+$A$119)^5+('Forecast'!J30-$A$119*'Forecast'!I40)/(1+$A$119)^6+('Forecast'!J30-$A$119*'Forecast'!I40)*(1+C112)/($A$119-C112)/(1+$A$119)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D119" s="54">
+        <f>(('Forecast'!E30-$A$119*'Forecast'!D40)/(1+$A$119)^1+('Forecast'!F30-$A$119*'Forecast'!E40)/(1+$A$119)^2+('Forecast'!G30-$A$119*'Forecast'!F40)/(1+$A$119)^3+('Forecast'!H30-$A$119*'Forecast'!G40)/(1+$A$119)^4+('Forecast'!I30-$A$119*'Forecast'!H40)/(1+$A$119)^5+('Forecast'!J30-$A$119*'Forecast'!I40)/(1+$A$119)^6+('Forecast'!J30-$A$119*'Forecast'!I40)*(1+D112)/($A$119-D112)/(1+$A$119)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E119" s="54">
+        <f>(('Forecast'!E30-$A$119*'Forecast'!D40)/(1+$A$119)^1+('Forecast'!F30-$A$119*'Forecast'!E40)/(1+$A$119)^2+('Forecast'!G30-$A$119*'Forecast'!F40)/(1+$A$119)^3+('Forecast'!H30-$A$119*'Forecast'!G40)/(1+$A$119)^4+('Forecast'!I30-$A$119*'Forecast'!H40)/(1+$A$119)^5+('Forecast'!J30-$A$119*'Forecast'!I40)/(1+$A$119)^6+('Forecast'!J30-$A$119*'Forecast'!I40)*(1+E112)/($A$119-E112)/(1+$A$119)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F119" s="54">
+        <f>(('Forecast'!E30-$A$119*'Forecast'!D40)/(1+$A$119)^1+('Forecast'!F30-$A$119*'Forecast'!E40)/(1+$A$119)^2+('Forecast'!G30-$A$119*'Forecast'!F40)/(1+$A$119)^3+('Forecast'!H30-$A$119*'Forecast'!G40)/(1+$A$119)^4+('Forecast'!I30-$A$119*'Forecast'!H40)/(1+$A$119)^5+('Forecast'!J30-$A$119*'Forecast'!I40)/(1+$A$119)^6+('Forecast'!J30-$A$119*'Forecast'!I40)*(1+F112)/($A$119-F112)/(1+$A$119)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G119" s="54">
+        <f>(('Forecast'!E30-$A$119*'Forecast'!D40)/(1+$A$119)^1+('Forecast'!F30-$A$119*'Forecast'!E40)/(1+$A$119)^2+('Forecast'!G30-$A$119*'Forecast'!F40)/(1+$A$119)^3+('Forecast'!H30-$A$119*'Forecast'!G40)/(1+$A$119)^4+('Forecast'!I30-$A$119*'Forecast'!H40)/(1+$A$119)^5+('Forecast'!J30-$A$119*'Forecast'!I40)/(1+$A$119)^6+('Forecast'!J30-$A$119*'Forecast'!I40)*(1+G112)/($A$119-G112)/(1+$A$119)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H119" s="54">
+        <f>(('Forecast'!E30-$A$119*'Forecast'!D40)/(1+$A$119)^1+('Forecast'!F30-$A$119*'Forecast'!E40)/(1+$A$119)^2+('Forecast'!G30-$A$119*'Forecast'!F40)/(1+$A$119)^3+('Forecast'!H30-$A$119*'Forecast'!G40)/(1+$A$119)^4+('Forecast'!I30-$A$119*'Forecast'!H40)/(1+$A$119)^5+('Forecast'!J30-$A$119*'Forecast'!I40)/(1+$A$119)^6+('Forecast'!J30-$A$119*'Forecast'!I40)*(1+H112)/($A$119-H112)/(1+$A$119)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="53" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="B120" s="54">
+        <f>(('Forecast'!E30-$A$120*'Forecast'!D40)/(1+$A$120)^1+('Forecast'!F30-$A$120*'Forecast'!E40)/(1+$A$120)^2+('Forecast'!G30-$A$120*'Forecast'!F40)/(1+$A$120)^3+('Forecast'!H30-$A$120*'Forecast'!G40)/(1+$A$120)^4+('Forecast'!I30-$A$120*'Forecast'!H40)/(1+$A$120)^5+('Forecast'!J30-$A$120*'Forecast'!I40)/(1+$A$120)^6+('Forecast'!J30-$A$120*'Forecast'!I40)*(1+B112)/($A$120-B112)/(1+$A$120)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C120" s="54">
+        <f>(('Forecast'!E30-$A$120*'Forecast'!D40)/(1+$A$120)^1+('Forecast'!F30-$A$120*'Forecast'!E40)/(1+$A$120)^2+('Forecast'!G30-$A$120*'Forecast'!F40)/(1+$A$120)^3+('Forecast'!H30-$A$120*'Forecast'!G40)/(1+$A$120)^4+('Forecast'!I30-$A$120*'Forecast'!H40)/(1+$A$120)^5+('Forecast'!J30-$A$120*'Forecast'!I40)/(1+$A$120)^6+('Forecast'!J30-$A$120*'Forecast'!I40)*(1+C112)/($A$120-C112)/(1+$A$120)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D120" s="54">
+        <f>(('Forecast'!E30-$A$120*'Forecast'!D40)/(1+$A$120)^1+('Forecast'!F30-$A$120*'Forecast'!E40)/(1+$A$120)^2+('Forecast'!G30-$A$120*'Forecast'!F40)/(1+$A$120)^3+('Forecast'!H30-$A$120*'Forecast'!G40)/(1+$A$120)^4+('Forecast'!I30-$A$120*'Forecast'!H40)/(1+$A$120)^5+('Forecast'!J30-$A$120*'Forecast'!I40)/(1+$A$120)^6+('Forecast'!J30-$A$120*'Forecast'!I40)*(1+D112)/($A$120-D112)/(1+$A$120)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E120" s="54">
+        <f>(('Forecast'!E30-$A$120*'Forecast'!D40)/(1+$A$120)^1+('Forecast'!F30-$A$120*'Forecast'!E40)/(1+$A$120)^2+('Forecast'!G30-$A$120*'Forecast'!F40)/(1+$A$120)^3+('Forecast'!H30-$A$120*'Forecast'!G40)/(1+$A$120)^4+('Forecast'!I30-$A$120*'Forecast'!H40)/(1+$A$120)^5+('Forecast'!J30-$A$120*'Forecast'!I40)/(1+$A$120)^6+('Forecast'!J30-$A$120*'Forecast'!I40)*(1+E112)/($A$120-E112)/(1+$A$120)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F120" s="54">
+        <f>(('Forecast'!E30-$A$120*'Forecast'!D40)/(1+$A$120)^1+('Forecast'!F30-$A$120*'Forecast'!E40)/(1+$A$120)^2+('Forecast'!G30-$A$120*'Forecast'!F40)/(1+$A$120)^3+('Forecast'!H30-$A$120*'Forecast'!G40)/(1+$A$120)^4+('Forecast'!I30-$A$120*'Forecast'!H40)/(1+$A$120)^5+('Forecast'!J30-$A$120*'Forecast'!I40)/(1+$A$120)^6+('Forecast'!J30-$A$120*'Forecast'!I40)*(1+F112)/($A$120-F112)/(1+$A$120)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G120" s="54">
+        <f>(('Forecast'!E30-$A$120*'Forecast'!D40)/(1+$A$120)^1+('Forecast'!F30-$A$120*'Forecast'!E40)/(1+$A$120)^2+('Forecast'!G30-$A$120*'Forecast'!F40)/(1+$A$120)^3+('Forecast'!H30-$A$120*'Forecast'!G40)/(1+$A$120)^4+('Forecast'!I30-$A$120*'Forecast'!H40)/(1+$A$120)^5+('Forecast'!J30-$A$120*'Forecast'!I40)/(1+$A$120)^6+('Forecast'!J30-$A$120*'Forecast'!I40)*(1+G112)/($A$120-G112)/(1+$A$120)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H120" s="54">
+        <f>(('Forecast'!E30-$A$120*'Forecast'!D40)/(1+$A$120)^1+('Forecast'!F30-$A$120*'Forecast'!E40)/(1+$A$120)^2+('Forecast'!G30-$A$120*'Forecast'!F40)/(1+$A$120)^3+('Forecast'!H30-$A$120*'Forecast'!G40)/(1+$A$120)^4+('Forecast'!I30-$A$120*'Forecast'!H40)/(1+$A$120)^5+('Forecast'!J30-$A$120*'Forecast'!I40)/(1+$A$120)^6+('Forecast'!J30-$A$120*'Forecast'!I40)*(1+H112)/($A$120-H112)/(1+$A$120)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="53" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="B121" s="54">
+        <f>(('Forecast'!E30-$A$121*'Forecast'!D40)/(1+$A$121)^1+('Forecast'!F30-$A$121*'Forecast'!E40)/(1+$A$121)^2+('Forecast'!G30-$A$121*'Forecast'!F40)/(1+$A$121)^3+('Forecast'!H30-$A$121*'Forecast'!G40)/(1+$A$121)^4+('Forecast'!I30-$A$121*'Forecast'!H40)/(1+$A$121)^5+('Forecast'!J30-$A$121*'Forecast'!I40)/(1+$A$121)^6+('Forecast'!J30-$A$121*'Forecast'!I40)*(1+B112)/($A$121-B112)/(1+$A$121)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C121" s="54">
+        <f>(('Forecast'!E30-$A$121*'Forecast'!D40)/(1+$A$121)^1+('Forecast'!F30-$A$121*'Forecast'!E40)/(1+$A$121)^2+('Forecast'!G30-$A$121*'Forecast'!F40)/(1+$A$121)^3+('Forecast'!H30-$A$121*'Forecast'!G40)/(1+$A$121)^4+('Forecast'!I30-$A$121*'Forecast'!H40)/(1+$A$121)^5+('Forecast'!J30-$A$121*'Forecast'!I40)/(1+$A$121)^6+('Forecast'!J30-$A$121*'Forecast'!I40)*(1+C112)/($A$121-C112)/(1+$A$121)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D121" s="54">
+        <f>(('Forecast'!E30-$A$121*'Forecast'!D40)/(1+$A$121)^1+('Forecast'!F30-$A$121*'Forecast'!E40)/(1+$A$121)^2+('Forecast'!G30-$A$121*'Forecast'!F40)/(1+$A$121)^3+('Forecast'!H30-$A$121*'Forecast'!G40)/(1+$A$121)^4+('Forecast'!I30-$A$121*'Forecast'!H40)/(1+$A$121)^5+('Forecast'!J30-$A$121*'Forecast'!I40)/(1+$A$121)^6+('Forecast'!J30-$A$121*'Forecast'!I40)*(1+D112)/($A$121-D112)/(1+$A$121)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E121" s="54">
+        <f>(('Forecast'!E30-$A$121*'Forecast'!D40)/(1+$A$121)^1+('Forecast'!F30-$A$121*'Forecast'!E40)/(1+$A$121)^2+('Forecast'!G30-$A$121*'Forecast'!F40)/(1+$A$121)^3+('Forecast'!H30-$A$121*'Forecast'!G40)/(1+$A$121)^4+('Forecast'!I30-$A$121*'Forecast'!H40)/(1+$A$121)^5+('Forecast'!J30-$A$121*'Forecast'!I40)/(1+$A$121)^6+('Forecast'!J30-$A$121*'Forecast'!I40)*(1+E112)/($A$121-E112)/(1+$A$121)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F121" s="54">
+        <f>(('Forecast'!E30-$A$121*'Forecast'!D40)/(1+$A$121)^1+('Forecast'!F30-$A$121*'Forecast'!E40)/(1+$A$121)^2+('Forecast'!G30-$A$121*'Forecast'!F40)/(1+$A$121)^3+('Forecast'!H30-$A$121*'Forecast'!G40)/(1+$A$121)^4+('Forecast'!I30-$A$121*'Forecast'!H40)/(1+$A$121)^5+('Forecast'!J30-$A$121*'Forecast'!I40)/(1+$A$121)^6+('Forecast'!J30-$A$121*'Forecast'!I40)*(1+F112)/($A$121-F112)/(1+$A$121)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G121" s="54">
+        <f>(('Forecast'!E30-$A$121*'Forecast'!D40)/(1+$A$121)^1+('Forecast'!F30-$A$121*'Forecast'!E40)/(1+$A$121)^2+('Forecast'!G30-$A$121*'Forecast'!F40)/(1+$A$121)^3+('Forecast'!H30-$A$121*'Forecast'!G40)/(1+$A$121)^4+('Forecast'!I30-$A$121*'Forecast'!H40)/(1+$A$121)^5+('Forecast'!J30-$A$121*'Forecast'!I40)/(1+$A$121)^6+('Forecast'!J30-$A$121*'Forecast'!I40)*(1+G112)/($A$121-G112)/(1+$A$121)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H121" s="54">
+        <f>(('Forecast'!E30-$A$121*'Forecast'!D40)/(1+$A$121)^1+('Forecast'!F30-$A$121*'Forecast'!E40)/(1+$A$121)^2+('Forecast'!G30-$A$121*'Forecast'!F40)/(1+$A$121)^3+('Forecast'!H30-$A$121*'Forecast'!G40)/(1+$A$121)^4+('Forecast'!I30-$A$121*'Forecast'!H40)/(1+$A$121)^5+('Forecast'!J30-$A$121*'Forecast'!I40)/(1+$A$121)^6+('Forecast'!J30-$A$121*'Forecast'!I40)*(1+H112)/($A$121-H112)/(1+$A$121)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="53" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="B122" s="54">
+        <f>(('Forecast'!E30-$A$122*'Forecast'!D40)/(1+$A$122)^1+('Forecast'!F30-$A$122*'Forecast'!E40)/(1+$A$122)^2+('Forecast'!G30-$A$122*'Forecast'!F40)/(1+$A$122)^3+('Forecast'!H30-$A$122*'Forecast'!G40)/(1+$A$122)^4+('Forecast'!I30-$A$122*'Forecast'!H40)/(1+$A$122)^5+('Forecast'!J30-$A$122*'Forecast'!I40)/(1+$A$122)^6+('Forecast'!J30-$A$122*'Forecast'!I40)*(1+B112)/($A$122-B112)/(1+$A$122)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C122" s="54">
+        <f>(('Forecast'!E30-$A$122*'Forecast'!D40)/(1+$A$122)^1+('Forecast'!F30-$A$122*'Forecast'!E40)/(1+$A$122)^2+('Forecast'!G30-$A$122*'Forecast'!F40)/(1+$A$122)^3+('Forecast'!H30-$A$122*'Forecast'!G40)/(1+$A$122)^4+('Forecast'!I30-$A$122*'Forecast'!H40)/(1+$A$122)^5+('Forecast'!J30-$A$122*'Forecast'!I40)/(1+$A$122)^6+('Forecast'!J30-$A$122*'Forecast'!I40)*(1+C112)/($A$122-C112)/(1+$A$122)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D122" s="54">
+        <f>(('Forecast'!E30-$A$122*'Forecast'!D40)/(1+$A$122)^1+('Forecast'!F30-$A$122*'Forecast'!E40)/(1+$A$122)^2+('Forecast'!G30-$A$122*'Forecast'!F40)/(1+$A$122)^3+('Forecast'!H30-$A$122*'Forecast'!G40)/(1+$A$122)^4+('Forecast'!I30-$A$122*'Forecast'!H40)/(1+$A$122)^5+('Forecast'!J30-$A$122*'Forecast'!I40)/(1+$A$122)^6+('Forecast'!J30-$A$122*'Forecast'!I40)*(1+D112)/($A$122-D112)/(1+$A$122)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E122" s="54">
+        <f>(('Forecast'!E30-$A$122*'Forecast'!D40)/(1+$A$122)^1+('Forecast'!F30-$A$122*'Forecast'!E40)/(1+$A$122)^2+('Forecast'!G30-$A$122*'Forecast'!F40)/(1+$A$122)^3+('Forecast'!H30-$A$122*'Forecast'!G40)/(1+$A$122)^4+('Forecast'!I30-$A$122*'Forecast'!H40)/(1+$A$122)^5+('Forecast'!J30-$A$122*'Forecast'!I40)/(1+$A$122)^6+('Forecast'!J30-$A$122*'Forecast'!I40)*(1+E112)/($A$122-E112)/(1+$A$122)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F122" s="54">
+        <f>(('Forecast'!E30-$A$122*'Forecast'!D40)/(1+$A$122)^1+('Forecast'!F30-$A$122*'Forecast'!E40)/(1+$A$122)^2+('Forecast'!G30-$A$122*'Forecast'!F40)/(1+$A$122)^3+('Forecast'!H30-$A$122*'Forecast'!G40)/(1+$A$122)^4+('Forecast'!I30-$A$122*'Forecast'!H40)/(1+$A$122)^5+('Forecast'!J30-$A$122*'Forecast'!I40)/(1+$A$122)^6+('Forecast'!J30-$A$122*'Forecast'!I40)*(1+F112)/($A$122-F112)/(1+$A$122)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G122" s="54">
+        <f>(('Forecast'!E30-$A$122*'Forecast'!D40)/(1+$A$122)^1+('Forecast'!F30-$A$122*'Forecast'!E40)/(1+$A$122)^2+('Forecast'!G30-$A$122*'Forecast'!F40)/(1+$A$122)^3+('Forecast'!H30-$A$122*'Forecast'!G40)/(1+$A$122)^4+('Forecast'!I30-$A$122*'Forecast'!H40)/(1+$A$122)^5+('Forecast'!J30-$A$122*'Forecast'!I40)/(1+$A$122)^6+('Forecast'!J30-$A$122*'Forecast'!I40)*(1+G112)/($A$122-G112)/(1+$A$122)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H122" s="54">
+        <f>(('Forecast'!E30-$A$122*'Forecast'!D40)/(1+$A$122)^1+('Forecast'!F30-$A$122*'Forecast'!E40)/(1+$A$122)^2+('Forecast'!G30-$A$122*'Forecast'!F40)/(1+$A$122)^3+('Forecast'!H30-$A$122*'Forecast'!G40)/(1+$A$122)^4+('Forecast'!I30-$A$122*'Forecast'!H40)/(1+$A$122)^5+('Forecast'!J30-$A$122*'Forecast'!I40)/(1+$A$122)^6+('Forecast'!J30-$A$122*'Forecast'!I40)*(1+H112)/($A$122-H112)/(1+$A$122)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="53" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="B123" s="54">
+        <f>(('Forecast'!E30-$A$123*'Forecast'!D40)/(1+$A$123)^1+('Forecast'!F30-$A$123*'Forecast'!E40)/(1+$A$123)^2+('Forecast'!G30-$A$123*'Forecast'!F40)/(1+$A$123)^3+('Forecast'!H30-$A$123*'Forecast'!G40)/(1+$A$123)^4+('Forecast'!I30-$A$123*'Forecast'!H40)/(1+$A$123)^5+('Forecast'!J30-$A$123*'Forecast'!I40)/(1+$A$123)^6+('Forecast'!J30-$A$123*'Forecast'!I40)*(1+B112)/($A$123-B112)/(1+$A$123)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="C123" s="54">
+        <f>(('Forecast'!E30-$A$123*'Forecast'!D40)/(1+$A$123)^1+('Forecast'!F30-$A$123*'Forecast'!E40)/(1+$A$123)^2+('Forecast'!G30-$A$123*'Forecast'!F40)/(1+$A$123)^3+('Forecast'!H30-$A$123*'Forecast'!G40)/(1+$A$123)^4+('Forecast'!I30-$A$123*'Forecast'!H40)/(1+$A$123)^5+('Forecast'!J30-$A$123*'Forecast'!I40)/(1+$A$123)^6+('Forecast'!J30-$A$123*'Forecast'!I40)*(1+C112)/($A$123-C112)/(1+$A$123)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="D123" s="54">
+        <f>(('Forecast'!E30-$A$123*'Forecast'!D40)/(1+$A$123)^1+('Forecast'!F30-$A$123*'Forecast'!E40)/(1+$A$123)^2+('Forecast'!G30-$A$123*'Forecast'!F40)/(1+$A$123)^3+('Forecast'!H30-$A$123*'Forecast'!G40)/(1+$A$123)^4+('Forecast'!I30-$A$123*'Forecast'!H40)/(1+$A$123)^5+('Forecast'!J30-$A$123*'Forecast'!I40)/(1+$A$123)^6+('Forecast'!J30-$A$123*'Forecast'!I40)*(1+D112)/($A$123-D112)/(1+$A$123)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="E123" s="54">
+        <f>(('Forecast'!E30-$A$123*'Forecast'!D40)/(1+$A$123)^1+('Forecast'!F30-$A$123*'Forecast'!E40)/(1+$A$123)^2+('Forecast'!G30-$A$123*'Forecast'!F40)/(1+$A$123)^3+('Forecast'!H30-$A$123*'Forecast'!G40)/(1+$A$123)^4+('Forecast'!I30-$A$123*'Forecast'!H40)/(1+$A$123)^5+('Forecast'!J30-$A$123*'Forecast'!I40)/(1+$A$123)^6+('Forecast'!J30-$A$123*'Forecast'!I40)*(1+E112)/($A$123-E112)/(1+$A$123)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="F123" s="54">
+        <f>(('Forecast'!E30-$A$123*'Forecast'!D40)/(1+$A$123)^1+('Forecast'!F30-$A$123*'Forecast'!E40)/(1+$A$123)^2+('Forecast'!G30-$A$123*'Forecast'!F40)/(1+$A$123)^3+('Forecast'!H30-$A$123*'Forecast'!G40)/(1+$A$123)^4+('Forecast'!I30-$A$123*'Forecast'!H40)/(1+$A$123)^5+('Forecast'!J30-$A$123*'Forecast'!I40)/(1+$A$123)^6+('Forecast'!J30-$A$123*'Forecast'!I40)*(1+F112)/($A$123-F112)/(1+$A$123)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="G123" s="54">
+        <f>(('Forecast'!E30-$A$123*'Forecast'!D40)/(1+$A$123)^1+('Forecast'!F30-$A$123*'Forecast'!E40)/(1+$A$123)^2+('Forecast'!G30-$A$123*'Forecast'!F40)/(1+$A$123)^3+('Forecast'!H30-$A$123*'Forecast'!G40)/(1+$A$123)^4+('Forecast'!I30-$A$123*'Forecast'!H40)/(1+$A$123)^5+('Forecast'!J30-$A$123*'Forecast'!I40)/(1+$A$123)^6+('Forecast'!J30-$A$123*'Forecast'!I40)*(1+G112)/($A$123-G112)/(1+$A$123)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+      <c r="H123" s="54">
+        <f>(('Forecast'!E30-$A$123*'Forecast'!D40)/(1+$A$123)^1+('Forecast'!F30-$A$123*'Forecast'!E40)/(1+$A$123)^2+('Forecast'!G30-$A$123*'Forecast'!F40)/(1+$A$123)^3+('Forecast'!H30-$A$123*'Forecast'!G40)/(1+$A$123)^4+('Forecast'!I30-$A$123*'Forecast'!H40)/(1+$A$123)^5+('Forecast'!J30-$A$123*'Forecast'!I40)/(1+$A$123)^6+('Forecast'!J30-$A$123*'Forecast'!I40)*(1+H112)/($A$123-H112)/(1+$A$123)^6+'Forecast'!D40-$B$15)/$B$20*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="19" t="inlineStr">
+        <is>
+          <t>COMPARABLE COMPANY ANALYSIS</t>
+        </is>
+      </c>
+      <c r="B126" s="20" t="n"/>
+      <c r="C126" s="20" t="n"/>
+      <c r="D126" s="20" t="n"/>
+      <c r="E126" s="20" t="n"/>
+      <c r="F126" s="20" t="n"/>
+      <c r="G126" s="20" t="n"/>
+      <c r="H126" s="20" t="n"/>
+      <c r="I126" s="20" t="n"/>
+      <c r="J126" s="20" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="51" t="inlineStr">
+        <is>
+          <t>Peer Company</t>
+        </is>
+      </c>
+      <c r="B128" s="55" t="inlineStr">
+        <is>
+          <t>AIXTRON SE</t>
+        </is>
+      </c>
+      <c r="C128" s="55" t="inlineStr">
+        <is>
+          <t>Applied Materials</t>
+        </is>
+      </c>
+      <c r="D128" s="55" t="inlineStr">
+        <is>
+          <t>Lam Research</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="11" t="inlineStr">
+        <is>
+          <t>Enterprise Value (EUR 000)</t>
+        </is>
+      </c>
+      <c r="B129" s="45" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="C129" s="45" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="D129" s="45" t="n">
+        <v>95000000</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="11" t="inlineStr">
+        <is>
+          <t>EBITDA (EUR 000)</t>
+        </is>
+      </c>
+      <c r="B130" s="45" t="n">
+        <v>120000</v>
+      </c>
+      <c r="C130" s="45" t="n">
+        <v>9500000</v>
+      </c>
+      <c r="D130" s="45" t="n">
+        <v>5800000</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="11" t="inlineStr">
+        <is>
+          <t>EBIT (EUR 000)</t>
+        </is>
+      </c>
+      <c r="B131" s="45" t="n">
+        <v>85000</v>
+      </c>
+      <c r="C131" s="45" t="n">
+        <v>8200000</v>
+      </c>
+      <c r="D131" s="45" t="n">
+        <v>4900000</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="11" t="inlineStr">
+        <is>
+          <t>EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="B132" s="56">
+        <f>IF(B130&lt;&gt;0,B129/B130,0)</f>
+        <v/>
+      </c>
+      <c r="C132" s="56">
+        <f>IF(C130&lt;&gt;0,C129/C130,0)</f>
+        <v/>
+      </c>
+      <c r="D132" s="56">
+        <f>IF(D130&lt;&gt;0,D129/D130,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="11" t="inlineStr">
+        <is>
+          <t>EV/EBIT</t>
+        </is>
+      </c>
+      <c r="B133" s="56">
+        <f>IF(B131&lt;&gt;0,B129/B131,0)</f>
+        <v/>
+      </c>
+      <c r="C133" s="56">
+        <f>IF(C131&lt;&gt;0,C129/C131,0)</f>
+        <v/>
+      </c>
+      <c r="D133" s="56">
+        <f>IF(D131&lt;&gt;0,D129/D131,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="22" t="inlineStr">
+        <is>
+          <t>Median EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="B135" s="57">
+        <f>MEDIAN(B132:D132)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="22" t="inlineStr">
+        <is>
+          <t>Median EV/EBIT</t>
+        </is>
+      </c>
+      <c r="B136" s="57">
+        <f>MEDIAN(B133:D133)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="22" t="inlineStr">
+        <is>
+          <t>ASM International - Implied Valuation</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="11" t="inlineStr">
+        <is>
+          <t>ASM EBITDA (2024, EUR 000)</t>
+        </is>
+      </c>
+      <c r="B139" s="21">
+        <f>'Adj ASM'!G25+'Adj ASM'!G14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="11" t="inlineStr">
+        <is>
+          <t>ASM EBIT (2024, EUR 000)</t>
+        </is>
+      </c>
+      <c r="B140" s="21">
+        <f>'Adj ASM'!G25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="11" t="inlineStr">
+        <is>
+          <t>Implied EV (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="B142" s="31">
+        <f>B139*B135</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="11" t="inlineStr">
+        <is>
+          <t>- Net Debt</t>
+        </is>
+      </c>
+      <c r="B143" s="31">
+        <f>B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="22">
+        <f> Equity Value (EV/EBITDA)</f>
+        <v/>
+      </c>
+      <c r="B144" s="23">
+        <f>B142-B143</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="22" t="inlineStr">
+        <is>
+          <t>Implied Price (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="B145" s="58">
+        <f>IF(B20&lt;&gt;0,B144/B20*1000,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="11" t="inlineStr">
+        <is>
+          <t>Implied EV (EV/EBIT)</t>
+        </is>
+      </c>
+      <c r="B147" s="31">
+        <f>B140*B136</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="11" t="inlineStr">
+        <is>
+          <t>- Net Debt</t>
+        </is>
+      </c>
+      <c r="B148" s="31">
+        <f>B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="22">
+        <f> Equity Value (EV/EBIT)</f>
+        <v/>
+      </c>
+      <c r="B149" s="23">
+        <f>B147-B148</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="26" t="inlineStr">
+        <is>
+          <t>Implied Price (EV/EBIT)</t>
+        </is>
+      </c>
+      <c r="B150" s="49">
+        <f>IF(B20&lt;&gt;0,B149/B20*1000,0)</f>
+        <v/>
+      </c>
+      <c r="C150" s="50" t="n"/>
+      <c r="D150" s="50" t="n"/>
+      <c r="E150" s="50" t="n"/>
+      <c r="F150" s="50" t="n"/>
+      <c r="G150" s="50" t="n"/>
+      <c r="H150" s="50" t="n"/>
+      <c r="I150" s="50" t="n"/>
+      <c r="J150" s="50" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="19" t="inlineStr">
+        <is>
+          <t>FOOTBALL FIELD SUMMARY</t>
+        </is>
+      </c>
+      <c r="B152" s="20" t="n"/>
+      <c r="C152" s="20" t="n"/>
+      <c r="D152" s="20" t="n"/>
+      <c r="E152" s="20" t="n"/>
+      <c r="F152" s="20" t="n"/>
+      <c r="G152" s="20" t="n"/>
+      <c r="H152" s="20" t="n"/>
+      <c r="I152" s="20" t="n"/>
+      <c r="J152" s="20" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="51" t="inlineStr">
+        <is>
+          <t>Valuation Method</t>
+        </is>
+      </c>
+      <c r="B154" s="55" t="inlineStr">
+        <is>
+          <t>Implied Price (EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="11" t="inlineStr">
+        <is>
+          <t>DCF (FCFF)</t>
+        </is>
+      </c>
+      <c r="B155" s="54">
+        <f>B39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="11" t="inlineStr">
+        <is>
+          <t>DCF (FCFE)</t>
+        </is>
+      </c>
+      <c r="B156" s="54">
+        <f>B53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="11" t="inlineStr">
+        <is>
+          <t>PVAOI</t>
+        </is>
+      </c>
+      <c r="B157" s="54">
+        <f>B73</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="11" t="inlineStr">
+        <is>
+          <t>PVAE</t>
+        </is>
+      </c>
+      <c r="B158" s="54">
+        <f>B91</f>
+        <v/>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="11" t="inlineStr">
+        <is>
+          <t>Comps (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="B159" s="54">
+        <f>B145</f>
+        <v/>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="11" t="inlineStr">
+        <is>
+          <t>Comps (EV/EBIT)</t>
+        </is>
+      </c>
+      <c r="B160" s="54">
+        <f>B150</f>
+        <v/>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="11" t="inlineStr">
+        <is>
+          <t>Current Share Price</t>
+        </is>
+      </c>
+      <c r="B161" s="54">
+        <f>B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="24" t="n"/>
+      <c r="B162" s="24" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="22" t="inlineStr">
+        <is>
+          <t>Average Implied Price</t>
+        </is>
+      </c>
+      <c r="B163" s="58">
+        <f>AVERAGE(B155:B160)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="26" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="B164" s="59">
+        <f>IF(B163&gt;B161,"BUY","SELL")</f>
+        <v/>
+      </c>
+      <c r="C164" s="50" t="n"/>
+      <c r="D164" s="50" t="n"/>
+      <c r="E164" s="50" t="n"/>
+      <c r="F164" s="50" t="n"/>
+      <c r="G164" s="50" t="n"/>
+      <c r="H164" s="50" t="n"/>
+      <c r="I164" s="50" t="n"/>
+      <c r="J164" s="50" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: complete ASM International valuation model with final polish
Add missing freeze panes on Adjustments and Ratio Definitions tabs.
Fix freeze pane positions on Ratio, Ratio Comparison, and Valuation tabs
for consistency with their row layouts.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/ASM_Valuation_Model.xlsx
+++ b/output/ASM_Valuation_Model.xlsx
@@ -3273,6 +3273,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="32" t="inlineStr">
         <is>
@@ -13170,6 +13171,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="38" t="inlineStr">
         <is>
@@ -13500,6 +13502,7 @@
         <v>2024</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -14568,6 +14571,7 @@
         <v>2024</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -15636,6 +15640,7 @@
         <v>2024</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -22085,6 +22090,7 @@
         <v>2024</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -23153,6 +23159,7 @@
         <v>2024</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -26656,7 +26663,6 @@
       <c r="I3" s="20" t="n"/>
       <c r="J3" s="20" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>

</xml_diff>